<commit_message>
root: update edge engine, world cup/tournament odds, betting tracker and sprint notes
</commit_message>
<xml_diff>
--- a/Betting Tracker Example.xlsx
+++ b/Betting Tracker Example.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="680" windowWidth="34200" windowHeight="21460" tabRatio="500" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="My Bets" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Ledger" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="My Bets" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Project Ledger" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterateDelta="0.0001"/>
@@ -17,13 +17,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="\£#,##0.00;&quot;(£&quot;#,##0.00\);\-"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="\£#,##0.00;\(\£#,##0.00\);&quot;-&quot;"/>
     <numFmt numFmtId="167" formatCode="\+0.0%;\-0.0%"/>
     <numFmt numFmtId="168" formatCode="£#,##0.00;(£#,##0.00);&quot;-&quot;"/>
     <numFmt numFmtId="169" formatCode="+0.0%;-0.0%"/>
+    <numFmt numFmtId="170" formatCode="+0;-0;0"/>
   </numFmts>
   <fonts count="12">
     <font>
@@ -146,7 +147,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -175,6 +176,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="169" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -249,6 +251,21 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Tracker</author>
+  </authors>
+  <commentList>
+    <comment ref="K3" authorId="0" shapeId="0">
+      <text>
+        <t>American (US) odds, auto-converted from the decimal Odds column (D). Decimal ≥ 2.00 → +(d-1)×100; 1.00–2.00 → -100/(d-1). Blank if no odds entered.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -646,7 +663,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J297"/>
+  <dimension ref="A1:K297"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" style="23" min="1" max="1"/>
@@ -658,6 +675,7 @@
     <col width="11" customWidth="1" style="23" min="7" max="8"/>
     <col width="12" customWidth="1" style="23" min="9" max="9"/>
     <col width="30" customWidth="1" style="23" min="10" max="10"/>
+    <col width="8" customWidth="1" style="23" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="17.25" customHeight="1" s="23">
@@ -731,6 +749,11 @@
       <c r="J3" s="10" t="inlineStr">
         <is>
           <t>Notes</t>
+        </is>
+      </c>
+      <c r="K3" s="10" t="inlineStr">
+        <is>
+          <t>US Odds</t>
         </is>
       </c>
     </row>
@@ -754,6 +777,10 @@
         <v/>
       </c>
       <c r="J4" s="12" t="n"/>
+      <c r="K4" s="26">
+        <f>IF(ISNUMBER($D4),IF($D4&gt;=2,ROUND(($D4-1)*100,0),IF($D4&gt;1,ROUND(-100/($D4-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="23">
       <c r="A5" s="11" t="n"/>
@@ -775,6 +802,10 @@
         <v/>
       </c>
       <c r="J5" s="12" t="n"/>
+      <c r="K5" s="26">
+        <f>IF(ISNUMBER($D5),IF($D5&gt;=2,ROUND(($D5-1)*100,0),IF($D5&gt;1,ROUND(-100/($D5-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="23">
       <c r="A6" s="11" t="n"/>
@@ -796,6 +827,10 @@
         <v/>
       </c>
       <c r="J6" s="12" t="n"/>
+      <c r="K6" s="26">
+        <f>IF(ISNUMBER($D6),IF($D6&gt;=2,ROUND(($D6-1)*100,0),IF($D6&gt;1,ROUND(-100/($D6-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="23">
       <c r="A7" s="11" t="n"/>
@@ -817,6 +852,10 @@
         <v/>
       </c>
       <c r="J7" s="12" t="n"/>
+      <c r="K7" s="26">
+        <f>IF(ISNUMBER($D7),IF($D7&gt;=2,ROUND(($D7-1)*100,0),IF($D7&gt;1,ROUND(-100/($D7-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="23">
       <c r="A8" s="11" t="n"/>
@@ -838,6 +877,10 @@
         <v/>
       </c>
       <c r="J8" s="12" t="n"/>
+      <c r="K8" s="26">
+        <f>IF(ISNUMBER($D8),IF($D8&gt;=2,ROUND(($D8-1)*100,0),IF($D8&gt;1,ROUND(-100/($D8-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="23">
       <c r="A9" s="11" t="n"/>
@@ -859,6 +902,10 @@
         <v/>
       </c>
       <c r="J9" s="12" t="n"/>
+      <c r="K9" s="26">
+        <f>IF(ISNUMBER($D9),IF($D9&gt;=2,ROUND(($D9-1)*100,0),IF($D9&gt;1,ROUND(-100/($D9-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="23">
       <c r="A10" s="11" t="n"/>
@@ -880,6 +927,10 @@
         <v/>
       </c>
       <c r="J10" s="12" t="n"/>
+      <c r="K10" s="26">
+        <f>IF(ISNUMBER($D10),IF($D10&gt;=2,ROUND(($D10-1)*100,0),IF($D10&gt;1,ROUND(-100/($D10-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="23">
       <c r="A11" s="11" t="n"/>
@@ -901,6 +952,10 @@
         <v/>
       </c>
       <c r="J11" s="12" t="n"/>
+      <c r="K11" s="26">
+        <f>IF(ISNUMBER($D11),IF($D11&gt;=2,ROUND(($D11-1)*100,0),IF($D11&gt;1,ROUND(-100/($D11-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="23">
       <c r="A12" s="11" t="n"/>
@@ -922,6 +977,10 @@
         <v/>
       </c>
       <c r="J12" s="12" t="n"/>
+      <c r="K12" s="26">
+        <f>IF(ISNUMBER($D12),IF($D12&gt;=2,ROUND(($D12-1)*100,0),IF($D12&gt;1,ROUND(-100/($D12-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="23">
       <c r="A13" s="11" t="n"/>
@@ -943,6 +1002,10 @@
         <v/>
       </c>
       <c r="J13" s="12" t="n"/>
+      <c r="K13" s="26">
+        <f>IF(ISNUMBER($D13),IF($D13&gt;=2,ROUND(($D13-1)*100,0),IF($D13&gt;1,ROUND(-100/($D13-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="23">
       <c r="A14" s="11" t="n"/>
@@ -964,6 +1027,10 @@
         <v/>
       </c>
       <c r="J14" s="12" t="n"/>
+      <c r="K14" s="26">
+        <f>IF(ISNUMBER($D14),IF($D14&gt;=2,ROUND(($D14-1)*100,0),IF($D14&gt;1,ROUND(-100/($D14-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="23">
       <c r="A15" s="11" t="n"/>
@@ -985,6 +1052,10 @@
         <v/>
       </c>
       <c r="J15" s="12" t="n"/>
+      <c r="K15" s="26">
+        <f>IF(ISNUMBER($D15),IF($D15&gt;=2,ROUND(($D15-1)*100,0),IF($D15&gt;1,ROUND(-100/($D15-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="23">
       <c r="A16" s="11" t="n"/>
@@ -1006,6 +1077,10 @@
         <v/>
       </c>
       <c r="J16" s="12" t="n"/>
+      <c r="K16" s="26">
+        <f>IF(ISNUMBER($D16),IF($D16&gt;=2,ROUND(($D16-1)*100,0),IF($D16&gt;1,ROUND(-100/($D16-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="23">
       <c r="A17" s="11" t="n"/>
@@ -1027,6 +1102,10 @@
         <v/>
       </c>
       <c r="J17" s="12" t="n"/>
+      <c r="K17" s="26">
+        <f>IF(ISNUMBER($D17),IF($D17&gt;=2,ROUND(($D17-1)*100,0),IF($D17&gt;1,ROUND(-100/($D17-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="23">
       <c r="A18" s="11" t="n"/>
@@ -1048,6 +1127,10 @@
         <v/>
       </c>
       <c r="J18" s="12" t="n"/>
+      <c r="K18" s="26">
+        <f>IF(ISNUMBER($D18),IF($D18&gt;=2,ROUND(($D18-1)*100,0),IF($D18&gt;1,ROUND(-100/($D18-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="23">
       <c r="A19" s="11" t="n"/>
@@ -1069,6 +1152,10 @@
         <v/>
       </c>
       <c r="J19" s="12" t="n"/>
+      <c r="K19" s="26">
+        <f>IF(ISNUMBER($D19),IF($D19&gt;=2,ROUND(($D19-1)*100,0),IF($D19&gt;1,ROUND(-100/($D19-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="23">
       <c r="A20" s="11" t="n"/>
@@ -1090,6 +1177,10 @@
         <v/>
       </c>
       <c r="J20" s="12" t="n"/>
+      <c r="K20" s="26">
+        <f>IF(ISNUMBER($D20),IF($D20&gt;=2,ROUND(($D20-1)*100,0),IF($D20&gt;1,ROUND(-100/($D20-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="23">
       <c r="A21" s="11" t="n"/>
@@ -1111,6 +1202,10 @@
         <v/>
       </c>
       <c r="J21" s="12" t="n"/>
+      <c r="K21" s="26">
+        <f>IF(ISNUMBER($D21),IF($D21&gt;=2,ROUND(($D21-1)*100,0),IF($D21&gt;1,ROUND(-100/($D21-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="23">
       <c r="A22" s="11" t="n"/>
@@ -1132,6 +1227,10 @@
         <v/>
       </c>
       <c r="J22" s="12" t="n"/>
+      <c r="K22" s="26">
+        <f>IF(ISNUMBER($D22),IF($D22&gt;=2,ROUND(($D22-1)*100,0),IF($D22&gt;1,ROUND(-100/($D22-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="23">
       <c r="A23" s="11" t="n"/>
@@ -1153,6 +1252,10 @@
         <v/>
       </c>
       <c r="J23" s="12" t="n"/>
+      <c r="K23" s="26">
+        <f>IF(ISNUMBER($D23),IF($D23&gt;=2,ROUND(($D23-1)*100,0),IF($D23&gt;1,ROUND(-100/($D23-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="23">
       <c r="A24" s="11" t="n"/>
@@ -1174,6 +1277,10 @@
         <v/>
       </c>
       <c r="J24" s="12" t="n"/>
+      <c r="K24" s="26">
+        <f>IF(ISNUMBER($D24),IF($D24&gt;=2,ROUND(($D24-1)*100,0),IF($D24&gt;1,ROUND(-100/($D24-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="23">
       <c r="A25" s="11" t="n"/>
@@ -1195,6 +1302,10 @@
         <v/>
       </c>
       <c r="J25" s="12" t="n"/>
+      <c r="K25" s="26">
+        <f>IF(ISNUMBER($D25),IF($D25&gt;=2,ROUND(($D25-1)*100,0),IF($D25&gt;1,ROUND(-100/($D25-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="23">
       <c r="A26" s="11" t="n"/>
@@ -1216,6 +1327,10 @@
         <v/>
       </c>
       <c r="J26" s="12" t="n"/>
+      <c r="K26" s="26">
+        <f>IF(ISNUMBER($D26),IF($D26&gt;=2,ROUND(($D26-1)*100,0),IF($D26&gt;1,ROUND(-100/($D26-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="23">
       <c r="A27" s="11" t="n"/>
@@ -1237,6 +1352,10 @@
         <v/>
       </c>
       <c r="J27" s="12" t="n"/>
+      <c r="K27" s="26">
+        <f>IF(ISNUMBER($D27),IF($D27&gt;=2,ROUND(($D27-1)*100,0),IF($D27&gt;1,ROUND(-100/($D27-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="23">
       <c r="A28" s="11" t="n"/>
@@ -1258,6 +1377,10 @@
         <v/>
       </c>
       <c r="J28" s="12" t="n"/>
+      <c r="K28" s="26">
+        <f>IF(ISNUMBER($D28),IF($D28&gt;=2,ROUND(($D28-1)*100,0),IF($D28&gt;1,ROUND(-100/($D28-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="23">
       <c r="A29" s="11" t="n"/>
@@ -1279,6 +1402,10 @@
         <v/>
       </c>
       <c r="J29" s="12" t="n"/>
+      <c r="K29" s="26">
+        <f>IF(ISNUMBER($D29),IF($D29&gt;=2,ROUND(($D29-1)*100,0),IF($D29&gt;1,ROUND(-100/($D29-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="23">
       <c r="A30" s="11" t="n"/>
@@ -1300,6 +1427,10 @@
         <v/>
       </c>
       <c r="J30" s="12" t="n"/>
+      <c r="K30" s="26">
+        <f>IF(ISNUMBER($D30),IF($D30&gt;=2,ROUND(($D30-1)*100,0),IF($D30&gt;1,ROUND(-100/($D30-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="23">
       <c r="A31" s="11" t="n"/>
@@ -1321,6 +1452,10 @@
         <v/>
       </c>
       <c r="J31" s="12" t="n"/>
+      <c r="K31" s="26">
+        <f>IF(ISNUMBER($D31),IF($D31&gt;=2,ROUND(($D31-1)*100,0),IF($D31&gt;1,ROUND(-100/($D31-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="23">
       <c r="A32" s="11" t="n"/>
@@ -1342,6 +1477,10 @@
         <v/>
       </c>
       <c r="J32" s="12" t="n"/>
+      <c r="K32" s="26">
+        <f>IF(ISNUMBER($D32),IF($D32&gt;=2,ROUND(($D32-1)*100,0),IF($D32&gt;1,ROUND(-100/($D32-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="23">
       <c r="A33" s="11" t="n"/>
@@ -1363,6 +1502,10 @@
         <v/>
       </c>
       <c r="J33" s="12" t="n"/>
+      <c r="K33" s="26">
+        <f>IF(ISNUMBER($D33),IF($D33&gt;=2,ROUND(($D33-1)*100,0),IF($D33&gt;1,ROUND(-100/($D33-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="23">
       <c r="A34" s="11" t="n"/>
@@ -1384,6 +1527,10 @@
         <v/>
       </c>
       <c r="J34" s="12" t="n"/>
+      <c r="K34" s="26">
+        <f>IF(ISNUMBER($D34),IF($D34&gt;=2,ROUND(($D34-1)*100,0),IF($D34&gt;1,ROUND(-100/($D34-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="23">
       <c r="A35" s="11" t="n"/>
@@ -1405,6 +1552,10 @@
         <v/>
       </c>
       <c r="J35" s="12" t="n"/>
+      <c r="K35" s="26">
+        <f>IF(ISNUMBER($D35),IF($D35&gt;=2,ROUND(($D35-1)*100,0),IF($D35&gt;1,ROUND(-100/($D35-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="23">
       <c r="A36" s="11" t="n"/>
@@ -1426,6 +1577,10 @@
         <v/>
       </c>
       <c r="J36" s="12" t="n"/>
+      <c r="K36" s="26">
+        <f>IF(ISNUMBER($D36),IF($D36&gt;=2,ROUND(($D36-1)*100,0),IF($D36&gt;1,ROUND(-100/($D36-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="23">
       <c r="A37" s="11" t="n"/>
@@ -1447,6 +1602,10 @@
         <v/>
       </c>
       <c r="J37" s="12" t="n"/>
+      <c r="K37" s="26">
+        <f>IF(ISNUMBER($D37),IF($D37&gt;=2,ROUND(($D37-1)*100,0),IF($D37&gt;1,ROUND(-100/($D37-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="38" ht="15" customHeight="1" s="23">
       <c r="A38" s="11" t="n"/>
@@ -1468,6 +1627,10 @@
         <v/>
       </c>
       <c r="J38" s="12" t="n"/>
+      <c r="K38" s="26">
+        <f>IF(ISNUMBER($D38),IF($D38&gt;=2,ROUND(($D38-1)*100,0),IF($D38&gt;1,ROUND(-100/($D38-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="23">
       <c r="A39" s="11" t="n"/>
@@ -1489,6 +1652,10 @@
         <v/>
       </c>
       <c r="J39" s="12" t="n"/>
+      <c r="K39" s="26">
+        <f>IF(ISNUMBER($D39),IF($D39&gt;=2,ROUND(($D39-1)*100,0),IF($D39&gt;1,ROUND(-100/($D39-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="23">
       <c r="A40" s="11" t="n"/>
@@ -1510,6 +1677,10 @@
         <v/>
       </c>
       <c r="J40" s="12" t="n"/>
+      <c r="K40" s="26">
+        <f>IF(ISNUMBER($D40),IF($D40&gt;=2,ROUND(($D40-1)*100,0),IF($D40&gt;1,ROUND(-100/($D40-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="23">
       <c r="A41" s="11" t="n"/>
@@ -1531,6 +1702,10 @@
         <v/>
       </c>
       <c r="J41" s="12" t="n"/>
+      <c r="K41" s="26">
+        <f>IF(ISNUMBER($D41),IF($D41&gt;=2,ROUND(($D41-1)*100,0),IF($D41&gt;1,ROUND(-100/($D41-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="23">
       <c r="A42" s="11" t="n"/>
@@ -1552,6 +1727,10 @@
         <v/>
       </c>
       <c r="J42" s="12" t="n"/>
+      <c r="K42" s="26">
+        <f>IF(ISNUMBER($D42),IF($D42&gt;=2,ROUND(($D42-1)*100,0),IF($D42&gt;1,ROUND(-100/($D42-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="23">
       <c r="A43" s="11" t="n"/>
@@ -1573,6 +1752,10 @@
         <v/>
       </c>
       <c r="J43" s="12" t="n"/>
+      <c r="K43" s="26">
+        <f>IF(ISNUMBER($D43),IF($D43&gt;=2,ROUND(($D43-1)*100,0),IF($D43&gt;1,ROUND(-100/($D43-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="23">
       <c r="A44" s="11" t="n"/>
@@ -1594,6 +1777,10 @@
         <v/>
       </c>
       <c r="J44" s="12" t="n"/>
+      <c r="K44" s="26">
+        <f>IF(ISNUMBER($D44),IF($D44&gt;=2,ROUND(($D44-1)*100,0),IF($D44&gt;1,ROUND(-100/($D44-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="23">
       <c r="A45" s="11" t="n"/>
@@ -1615,6 +1802,10 @@
         <v/>
       </c>
       <c r="J45" s="12" t="n"/>
+      <c r="K45" s="26">
+        <f>IF(ISNUMBER($D45),IF($D45&gt;=2,ROUND(($D45-1)*100,0),IF($D45&gt;1,ROUND(-100/($D45-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="23">
       <c r="A46" s="11" t="n"/>
@@ -1636,6 +1827,10 @@
         <v/>
       </c>
       <c r="J46" s="12" t="n"/>
+      <c r="K46" s="26">
+        <f>IF(ISNUMBER($D46),IF($D46&gt;=2,ROUND(($D46-1)*100,0),IF($D46&gt;1,ROUND(-100/($D46-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="23">
       <c r="A47" s="11" t="n"/>
@@ -1657,6 +1852,10 @@
         <v/>
       </c>
       <c r="J47" s="12" t="n"/>
+      <c r="K47" s="26">
+        <f>IF(ISNUMBER($D47),IF($D47&gt;=2,ROUND(($D47-1)*100,0),IF($D47&gt;1,ROUND(-100/($D47-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="48" ht="15" customHeight="1" s="23">
       <c r="A48" s="11" t="n"/>
@@ -1678,6 +1877,10 @@
         <v/>
       </c>
       <c r="J48" s="12" t="n"/>
+      <c r="K48" s="26">
+        <f>IF(ISNUMBER($D48),IF($D48&gt;=2,ROUND(($D48-1)*100,0),IF($D48&gt;1,ROUND(-100/($D48-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="49" ht="15" customHeight="1" s="23">
       <c r="A49" s="11" t="n"/>
@@ -1699,6 +1902,10 @@
         <v/>
       </c>
       <c r="J49" s="12" t="n"/>
+      <c r="K49" s="26">
+        <f>IF(ISNUMBER($D49),IF($D49&gt;=2,ROUND(($D49-1)*100,0),IF($D49&gt;1,ROUND(-100/($D49-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="23">
       <c r="A50" s="11" t="n"/>
@@ -1720,6 +1927,10 @@
         <v/>
       </c>
       <c r="J50" s="12" t="n"/>
+      <c r="K50" s="26">
+        <f>IF(ISNUMBER($D50),IF($D50&gt;=2,ROUND(($D50-1)*100,0),IF($D50&gt;1,ROUND(-100/($D50-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="23">
       <c r="A51" s="11" t="n"/>
@@ -1741,6 +1952,10 @@
         <v/>
       </c>
       <c r="J51" s="12" t="n"/>
+      <c r="K51" s="26">
+        <f>IF(ISNUMBER($D51),IF($D51&gt;=2,ROUND(($D51-1)*100,0),IF($D51&gt;1,ROUND(-100/($D51-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="23">
       <c r="A52" s="11" t="n"/>
@@ -1762,6 +1977,10 @@
         <v/>
       </c>
       <c r="J52" s="12" t="n"/>
+      <c r="K52" s="26">
+        <f>IF(ISNUMBER($D52),IF($D52&gt;=2,ROUND(($D52-1)*100,0),IF($D52&gt;1,ROUND(-100/($D52-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="23">
       <c r="A53" s="11" t="n"/>
@@ -1783,6 +2002,10 @@
         <v/>
       </c>
       <c r="J53" s="12" t="n"/>
+      <c r="K53" s="26">
+        <f>IF(ISNUMBER($D53),IF($D53&gt;=2,ROUND(($D53-1)*100,0),IF($D53&gt;1,ROUND(-100/($D53-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="23">
       <c r="A54" s="11" t="n"/>
@@ -1804,6 +2027,10 @@
         <v/>
       </c>
       <c r="J54" s="12" t="n"/>
+      <c r="K54" s="26">
+        <f>IF(ISNUMBER($D54),IF($D54&gt;=2,ROUND(($D54-1)*100,0),IF($D54&gt;1,ROUND(-100/($D54-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="23">
       <c r="A55" s="11" t="n"/>
@@ -1825,6 +2052,10 @@
         <v/>
       </c>
       <c r="J55" s="12" t="n"/>
+      <c r="K55" s="26">
+        <f>IF(ISNUMBER($D55),IF($D55&gt;=2,ROUND(($D55-1)*100,0),IF($D55&gt;1,ROUND(-100/($D55-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="23">
       <c r="A56" s="11" t="n"/>
@@ -1846,6 +2077,10 @@
         <v/>
       </c>
       <c r="J56" s="12" t="n"/>
+      <c r="K56" s="26">
+        <f>IF(ISNUMBER($D56),IF($D56&gt;=2,ROUND(($D56-1)*100,0),IF($D56&gt;1,ROUND(-100/($D56-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="23">
       <c r="A57" s="11" t="n"/>
@@ -1867,6 +2102,10 @@
         <v/>
       </c>
       <c r="J57" s="12" t="n"/>
+      <c r="K57" s="26">
+        <f>IF(ISNUMBER($D57),IF($D57&gt;=2,ROUND(($D57-1)*100,0),IF($D57&gt;1,ROUND(-100/($D57-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="23">
       <c r="A58" s="11" t="n"/>
@@ -1888,6 +2127,10 @@
         <v/>
       </c>
       <c r="J58" s="12" t="n"/>
+      <c r="K58" s="26">
+        <f>IF(ISNUMBER($D58),IF($D58&gt;=2,ROUND(($D58-1)*100,0),IF($D58&gt;1,ROUND(-100/($D58-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="23">
       <c r="A59" s="11" t="n"/>
@@ -1909,6 +2152,10 @@
         <v/>
       </c>
       <c r="J59" s="12" t="n"/>
+      <c r="K59" s="26">
+        <f>IF(ISNUMBER($D59),IF($D59&gt;=2,ROUND(($D59-1)*100,0),IF($D59&gt;1,ROUND(-100/($D59-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="23">
       <c r="A60" s="11" t="n"/>
@@ -1930,6 +2177,10 @@
         <v/>
       </c>
       <c r="J60" s="12" t="n"/>
+      <c r="K60" s="26">
+        <f>IF(ISNUMBER($D60),IF($D60&gt;=2,ROUND(($D60-1)*100,0),IF($D60&gt;1,ROUND(-100/($D60-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="23">
       <c r="A61" s="11" t="n"/>
@@ -1951,6 +2202,10 @@
         <v/>
       </c>
       <c r="J61" s="12" t="n"/>
+      <c r="K61" s="26">
+        <f>IF(ISNUMBER($D61),IF($D61&gt;=2,ROUND(($D61-1)*100,0),IF($D61&gt;1,ROUND(-100/($D61-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="23">
       <c r="A62" s="11" t="n"/>
@@ -1972,6 +2227,10 @@
         <v/>
       </c>
       <c r="J62" s="12" t="n"/>
+      <c r="K62" s="26">
+        <f>IF(ISNUMBER($D62),IF($D62&gt;=2,ROUND(($D62-1)*100,0),IF($D62&gt;1,ROUND(-100/($D62-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="23">
       <c r="A63" s="11" t="n"/>
@@ -1993,6 +2252,10 @@
         <v/>
       </c>
       <c r="J63" s="12" t="n"/>
+      <c r="K63" s="26">
+        <f>IF(ISNUMBER($D63),IF($D63&gt;=2,ROUND(($D63-1)*100,0),IF($D63&gt;1,ROUND(-100/($D63-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="23">
       <c r="A64" s="11" t="n"/>
@@ -2014,6 +2277,10 @@
         <v/>
       </c>
       <c r="J64" s="12" t="n"/>
+      <c r="K64" s="26">
+        <f>IF(ISNUMBER($D64),IF($D64&gt;=2,ROUND(($D64-1)*100,0),IF($D64&gt;1,ROUND(-100/($D64-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="23">
       <c r="A65" s="11" t="n"/>
@@ -2035,6 +2302,10 @@
         <v/>
       </c>
       <c r="J65" s="12" t="n"/>
+      <c r="K65" s="26">
+        <f>IF(ISNUMBER($D65),IF($D65&gt;=2,ROUND(($D65-1)*100,0),IF($D65&gt;1,ROUND(-100/($D65-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="23">
       <c r="A66" s="11" t="n"/>
@@ -2056,6 +2327,10 @@
         <v/>
       </c>
       <c r="J66" s="12" t="n"/>
+      <c r="K66" s="26">
+        <f>IF(ISNUMBER($D66),IF($D66&gt;=2,ROUND(($D66-1)*100,0),IF($D66&gt;1,ROUND(-100/($D66-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="23">
       <c r="A67" s="11" t="n"/>
@@ -2077,6 +2352,10 @@
         <v/>
       </c>
       <c r="J67" s="12" t="n"/>
+      <c r="K67" s="26">
+        <f>IF(ISNUMBER($D67),IF($D67&gt;=2,ROUND(($D67-1)*100,0),IF($D67&gt;1,ROUND(-100/($D67-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="23">
       <c r="A68" s="11" t="n"/>
@@ -2098,6 +2377,10 @@
         <v/>
       </c>
       <c r="J68" s="12" t="n"/>
+      <c r="K68" s="26">
+        <f>IF(ISNUMBER($D68),IF($D68&gt;=2,ROUND(($D68-1)*100,0),IF($D68&gt;1,ROUND(-100/($D68-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="23">
       <c r="A69" s="11" t="n"/>
@@ -2119,6 +2402,10 @@
         <v/>
       </c>
       <c r="J69" s="12" t="n"/>
+      <c r="K69" s="26">
+        <f>IF(ISNUMBER($D69),IF($D69&gt;=2,ROUND(($D69-1)*100,0),IF($D69&gt;1,ROUND(-100/($D69-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="23">
       <c r="A70" s="11" t="n"/>
@@ -2140,6 +2427,10 @@
         <v/>
       </c>
       <c r="J70" s="12" t="n"/>
+      <c r="K70" s="26">
+        <f>IF(ISNUMBER($D70),IF($D70&gt;=2,ROUND(($D70-1)*100,0),IF($D70&gt;1,ROUND(-100/($D70-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="23">
       <c r="A71" s="11" t="n"/>
@@ -2161,6 +2452,10 @@
         <v/>
       </c>
       <c r="J71" s="12" t="n"/>
+      <c r="K71" s="26">
+        <f>IF(ISNUMBER($D71),IF($D71&gt;=2,ROUND(($D71-1)*100,0),IF($D71&gt;1,ROUND(-100/($D71-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="23">
       <c r="A72" s="11" t="n"/>
@@ -2182,6 +2477,10 @@
         <v/>
       </c>
       <c r="J72" s="12" t="n"/>
+      <c r="K72" s="26">
+        <f>IF(ISNUMBER($D72),IF($D72&gt;=2,ROUND(($D72-1)*100,0),IF($D72&gt;1,ROUND(-100/($D72-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="23">
       <c r="A73" s="11" t="n"/>
@@ -2203,6 +2502,10 @@
         <v/>
       </c>
       <c r="J73" s="12" t="n"/>
+      <c r="K73" s="26">
+        <f>IF(ISNUMBER($D73),IF($D73&gt;=2,ROUND(($D73-1)*100,0),IF($D73&gt;1,ROUND(-100/($D73-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="23">
       <c r="A74" s="11" t="n"/>
@@ -2224,6 +2527,10 @@
         <v/>
       </c>
       <c r="J74" s="12" t="n"/>
+      <c r="K74" s="26">
+        <f>IF(ISNUMBER($D74),IF($D74&gt;=2,ROUND(($D74-1)*100,0),IF($D74&gt;1,ROUND(-100/($D74-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="75" ht="15" customHeight="1" s="23">
       <c r="A75" s="11" t="n"/>
@@ -2245,6 +2552,10 @@
         <v/>
       </c>
       <c r="J75" s="12" t="n"/>
+      <c r="K75" s="26">
+        <f>IF(ISNUMBER($D75),IF($D75&gt;=2,ROUND(($D75-1)*100,0),IF($D75&gt;1,ROUND(-100/($D75-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="23">
       <c r="A76" s="11" t="n"/>
@@ -2266,6 +2577,10 @@
         <v/>
       </c>
       <c r="J76" s="12" t="n"/>
+      <c r="K76" s="26">
+        <f>IF(ISNUMBER($D76),IF($D76&gt;=2,ROUND(($D76-1)*100,0),IF($D76&gt;1,ROUND(-100/($D76-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="23">
       <c r="A77" s="11" t="n"/>
@@ -2287,6 +2602,10 @@
         <v/>
       </c>
       <c r="J77" s="12" t="n"/>
+      <c r="K77" s="26">
+        <f>IF(ISNUMBER($D77),IF($D77&gt;=2,ROUND(($D77-1)*100,0),IF($D77&gt;1,ROUND(-100/($D77-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="78" ht="15" customHeight="1" s="23">
       <c r="A78" s="11" t="n"/>
@@ -2308,6 +2627,10 @@
         <v/>
       </c>
       <c r="J78" s="12" t="n"/>
+      <c r="K78" s="26">
+        <f>IF(ISNUMBER($D78),IF($D78&gt;=2,ROUND(($D78-1)*100,0),IF($D78&gt;1,ROUND(-100/($D78-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="23">
       <c r="A79" s="11" t="n"/>
@@ -2329,6 +2652,10 @@
         <v/>
       </c>
       <c r="J79" s="12" t="n"/>
+      <c r="K79" s="26">
+        <f>IF(ISNUMBER($D79),IF($D79&gt;=2,ROUND(($D79-1)*100,0),IF($D79&gt;1,ROUND(-100/($D79-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="80" ht="15" customHeight="1" s="23">
       <c r="A80" s="11" t="n"/>
@@ -2350,6 +2677,10 @@
         <v/>
       </c>
       <c r="J80" s="12" t="n"/>
+      <c r="K80" s="26">
+        <f>IF(ISNUMBER($D80),IF($D80&gt;=2,ROUND(($D80-1)*100,0),IF($D80&gt;1,ROUND(-100/($D80-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="23">
       <c r="A81" s="11" t="n"/>
@@ -2371,6 +2702,10 @@
         <v/>
       </c>
       <c r="J81" s="12" t="n"/>
+      <c r="K81" s="26">
+        <f>IF(ISNUMBER($D81),IF($D81&gt;=2,ROUND(($D81-1)*100,0),IF($D81&gt;1,ROUND(-100/($D81-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="23">
       <c r="A82" s="11" t="n"/>
@@ -2392,6 +2727,10 @@
         <v/>
       </c>
       <c r="J82" s="12" t="n"/>
+      <c r="K82" s="26">
+        <f>IF(ISNUMBER($D82),IF($D82&gt;=2,ROUND(($D82-1)*100,0),IF($D82&gt;1,ROUND(-100/($D82-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="23">
       <c r="A83" s="11" t="n"/>
@@ -2413,6 +2752,10 @@
         <v/>
       </c>
       <c r="J83" s="12" t="n"/>
+      <c r="K83" s="26">
+        <f>IF(ISNUMBER($D83),IF($D83&gt;=2,ROUND(($D83-1)*100,0),IF($D83&gt;1,ROUND(-100/($D83-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="23">
       <c r="A84" s="11" t="n"/>
@@ -2434,6 +2777,10 @@
         <v/>
       </c>
       <c r="J84" s="12" t="n"/>
+      <c r="K84" s="26">
+        <f>IF(ISNUMBER($D84),IF($D84&gt;=2,ROUND(($D84-1)*100,0),IF($D84&gt;1,ROUND(-100/($D84-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="23">
       <c r="A85" s="11" t="n"/>
@@ -2455,6 +2802,10 @@
         <v/>
       </c>
       <c r="J85" s="12" t="n"/>
+      <c r="K85" s="26">
+        <f>IF(ISNUMBER($D85),IF($D85&gt;=2,ROUND(($D85-1)*100,0),IF($D85&gt;1,ROUND(-100/($D85-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="23">
       <c r="A86" s="11" t="n"/>
@@ -2476,6 +2827,10 @@
         <v/>
       </c>
       <c r="J86" s="12" t="n"/>
+      <c r="K86" s="26">
+        <f>IF(ISNUMBER($D86),IF($D86&gt;=2,ROUND(($D86-1)*100,0),IF($D86&gt;1,ROUND(-100/($D86-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="23">
       <c r="A87" s="11" t="n"/>
@@ -2497,6 +2852,10 @@
         <v/>
       </c>
       <c r="J87" s="12" t="n"/>
+      <c r="K87" s="26">
+        <f>IF(ISNUMBER($D87),IF($D87&gt;=2,ROUND(($D87-1)*100,0),IF($D87&gt;1,ROUND(-100/($D87-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="23">
       <c r="A88" s="11" t="n"/>
@@ -2518,6 +2877,10 @@
         <v/>
       </c>
       <c r="J88" s="12" t="n"/>
+      <c r="K88" s="26">
+        <f>IF(ISNUMBER($D88),IF($D88&gt;=2,ROUND(($D88-1)*100,0),IF($D88&gt;1,ROUND(-100/($D88-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="23">
       <c r="A89" s="11" t="n"/>
@@ -2539,6 +2902,10 @@
         <v/>
       </c>
       <c r="J89" s="12" t="n"/>
+      <c r="K89" s="26">
+        <f>IF(ISNUMBER($D89),IF($D89&gt;=2,ROUND(($D89-1)*100,0),IF($D89&gt;1,ROUND(-100/($D89-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="23">
       <c r="A90" s="11" t="n"/>
@@ -2560,6 +2927,10 @@
         <v/>
       </c>
       <c r="J90" s="12" t="n"/>
+      <c r="K90" s="26">
+        <f>IF(ISNUMBER($D90),IF($D90&gt;=2,ROUND(($D90-1)*100,0),IF($D90&gt;1,ROUND(-100/($D90-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="23">
       <c r="A91" s="11" t="n"/>
@@ -2581,6 +2952,10 @@
         <v/>
       </c>
       <c r="J91" s="12" t="n"/>
+      <c r="K91" s="26">
+        <f>IF(ISNUMBER($D91),IF($D91&gt;=2,ROUND(($D91-1)*100,0),IF($D91&gt;1,ROUND(-100/($D91-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="92" ht="15" customHeight="1" s="23">
       <c r="A92" s="11" t="n"/>
@@ -2602,6 +2977,10 @@
         <v/>
       </c>
       <c r="J92" s="12" t="n"/>
+      <c r="K92" s="26">
+        <f>IF(ISNUMBER($D92),IF($D92&gt;=2,ROUND(($D92-1)*100,0),IF($D92&gt;1,ROUND(-100/($D92-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="23">
       <c r="A93" s="11" t="n"/>
@@ -2623,6 +3002,10 @@
         <v/>
       </c>
       <c r="J93" s="12" t="n"/>
+      <c r="K93" s="26">
+        <f>IF(ISNUMBER($D93),IF($D93&gt;=2,ROUND(($D93-1)*100,0),IF($D93&gt;1,ROUND(-100/($D93-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="23">
       <c r="A94" s="11" t="n"/>
@@ -2644,6 +3027,10 @@
         <v/>
       </c>
       <c r="J94" s="12" t="n"/>
+      <c r="K94" s="26">
+        <f>IF(ISNUMBER($D94),IF($D94&gt;=2,ROUND(($D94-1)*100,0),IF($D94&gt;1,ROUND(-100/($D94-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="23">
       <c r="A95" s="11" t="n"/>
@@ -2665,6 +3052,10 @@
         <v/>
       </c>
       <c r="J95" s="12" t="n"/>
+      <c r="K95" s="26">
+        <f>IF(ISNUMBER($D95),IF($D95&gt;=2,ROUND(($D95-1)*100,0),IF($D95&gt;1,ROUND(-100/($D95-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="23">
       <c r="A96" s="11" t="n"/>
@@ -2686,6 +3077,10 @@
         <v/>
       </c>
       <c r="J96" s="12" t="n"/>
+      <c r="K96" s="26">
+        <f>IF(ISNUMBER($D96),IF($D96&gt;=2,ROUND(($D96-1)*100,0),IF($D96&gt;1,ROUND(-100/($D96-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="23">
       <c r="A97" s="11" t="n"/>
@@ -2707,6 +3102,10 @@
         <v/>
       </c>
       <c r="J97" s="12" t="n"/>
+      <c r="K97" s="26">
+        <f>IF(ISNUMBER($D97),IF($D97&gt;=2,ROUND(($D97-1)*100,0),IF($D97&gt;1,ROUND(-100/($D97-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="23">
       <c r="A98" s="11" t="n"/>
@@ -2728,6 +3127,10 @@
         <v/>
       </c>
       <c r="J98" s="12" t="n"/>
+      <c r="K98" s="26">
+        <f>IF(ISNUMBER($D98),IF($D98&gt;=2,ROUND(($D98-1)*100,0),IF($D98&gt;1,ROUND(-100/($D98-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="23">
       <c r="A99" s="11" t="n"/>
@@ -2749,6 +3152,10 @@
         <v/>
       </c>
       <c r="J99" s="12" t="n"/>
+      <c r="K99" s="26">
+        <f>IF(ISNUMBER($D99),IF($D99&gt;=2,ROUND(($D99-1)*100,0),IF($D99&gt;1,ROUND(-100/($D99-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="23">
       <c r="A100" s="11" t="n"/>
@@ -2770,6 +3177,10 @@
         <v/>
       </c>
       <c r="J100" s="12" t="n"/>
+      <c r="K100" s="26">
+        <f>IF(ISNUMBER($D100),IF($D100&gt;=2,ROUND(($D100-1)*100,0),IF($D100&gt;1,ROUND(-100/($D100-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="23">
       <c r="A101" s="11" t="n"/>
@@ -2791,6 +3202,10 @@
         <v/>
       </c>
       <c r="J101" s="12" t="n"/>
+      <c r="K101" s="26">
+        <f>IF(ISNUMBER($D101),IF($D101&gt;=2,ROUND(($D101-1)*100,0),IF($D101&gt;1,ROUND(-100/($D101-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="23">
       <c r="A102" s="11" t="n"/>
@@ -2812,6 +3227,10 @@
         <v/>
       </c>
       <c r="J102" s="12" t="n"/>
+      <c r="K102" s="26">
+        <f>IF(ISNUMBER($D102),IF($D102&gt;=2,ROUND(($D102-1)*100,0),IF($D102&gt;1,ROUND(-100/($D102-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="23">
       <c r="A103" s="11" t="n"/>
@@ -2833,6 +3252,10 @@
         <v/>
       </c>
       <c r="J103" s="12" t="n"/>
+      <c r="K103" s="26">
+        <f>IF(ISNUMBER($D103),IF($D103&gt;=2,ROUND(($D103-1)*100,0),IF($D103&gt;1,ROUND(-100/($D103-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="104" ht="15" customHeight="1" s="23">
       <c r="A104" s="11" t="n"/>
@@ -2854,6 +3277,10 @@
         <v/>
       </c>
       <c r="J104" s="12" t="n"/>
+      <c r="K104" s="26">
+        <f>IF(ISNUMBER($D104),IF($D104&gt;=2,ROUND(($D104-1)*100,0),IF($D104&gt;1,ROUND(-100/($D104-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="105" ht="15" customHeight="1" s="23">
       <c r="A105" s="11" t="n"/>
@@ -2875,6 +3302,10 @@
         <v/>
       </c>
       <c r="J105" s="12" t="n"/>
+      <c r="K105" s="26">
+        <f>IF(ISNUMBER($D105),IF($D105&gt;=2,ROUND(($D105-1)*100,0),IF($D105&gt;1,ROUND(-100/($D105-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="23">
       <c r="A106" s="11" t="n"/>
@@ -2896,6 +3327,10 @@
         <v/>
       </c>
       <c r="J106" s="12" t="n"/>
+      <c r="K106" s="26">
+        <f>IF(ISNUMBER($D106),IF($D106&gt;=2,ROUND(($D106-1)*100,0),IF($D106&gt;1,ROUND(-100/($D106-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="23">
       <c r="A107" s="11" t="n"/>
@@ -2917,6 +3352,10 @@
         <v/>
       </c>
       <c r="J107" s="12" t="n"/>
+      <c r="K107" s="26">
+        <f>IF(ISNUMBER($D107),IF($D107&gt;=2,ROUND(($D107-1)*100,0),IF($D107&gt;1,ROUND(-100/($D107-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="108" ht="15" customHeight="1" s="23">
       <c r="A108" s="11" t="n"/>
@@ -2938,6 +3377,10 @@
         <v/>
       </c>
       <c r="J108" s="12" t="n"/>
+      <c r="K108" s="26">
+        <f>IF(ISNUMBER($D108),IF($D108&gt;=2,ROUND(($D108-1)*100,0),IF($D108&gt;1,ROUND(-100/($D108-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="109" ht="15" customHeight="1" s="23">
       <c r="A109" s="11" t="n"/>
@@ -2959,6 +3402,10 @@
         <v/>
       </c>
       <c r="J109" s="12" t="n"/>
+      <c r="K109" s="26">
+        <f>IF(ISNUMBER($D109),IF($D109&gt;=2,ROUND(($D109-1)*100,0),IF($D109&gt;1,ROUND(-100/($D109-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="110" ht="15" customHeight="1" s="23">
       <c r="A110" s="11" t="n"/>
@@ -2980,6 +3427,10 @@
         <v/>
       </c>
       <c r="J110" s="12" t="n"/>
+      <c r="K110" s="26">
+        <f>IF(ISNUMBER($D110),IF($D110&gt;=2,ROUND(($D110-1)*100,0),IF($D110&gt;1,ROUND(-100/($D110-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="111" ht="15" customHeight="1" s="23">
       <c r="A111" s="11" t="n"/>
@@ -3001,6 +3452,10 @@
         <v/>
       </c>
       <c r="J111" s="12" t="n"/>
+      <c r="K111" s="26">
+        <f>IF(ISNUMBER($D111),IF($D111&gt;=2,ROUND(($D111-1)*100,0),IF($D111&gt;1,ROUND(-100/($D111-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="112" ht="15" customHeight="1" s="23">
       <c r="A112" s="11" t="n"/>
@@ -3022,6 +3477,10 @@
         <v/>
       </c>
       <c r="J112" s="12" t="n"/>
+      <c r="K112" s="26">
+        <f>IF(ISNUMBER($D112),IF($D112&gt;=2,ROUND(($D112-1)*100,0),IF($D112&gt;1,ROUND(-100/($D112-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="113" ht="15" customHeight="1" s="23">
       <c r="A113" s="11" t="n"/>
@@ -3043,6 +3502,10 @@
         <v/>
       </c>
       <c r="J113" s="12" t="n"/>
+      <c r="K113" s="26">
+        <f>IF(ISNUMBER($D113),IF($D113&gt;=2,ROUND(($D113-1)*100,0),IF($D113&gt;1,ROUND(-100/($D113-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="114" ht="15" customHeight="1" s="23">
       <c r="A114" s="11" t="n"/>
@@ -3064,6 +3527,10 @@
         <v/>
       </c>
       <c r="J114" s="12" t="n"/>
+      <c r="K114" s="26">
+        <f>IF(ISNUMBER($D114),IF($D114&gt;=2,ROUND(($D114-1)*100,0),IF($D114&gt;1,ROUND(-100/($D114-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="115" ht="15" customHeight="1" s="23">
       <c r="A115" s="11" t="n"/>
@@ -3085,6 +3552,10 @@
         <v/>
       </c>
       <c r="J115" s="12" t="n"/>
+      <c r="K115" s="26">
+        <f>IF(ISNUMBER($D115),IF($D115&gt;=2,ROUND(($D115-1)*100,0),IF($D115&gt;1,ROUND(-100/($D115-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="116" ht="15" customHeight="1" s="23">
       <c r="A116" s="11" t="n"/>
@@ -3106,6 +3577,10 @@
         <v/>
       </c>
       <c r="J116" s="12" t="n"/>
+      <c r="K116" s="26">
+        <f>IF(ISNUMBER($D116),IF($D116&gt;=2,ROUND(($D116-1)*100,0),IF($D116&gt;1,ROUND(-100/($D116-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="117" ht="15" customHeight="1" s="23">
       <c r="A117" s="11" t="n"/>
@@ -3127,6 +3602,10 @@
         <v/>
       </c>
       <c r="J117" s="12" t="n"/>
+      <c r="K117" s="26">
+        <f>IF(ISNUMBER($D117),IF($D117&gt;=2,ROUND(($D117-1)*100,0),IF($D117&gt;1,ROUND(-100/($D117-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="118" ht="15" customHeight="1" s="23">
       <c r="A118" s="11" t="n"/>
@@ -3148,6 +3627,10 @@
         <v/>
       </c>
       <c r="J118" s="12" t="n"/>
+      <c r="K118" s="26">
+        <f>IF(ISNUMBER($D118),IF($D118&gt;=2,ROUND(($D118-1)*100,0),IF($D118&gt;1,ROUND(-100/($D118-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="119" ht="15" customHeight="1" s="23">
       <c r="A119" s="11" t="n"/>
@@ -3169,6 +3652,10 @@
         <v/>
       </c>
       <c r="J119" s="12" t="n"/>
+      <c r="K119" s="26">
+        <f>IF(ISNUMBER($D119),IF($D119&gt;=2,ROUND(($D119-1)*100,0),IF($D119&gt;1,ROUND(-100/($D119-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="120" ht="15" customHeight="1" s="23">
       <c r="A120" s="11" t="n"/>
@@ -3190,6 +3677,10 @@
         <v/>
       </c>
       <c r="J120" s="12" t="n"/>
+      <c r="K120" s="26">
+        <f>IF(ISNUMBER($D120),IF($D120&gt;=2,ROUND(($D120-1)*100,0),IF($D120&gt;1,ROUND(-100/($D120-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="121" ht="15" customHeight="1" s="23">
       <c r="A121" s="11" t="n"/>
@@ -3211,6 +3702,10 @@
         <v/>
       </c>
       <c r="J121" s="12" t="n"/>
+      <c r="K121" s="26">
+        <f>IF(ISNUMBER($D121),IF($D121&gt;=2,ROUND(($D121-1)*100,0),IF($D121&gt;1,ROUND(-100/($D121-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="122" ht="15" customHeight="1" s="23">
       <c r="A122" s="11" t="n"/>
@@ -3232,6 +3727,10 @@
         <v/>
       </c>
       <c r="J122" s="12" t="n"/>
+      <c r="K122" s="26">
+        <f>IF(ISNUMBER($D122),IF($D122&gt;=2,ROUND(($D122-1)*100,0),IF($D122&gt;1,ROUND(-100/($D122-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="123" ht="15" customHeight="1" s="23">
       <c r="A123" s="11" t="n"/>
@@ -3253,6 +3752,10 @@
         <v/>
       </c>
       <c r="J123" s="12" t="n"/>
+      <c r="K123" s="26">
+        <f>IF(ISNUMBER($D123),IF($D123&gt;=2,ROUND(($D123-1)*100,0),IF($D123&gt;1,ROUND(-100/($D123-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="124" ht="15" customHeight="1" s="23">
       <c r="A124" s="11" t="n"/>
@@ -3274,6 +3777,10 @@
         <v/>
       </c>
       <c r="J124" s="12" t="n"/>
+      <c r="K124" s="26">
+        <f>IF(ISNUMBER($D124),IF($D124&gt;=2,ROUND(($D124-1)*100,0),IF($D124&gt;1,ROUND(-100/($D124-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="125" ht="15" customHeight="1" s="23">
       <c r="A125" s="11" t="n"/>
@@ -3295,6 +3802,10 @@
         <v/>
       </c>
       <c r="J125" s="12" t="n"/>
+      <c r="K125" s="26">
+        <f>IF(ISNUMBER($D125),IF($D125&gt;=2,ROUND(($D125-1)*100,0),IF($D125&gt;1,ROUND(-100/($D125-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="126" ht="15" customHeight="1" s="23">
       <c r="A126" s="11" t="n"/>
@@ -3316,6 +3827,10 @@
         <v/>
       </c>
       <c r="J126" s="12" t="n"/>
+      <c r="K126" s="26">
+        <f>IF(ISNUMBER($D126),IF($D126&gt;=2,ROUND(($D126-1)*100,0),IF($D126&gt;1,ROUND(-100/($D126-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="127" ht="15" customHeight="1" s="23">
       <c r="A127" s="11" t="n"/>
@@ -3337,6 +3852,10 @@
         <v/>
       </c>
       <c r="J127" s="12" t="n"/>
+      <c r="K127" s="26">
+        <f>IF(ISNUMBER($D127),IF($D127&gt;=2,ROUND(($D127-1)*100,0),IF($D127&gt;1,ROUND(-100/($D127-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="128" ht="15" customHeight="1" s="23">
       <c r="A128" s="11" t="n"/>
@@ -3358,6 +3877,10 @@
         <v/>
       </c>
       <c r="J128" s="12" t="n"/>
+      <c r="K128" s="26">
+        <f>IF(ISNUMBER($D128),IF($D128&gt;=2,ROUND(($D128-1)*100,0),IF($D128&gt;1,ROUND(-100/($D128-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="129" ht="15" customHeight="1" s="23">
       <c r="A129" s="11" t="n"/>
@@ -3379,6 +3902,10 @@
         <v/>
       </c>
       <c r="J129" s="12" t="n"/>
+      <c r="K129" s="26">
+        <f>IF(ISNUMBER($D129),IF($D129&gt;=2,ROUND(($D129-1)*100,0),IF($D129&gt;1,ROUND(-100/($D129-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="130" ht="15" customHeight="1" s="23">
       <c r="A130" s="11" t="n"/>
@@ -3400,6 +3927,10 @@
         <v/>
       </c>
       <c r="J130" s="12" t="n"/>
+      <c r="K130" s="26">
+        <f>IF(ISNUMBER($D130),IF($D130&gt;=2,ROUND(($D130-1)*100,0),IF($D130&gt;1,ROUND(-100/($D130-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="131" ht="15" customHeight="1" s="23">
       <c r="A131" s="11" t="n"/>
@@ -3421,6 +3952,10 @@
         <v/>
       </c>
       <c r="J131" s="12" t="n"/>
+      <c r="K131" s="26">
+        <f>IF(ISNUMBER($D131),IF($D131&gt;=2,ROUND(($D131-1)*100,0),IF($D131&gt;1,ROUND(-100/($D131-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="132" ht="15" customHeight="1" s="23">
       <c r="A132" s="11" t="n"/>
@@ -3442,6 +3977,10 @@
         <v/>
       </c>
       <c r="J132" s="12" t="n"/>
+      <c r="K132" s="26">
+        <f>IF(ISNUMBER($D132),IF($D132&gt;=2,ROUND(($D132-1)*100,0),IF($D132&gt;1,ROUND(-100/($D132-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="133" ht="15" customHeight="1" s="23">
       <c r="A133" s="11" t="n"/>
@@ -3463,6 +4002,10 @@
         <v/>
       </c>
       <c r="J133" s="12" t="n"/>
+      <c r="K133" s="26">
+        <f>IF(ISNUMBER($D133),IF($D133&gt;=2,ROUND(($D133-1)*100,0),IF($D133&gt;1,ROUND(-100/($D133-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="134" ht="15" customHeight="1" s="23">
       <c r="A134" s="11" t="n"/>
@@ -3484,6 +4027,10 @@
         <v/>
       </c>
       <c r="J134" s="12" t="n"/>
+      <c r="K134" s="26">
+        <f>IF(ISNUMBER($D134),IF($D134&gt;=2,ROUND(($D134-1)*100,0),IF($D134&gt;1,ROUND(-100/($D134-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="135" ht="15" customHeight="1" s="23">
       <c r="A135" s="11" t="n"/>
@@ -3505,6 +4052,10 @@
         <v/>
       </c>
       <c r="J135" s="12" t="n"/>
+      <c r="K135" s="26">
+        <f>IF(ISNUMBER($D135),IF($D135&gt;=2,ROUND(($D135-1)*100,0),IF($D135&gt;1,ROUND(-100/($D135-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="136" ht="15" customHeight="1" s="23">
       <c r="A136" s="11" t="n"/>
@@ -3526,6 +4077,10 @@
         <v/>
       </c>
       <c r="J136" s="12" t="n"/>
+      <c r="K136" s="26">
+        <f>IF(ISNUMBER($D136),IF($D136&gt;=2,ROUND(($D136-1)*100,0),IF($D136&gt;1,ROUND(-100/($D136-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="137" ht="15" customHeight="1" s="23">
       <c r="A137" s="11" t="n"/>
@@ -3547,6 +4102,10 @@
         <v/>
       </c>
       <c r="J137" s="12" t="n"/>
+      <c r="K137" s="26">
+        <f>IF(ISNUMBER($D137),IF($D137&gt;=2,ROUND(($D137-1)*100,0),IF($D137&gt;1,ROUND(-100/($D137-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="138" ht="15" customHeight="1" s="23">
       <c r="A138" s="11" t="n"/>
@@ -3568,6 +4127,10 @@
         <v/>
       </c>
       <c r="J138" s="12" t="n"/>
+      <c r="K138" s="26">
+        <f>IF(ISNUMBER($D138),IF($D138&gt;=2,ROUND(($D138-1)*100,0),IF($D138&gt;1,ROUND(-100/($D138-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="139" ht="15" customHeight="1" s="23">
       <c r="A139" s="11" t="n"/>
@@ -3589,6 +4152,10 @@
         <v/>
       </c>
       <c r="J139" s="12" t="n"/>
+      <c r="K139" s="26">
+        <f>IF(ISNUMBER($D139),IF($D139&gt;=2,ROUND(($D139-1)*100,0),IF($D139&gt;1,ROUND(-100/($D139-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="140" ht="15" customHeight="1" s="23">
       <c r="A140" s="11" t="n"/>
@@ -3610,6 +4177,10 @@
         <v/>
       </c>
       <c r="J140" s="12" t="n"/>
+      <c r="K140" s="26">
+        <f>IF(ISNUMBER($D140),IF($D140&gt;=2,ROUND(($D140-1)*100,0),IF($D140&gt;1,ROUND(-100/($D140-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="141" ht="15" customHeight="1" s="23">
       <c r="A141" s="11" t="n"/>
@@ -3631,6 +4202,10 @@
         <v/>
       </c>
       <c r="J141" s="12" t="n"/>
+      <c r="K141" s="26">
+        <f>IF(ISNUMBER($D141),IF($D141&gt;=2,ROUND(($D141-1)*100,0),IF($D141&gt;1,ROUND(-100/($D141-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="142" ht="15" customHeight="1" s="23">
       <c r="A142" s="11" t="n"/>
@@ -3652,6 +4227,10 @@
         <v/>
       </c>
       <c r="J142" s="12" t="n"/>
+      <c r="K142" s="26">
+        <f>IF(ISNUMBER($D142),IF($D142&gt;=2,ROUND(($D142-1)*100,0),IF($D142&gt;1,ROUND(-100/($D142-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="143" ht="15" customHeight="1" s="23">
       <c r="A143" s="11" t="n"/>
@@ -3673,6 +4252,10 @@
         <v/>
       </c>
       <c r="J143" s="12" t="n"/>
+      <c r="K143" s="26">
+        <f>IF(ISNUMBER($D143),IF($D143&gt;=2,ROUND(($D143-1)*100,0),IF($D143&gt;1,ROUND(-100/($D143-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="144" ht="15" customHeight="1" s="23">
       <c r="A144" s="11" t="n"/>
@@ -3694,6 +4277,10 @@
         <v/>
       </c>
       <c r="J144" s="12" t="n"/>
+      <c r="K144" s="26">
+        <f>IF(ISNUMBER($D144),IF($D144&gt;=2,ROUND(($D144-1)*100,0),IF($D144&gt;1,ROUND(-100/($D144-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="145" ht="15" customHeight="1" s="23">
       <c r="A145" s="11" t="n"/>
@@ -3715,6 +4302,10 @@
         <v/>
       </c>
       <c r="J145" s="12" t="n"/>
+      <c r="K145" s="26">
+        <f>IF(ISNUMBER($D145),IF($D145&gt;=2,ROUND(($D145-1)*100,0),IF($D145&gt;1,ROUND(-100/($D145-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="146" ht="15" customHeight="1" s="23">
       <c r="A146" s="11" t="n"/>
@@ -3736,6 +4327,10 @@
         <v/>
       </c>
       <c r="J146" s="12" t="n"/>
+      <c r="K146" s="26">
+        <f>IF(ISNUMBER($D146),IF($D146&gt;=2,ROUND(($D146-1)*100,0),IF($D146&gt;1,ROUND(-100/($D146-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="147" ht="15" customHeight="1" s="23">
       <c r="A147" s="11" t="n"/>
@@ -3757,6 +4352,10 @@
         <v/>
       </c>
       <c r="J147" s="12" t="n"/>
+      <c r="K147" s="26">
+        <f>IF(ISNUMBER($D147),IF($D147&gt;=2,ROUND(($D147-1)*100,0),IF($D147&gt;1,ROUND(-100/($D147-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="148" ht="15" customHeight="1" s="23">
       <c r="A148" s="11" t="n"/>
@@ -3778,6 +4377,10 @@
         <v/>
       </c>
       <c r="J148" s="12" t="n"/>
+      <c r="K148" s="26">
+        <f>IF(ISNUMBER($D148),IF($D148&gt;=2,ROUND(($D148-1)*100,0),IF($D148&gt;1,ROUND(-100/($D148-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="149" ht="15" customHeight="1" s="23">
       <c r="A149" s="11" t="n"/>
@@ -3799,6 +4402,10 @@
         <v/>
       </c>
       <c r="J149" s="12" t="n"/>
+      <c r="K149" s="26">
+        <f>IF(ISNUMBER($D149),IF($D149&gt;=2,ROUND(($D149-1)*100,0),IF($D149&gt;1,ROUND(-100/($D149-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="150" ht="15" customHeight="1" s="23">
       <c r="A150" s="11" t="n"/>
@@ -3820,6 +4427,10 @@
         <v/>
       </c>
       <c r="J150" s="12" t="n"/>
+      <c r="K150" s="26">
+        <f>IF(ISNUMBER($D150),IF($D150&gt;=2,ROUND(($D150-1)*100,0),IF($D150&gt;1,ROUND(-100/($D150-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="151" ht="15" customHeight="1" s="23">
       <c r="A151" s="11" t="n"/>
@@ -3841,6 +4452,10 @@
         <v/>
       </c>
       <c r="J151" s="12" t="n"/>
+      <c r="K151" s="26">
+        <f>IF(ISNUMBER($D151),IF($D151&gt;=2,ROUND(($D151-1)*100,0),IF($D151&gt;1,ROUND(-100/($D151-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="152" ht="15" customHeight="1" s="23">
       <c r="A152" s="11" t="n"/>
@@ -3862,6 +4477,10 @@
         <v/>
       </c>
       <c r="J152" s="12" t="n"/>
+      <c r="K152" s="26">
+        <f>IF(ISNUMBER($D152),IF($D152&gt;=2,ROUND(($D152-1)*100,0),IF($D152&gt;1,ROUND(-100/($D152-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="153" ht="15" customHeight="1" s="23">
       <c r="A153" s="11" t="n"/>
@@ -3883,6 +4502,10 @@
         <v/>
       </c>
       <c r="J153" s="12" t="n"/>
+      <c r="K153" s="26">
+        <f>IF(ISNUMBER($D153),IF($D153&gt;=2,ROUND(($D153-1)*100,0),IF($D153&gt;1,ROUND(-100/($D153-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="154" ht="15" customHeight="1" s="23">
       <c r="A154" s="11" t="n"/>
@@ -3904,6 +4527,10 @@
         <v/>
       </c>
       <c r="J154" s="12" t="n"/>
+      <c r="K154" s="26">
+        <f>IF(ISNUMBER($D154),IF($D154&gt;=2,ROUND(($D154-1)*100,0),IF($D154&gt;1,ROUND(-100/($D154-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="155" ht="15" customHeight="1" s="23">
       <c r="A155" s="11" t="n"/>
@@ -3925,6 +4552,10 @@
         <v/>
       </c>
       <c r="J155" s="12" t="n"/>
+      <c r="K155" s="26">
+        <f>IF(ISNUMBER($D155),IF($D155&gt;=2,ROUND(($D155-1)*100,0),IF($D155&gt;1,ROUND(-100/($D155-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="156" ht="15" customHeight="1" s="23">
       <c r="A156" s="11" t="n"/>
@@ -3946,6 +4577,10 @@
         <v/>
       </c>
       <c r="J156" s="12" t="n"/>
+      <c r="K156" s="26">
+        <f>IF(ISNUMBER($D156),IF($D156&gt;=2,ROUND(($D156-1)*100,0),IF($D156&gt;1,ROUND(-100/($D156-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="157" ht="15" customHeight="1" s="23">
       <c r="A157" s="11" t="n"/>
@@ -3967,6 +4602,10 @@
         <v/>
       </c>
       <c r="J157" s="12" t="n"/>
+      <c r="K157" s="26">
+        <f>IF(ISNUMBER($D157),IF($D157&gt;=2,ROUND(($D157-1)*100,0),IF($D157&gt;1,ROUND(-100/($D157-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="158" ht="15" customHeight="1" s="23">
       <c r="A158" s="11" t="n"/>
@@ -3988,6 +4627,10 @@
         <v/>
       </c>
       <c r="J158" s="12" t="n"/>
+      <c r="K158" s="26">
+        <f>IF(ISNUMBER($D158),IF($D158&gt;=2,ROUND(($D158-1)*100,0),IF($D158&gt;1,ROUND(-100/($D158-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="159" ht="15" customHeight="1" s="23">
       <c r="A159" s="11" t="n"/>
@@ -4009,6 +4652,10 @@
         <v/>
       </c>
       <c r="J159" s="12" t="n"/>
+      <c r="K159" s="26">
+        <f>IF(ISNUMBER($D159),IF($D159&gt;=2,ROUND(($D159-1)*100,0),IF($D159&gt;1,ROUND(-100/($D159-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="160" ht="15" customHeight="1" s="23">
       <c r="A160" s="11" t="n"/>
@@ -4030,6 +4677,10 @@
         <v/>
       </c>
       <c r="J160" s="12" t="n"/>
+      <c r="K160" s="26">
+        <f>IF(ISNUMBER($D160),IF($D160&gt;=2,ROUND(($D160-1)*100,0),IF($D160&gt;1,ROUND(-100/($D160-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="161" ht="15" customHeight="1" s="23">
       <c r="A161" s="11" t="n"/>
@@ -4051,6 +4702,10 @@
         <v/>
       </c>
       <c r="J161" s="12" t="n"/>
+      <c r="K161" s="26">
+        <f>IF(ISNUMBER($D161),IF($D161&gt;=2,ROUND(($D161-1)*100,0),IF($D161&gt;1,ROUND(-100/($D161-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="162" ht="15" customHeight="1" s="23">
       <c r="A162" s="11" t="n"/>
@@ -4072,6 +4727,10 @@
         <v/>
       </c>
       <c r="J162" s="12" t="n"/>
+      <c r="K162" s="26">
+        <f>IF(ISNUMBER($D162),IF($D162&gt;=2,ROUND(($D162-1)*100,0),IF($D162&gt;1,ROUND(-100/($D162-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="163" ht="15" customHeight="1" s="23">
       <c r="A163" s="11" t="n"/>
@@ -4093,6 +4752,10 @@
         <v/>
       </c>
       <c r="J163" s="12" t="n"/>
+      <c r="K163" s="26">
+        <f>IF(ISNUMBER($D163),IF($D163&gt;=2,ROUND(($D163-1)*100,0),IF($D163&gt;1,ROUND(-100/($D163-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="164" ht="15" customHeight="1" s="23">
       <c r="A164" s="11" t="n"/>
@@ -4114,6 +4777,10 @@
         <v/>
       </c>
       <c r="J164" s="12" t="n"/>
+      <c r="K164" s="26">
+        <f>IF(ISNUMBER($D164),IF($D164&gt;=2,ROUND(($D164-1)*100,0),IF($D164&gt;1,ROUND(-100/($D164-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="165" ht="15" customHeight="1" s="23">
       <c r="A165" s="11" t="n"/>
@@ -4135,6 +4802,10 @@
         <v/>
       </c>
       <c r="J165" s="12" t="n"/>
+      <c r="K165" s="26">
+        <f>IF(ISNUMBER($D165),IF($D165&gt;=2,ROUND(($D165-1)*100,0),IF($D165&gt;1,ROUND(-100/($D165-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="166" ht="15" customHeight="1" s="23">
       <c r="A166" s="11" t="n"/>
@@ -4156,6 +4827,10 @@
         <v/>
       </c>
       <c r="J166" s="12" t="n"/>
+      <c r="K166" s="26">
+        <f>IF(ISNUMBER($D166),IF($D166&gt;=2,ROUND(($D166-1)*100,0),IF($D166&gt;1,ROUND(-100/($D166-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="167" ht="15" customHeight="1" s="23">
       <c r="A167" s="11" t="n"/>
@@ -4177,6 +4852,10 @@
         <v/>
       </c>
       <c r="J167" s="12" t="n"/>
+      <c r="K167" s="26">
+        <f>IF(ISNUMBER($D167),IF($D167&gt;=2,ROUND(($D167-1)*100,0),IF($D167&gt;1,ROUND(-100/($D167-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="168" ht="15" customHeight="1" s="23">
       <c r="A168" s="11" t="n"/>
@@ -4198,6 +4877,10 @@
         <v/>
       </c>
       <c r="J168" s="12" t="n"/>
+      <c r="K168" s="26">
+        <f>IF(ISNUMBER($D168),IF($D168&gt;=2,ROUND(($D168-1)*100,0),IF($D168&gt;1,ROUND(-100/($D168-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="169" ht="15" customHeight="1" s="23">
       <c r="A169" s="11" t="n"/>
@@ -4219,6 +4902,10 @@
         <v/>
       </c>
       <c r="J169" s="12" t="n"/>
+      <c r="K169" s="26">
+        <f>IF(ISNUMBER($D169),IF($D169&gt;=2,ROUND(($D169-1)*100,0),IF($D169&gt;1,ROUND(-100/($D169-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="170" ht="15" customHeight="1" s="23">
       <c r="A170" s="11" t="n"/>
@@ -4240,6 +4927,10 @@
         <v/>
       </c>
       <c r="J170" s="12" t="n"/>
+      <c r="K170" s="26">
+        <f>IF(ISNUMBER($D170),IF($D170&gt;=2,ROUND(($D170-1)*100,0),IF($D170&gt;1,ROUND(-100/($D170-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="171" ht="15" customHeight="1" s="23">
       <c r="A171" s="11" t="n"/>
@@ -4261,6 +4952,10 @@
         <v/>
       </c>
       <c r="J171" s="12" t="n"/>
+      <c r="K171" s="26">
+        <f>IF(ISNUMBER($D171),IF($D171&gt;=2,ROUND(($D171-1)*100,0),IF($D171&gt;1,ROUND(-100/($D171-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="172" ht="15" customHeight="1" s="23">
       <c r="A172" s="11" t="n"/>
@@ -4282,6 +4977,10 @@
         <v/>
       </c>
       <c r="J172" s="12" t="n"/>
+      <c r="K172" s="26">
+        <f>IF(ISNUMBER($D172),IF($D172&gt;=2,ROUND(($D172-1)*100,0),IF($D172&gt;1,ROUND(-100/($D172-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="173" ht="15" customHeight="1" s="23">
       <c r="A173" s="11" t="n"/>
@@ -4303,6 +5002,10 @@
         <v/>
       </c>
       <c r="J173" s="12" t="n"/>
+      <c r="K173" s="26">
+        <f>IF(ISNUMBER($D173),IF($D173&gt;=2,ROUND(($D173-1)*100,0),IF($D173&gt;1,ROUND(-100/($D173-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="174" ht="15" customHeight="1" s="23">
       <c r="A174" s="11" t="n"/>
@@ -4324,6 +5027,10 @@
         <v/>
       </c>
       <c r="J174" s="12" t="n"/>
+      <c r="K174" s="26">
+        <f>IF(ISNUMBER($D174),IF($D174&gt;=2,ROUND(($D174-1)*100,0),IF($D174&gt;1,ROUND(-100/($D174-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="175" ht="15" customHeight="1" s="23">
       <c r="A175" s="11" t="n"/>
@@ -4345,6 +5052,10 @@
         <v/>
       </c>
       <c r="J175" s="12" t="n"/>
+      <c r="K175" s="26">
+        <f>IF(ISNUMBER($D175),IF($D175&gt;=2,ROUND(($D175-1)*100,0),IF($D175&gt;1,ROUND(-100/($D175-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="176" ht="15" customHeight="1" s="23">
       <c r="A176" s="11" t="n"/>
@@ -4366,6 +5077,10 @@
         <v/>
       </c>
       <c r="J176" s="12" t="n"/>
+      <c r="K176" s="26">
+        <f>IF(ISNUMBER($D176),IF($D176&gt;=2,ROUND(($D176-1)*100,0),IF($D176&gt;1,ROUND(-100/($D176-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="177" ht="15" customHeight="1" s="23">
       <c r="A177" s="11" t="n"/>
@@ -4387,6 +5102,10 @@
         <v/>
       </c>
       <c r="J177" s="12" t="n"/>
+      <c r="K177" s="26">
+        <f>IF(ISNUMBER($D177),IF($D177&gt;=2,ROUND(($D177-1)*100,0),IF($D177&gt;1,ROUND(-100/($D177-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="178" ht="15" customHeight="1" s="23">
       <c r="A178" s="11" t="n"/>
@@ -4408,6 +5127,10 @@
         <v/>
       </c>
       <c r="J178" s="12" t="n"/>
+      <c r="K178" s="26">
+        <f>IF(ISNUMBER($D178),IF($D178&gt;=2,ROUND(($D178-1)*100,0),IF($D178&gt;1,ROUND(-100/($D178-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="179" ht="15" customHeight="1" s="23">
       <c r="A179" s="11" t="n"/>
@@ -4429,6 +5152,10 @@
         <v/>
       </c>
       <c r="J179" s="12" t="n"/>
+      <c r="K179" s="26">
+        <f>IF(ISNUMBER($D179),IF($D179&gt;=2,ROUND(($D179-1)*100,0),IF($D179&gt;1,ROUND(-100/($D179-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="180" ht="15" customHeight="1" s="23">
       <c r="A180" s="11" t="n"/>
@@ -4450,6 +5177,10 @@
         <v/>
       </c>
       <c r="J180" s="12" t="n"/>
+      <c r="K180" s="26">
+        <f>IF(ISNUMBER($D180),IF($D180&gt;=2,ROUND(($D180-1)*100,0),IF($D180&gt;1,ROUND(-100/($D180-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="181" ht="15" customHeight="1" s="23">
       <c r="A181" s="11" t="n"/>
@@ -4471,6 +5202,10 @@
         <v/>
       </c>
       <c r="J181" s="12" t="n"/>
+      <c r="K181" s="26">
+        <f>IF(ISNUMBER($D181),IF($D181&gt;=2,ROUND(($D181-1)*100,0),IF($D181&gt;1,ROUND(-100/($D181-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="182" ht="15" customHeight="1" s="23">
       <c r="A182" s="11" t="n"/>
@@ -4492,6 +5227,10 @@
         <v/>
       </c>
       <c r="J182" s="12" t="n"/>
+      <c r="K182" s="26">
+        <f>IF(ISNUMBER($D182),IF($D182&gt;=2,ROUND(($D182-1)*100,0),IF($D182&gt;1,ROUND(-100/($D182-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="183" ht="15" customHeight="1" s="23">
       <c r="A183" s="11" t="n"/>
@@ -4513,6 +5252,10 @@
         <v/>
       </c>
       <c r="J183" s="12" t="n"/>
+      <c r="K183" s="26">
+        <f>IF(ISNUMBER($D183),IF($D183&gt;=2,ROUND(($D183-1)*100,0),IF($D183&gt;1,ROUND(-100/($D183-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="184" ht="15" customHeight="1" s="23">
       <c r="A184" s="11" t="n"/>
@@ -4534,6 +5277,10 @@
         <v/>
       </c>
       <c r="J184" s="12" t="n"/>
+      <c r="K184" s="26">
+        <f>IF(ISNUMBER($D184),IF($D184&gt;=2,ROUND(($D184-1)*100,0),IF($D184&gt;1,ROUND(-100/($D184-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="185" ht="15" customHeight="1" s="23">
       <c r="A185" s="11" t="n"/>
@@ -4555,6 +5302,10 @@
         <v/>
       </c>
       <c r="J185" s="12" t="n"/>
+      <c r="K185" s="26">
+        <f>IF(ISNUMBER($D185),IF($D185&gt;=2,ROUND(($D185-1)*100,0),IF($D185&gt;1,ROUND(-100/($D185-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="186" ht="15" customHeight="1" s="23">
       <c r="A186" s="11" t="n"/>
@@ -4576,6 +5327,10 @@
         <v/>
       </c>
       <c r="J186" s="12" t="n"/>
+      <c r="K186" s="26">
+        <f>IF(ISNUMBER($D186),IF($D186&gt;=2,ROUND(($D186-1)*100,0),IF($D186&gt;1,ROUND(-100/($D186-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="187" ht="15" customHeight="1" s="23">
       <c r="A187" s="11" t="n"/>
@@ -4597,6 +5352,10 @@
         <v/>
       </c>
       <c r="J187" s="12" t="n"/>
+      <c r="K187" s="26">
+        <f>IF(ISNUMBER($D187),IF($D187&gt;=2,ROUND(($D187-1)*100,0),IF($D187&gt;1,ROUND(-100/($D187-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="188" ht="15" customHeight="1" s="23">
       <c r="A188" s="11" t="n"/>
@@ -4618,6 +5377,10 @@
         <v/>
       </c>
       <c r="J188" s="12" t="n"/>
+      <c r="K188" s="26">
+        <f>IF(ISNUMBER($D188),IF($D188&gt;=2,ROUND(($D188-1)*100,0),IF($D188&gt;1,ROUND(-100/($D188-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="189" ht="15" customHeight="1" s="23">
       <c r="A189" s="11" t="n"/>
@@ -4639,6 +5402,10 @@
         <v/>
       </c>
       <c r="J189" s="12" t="n"/>
+      <c r="K189" s="26">
+        <f>IF(ISNUMBER($D189),IF($D189&gt;=2,ROUND(($D189-1)*100,0),IF($D189&gt;1,ROUND(-100/($D189-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="190" ht="15" customHeight="1" s="23">
       <c r="A190" s="11" t="n"/>
@@ -4660,6 +5427,10 @@
         <v/>
       </c>
       <c r="J190" s="12" t="n"/>
+      <c r="K190" s="26">
+        <f>IF(ISNUMBER($D190),IF($D190&gt;=2,ROUND(($D190-1)*100,0),IF($D190&gt;1,ROUND(-100/($D190-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="191" ht="15" customHeight="1" s="23">
       <c r="A191" s="11" t="n"/>
@@ -4681,6 +5452,10 @@
         <v/>
       </c>
       <c r="J191" s="12" t="n"/>
+      <c r="K191" s="26">
+        <f>IF(ISNUMBER($D191),IF($D191&gt;=2,ROUND(($D191-1)*100,0),IF($D191&gt;1,ROUND(-100/($D191-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="192" ht="15" customHeight="1" s="23">
       <c r="A192" s="11" t="n"/>
@@ -4702,6 +5477,10 @@
         <v/>
       </c>
       <c r="J192" s="12" t="n"/>
+      <c r="K192" s="26">
+        <f>IF(ISNUMBER($D192),IF($D192&gt;=2,ROUND(($D192-1)*100,0),IF($D192&gt;1,ROUND(-100/($D192-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="193" ht="15" customHeight="1" s="23">
       <c r="A193" s="11" t="n"/>
@@ -4723,6 +5502,10 @@
         <v/>
       </c>
       <c r="J193" s="12" t="n"/>
+      <c r="K193" s="26">
+        <f>IF(ISNUMBER($D193),IF($D193&gt;=2,ROUND(($D193-1)*100,0),IF($D193&gt;1,ROUND(-100/($D193-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="194" ht="15" customHeight="1" s="23">
       <c r="A194" s="11" t="n"/>
@@ -4744,6 +5527,10 @@
         <v/>
       </c>
       <c r="J194" s="12" t="n"/>
+      <c r="K194" s="26">
+        <f>IF(ISNUMBER($D194),IF($D194&gt;=2,ROUND(($D194-1)*100,0),IF($D194&gt;1,ROUND(-100/($D194-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="195" ht="15" customHeight="1" s="23">
       <c r="A195" s="11" t="n"/>
@@ -4765,6 +5552,10 @@
         <v/>
       </c>
       <c r="J195" s="12" t="n"/>
+      <c r="K195" s="26">
+        <f>IF(ISNUMBER($D195),IF($D195&gt;=2,ROUND(($D195-1)*100,0),IF($D195&gt;1,ROUND(-100/($D195-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="196" ht="15" customHeight="1" s="23">
       <c r="A196" s="11" t="n"/>
@@ -4786,6 +5577,10 @@
         <v/>
       </c>
       <c r="J196" s="12" t="n"/>
+      <c r="K196" s="26">
+        <f>IF(ISNUMBER($D196),IF($D196&gt;=2,ROUND(($D196-1)*100,0),IF($D196&gt;1,ROUND(-100/($D196-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="197" ht="15" customHeight="1" s="23">
       <c r="A197" s="11" t="n"/>
@@ -4807,6 +5602,10 @@
         <v/>
       </c>
       <c r="J197" s="12" t="n"/>
+      <c r="K197" s="26">
+        <f>IF(ISNUMBER($D197),IF($D197&gt;=2,ROUND(($D197-1)*100,0),IF($D197&gt;1,ROUND(-100/($D197-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="198" ht="15" customHeight="1" s="23">
       <c r="A198" s="11" t="n"/>
@@ -4828,6 +5627,10 @@
         <v/>
       </c>
       <c r="J198" s="12" t="n"/>
+      <c r="K198" s="26">
+        <f>IF(ISNUMBER($D198),IF($D198&gt;=2,ROUND(($D198-1)*100,0),IF($D198&gt;1,ROUND(-100/($D198-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="199" ht="15" customHeight="1" s="23">
       <c r="A199" s="11" t="n"/>
@@ -4849,6 +5652,10 @@
         <v/>
       </c>
       <c r="J199" s="12" t="n"/>
+      <c r="K199" s="26">
+        <f>IF(ISNUMBER($D199),IF($D199&gt;=2,ROUND(($D199-1)*100,0),IF($D199&gt;1,ROUND(-100/($D199-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="200" ht="15" customHeight="1" s="23">
       <c r="A200" s="11" t="n"/>
@@ -4870,6 +5677,10 @@
         <v/>
       </c>
       <c r="J200" s="12" t="n"/>
+      <c r="K200" s="26">
+        <f>IF(ISNUMBER($D200),IF($D200&gt;=2,ROUND(($D200-1)*100,0),IF($D200&gt;1,ROUND(-100/($D200-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="201" ht="15" customHeight="1" s="23">
       <c r="A201" s="11" t="n"/>
@@ -4891,6 +5702,10 @@
         <v/>
       </c>
       <c r="J201" s="12" t="n"/>
+      <c r="K201" s="26">
+        <f>IF(ISNUMBER($D201),IF($D201&gt;=2,ROUND(($D201-1)*100,0),IF($D201&gt;1,ROUND(-100/($D201-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="202" ht="15" customHeight="1" s="23">
       <c r="A202" s="11" t="n"/>
@@ -4912,6 +5727,10 @@
         <v/>
       </c>
       <c r="J202" s="12" t="n"/>
+      <c r="K202" s="26">
+        <f>IF(ISNUMBER($D202),IF($D202&gt;=2,ROUND(($D202-1)*100,0),IF($D202&gt;1,ROUND(-100/($D202-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="203" ht="15" customHeight="1" s="23">
       <c r="A203" s="11" t="n"/>
@@ -4933,6 +5752,10 @@
         <v/>
       </c>
       <c r="J203" s="12" t="n"/>
+      <c r="K203" s="26">
+        <f>IF(ISNUMBER($D203),IF($D203&gt;=2,ROUND(($D203-1)*100,0),IF($D203&gt;1,ROUND(-100/($D203-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="204" ht="15" customHeight="1" s="23">
       <c r="A204" s="11" t="n"/>
@@ -4954,6 +5777,10 @@
         <v/>
       </c>
       <c r="J204" s="12" t="n"/>
+      <c r="K204" s="26">
+        <f>IF(ISNUMBER($D204),IF($D204&gt;=2,ROUND(($D204-1)*100,0),IF($D204&gt;1,ROUND(-100/($D204-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="205" ht="15" customHeight="1" s="23">
       <c r="A205" s="11" t="n"/>
@@ -4975,6 +5802,10 @@
         <v/>
       </c>
       <c r="J205" s="12" t="n"/>
+      <c r="K205" s="26">
+        <f>IF(ISNUMBER($D205),IF($D205&gt;=2,ROUND(($D205-1)*100,0),IF($D205&gt;1,ROUND(-100/($D205-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="206" ht="15" customHeight="1" s="23">
       <c r="A206" s="11" t="n"/>
@@ -4996,6 +5827,10 @@
         <v/>
       </c>
       <c r="J206" s="12" t="n"/>
+      <c r="K206" s="26">
+        <f>IF(ISNUMBER($D206),IF($D206&gt;=2,ROUND(($D206-1)*100,0),IF($D206&gt;1,ROUND(-100/($D206-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="207" ht="15" customHeight="1" s="23">
       <c r="A207" s="11" t="n"/>
@@ -5017,6 +5852,10 @@
         <v/>
       </c>
       <c r="J207" s="12" t="n"/>
+      <c r="K207" s="26">
+        <f>IF(ISNUMBER($D207),IF($D207&gt;=2,ROUND(($D207-1)*100,0),IF($D207&gt;1,ROUND(-100/($D207-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="208" ht="15" customHeight="1" s="23">
       <c r="A208" s="11" t="n"/>
@@ -5038,6 +5877,10 @@
         <v/>
       </c>
       <c r="J208" s="12" t="n"/>
+      <c r="K208" s="26">
+        <f>IF(ISNUMBER($D208),IF($D208&gt;=2,ROUND(($D208-1)*100,0),IF($D208&gt;1,ROUND(-100/($D208-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="209" ht="15" customHeight="1" s="23">
       <c r="A209" s="11" t="n"/>
@@ -5059,6 +5902,10 @@
         <v/>
       </c>
       <c r="J209" s="12" t="n"/>
+      <c r="K209" s="26">
+        <f>IF(ISNUMBER($D209),IF($D209&gt;=2,ROUND(($D209-1)*100,0),IF($D209&gt;1,ROUND(-100/($D209-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="210" ht="15" customHeight="1" s="23">
       <c r="A210" s="11" t="n"/>
@@ -5080,6 +5927,10 @@
         <v/>
       </c>
       <c r="J210" s="12" t="n"/>
+      <c r="K210" s="26">
+        <f>IF(ISNUMBER($D210),IF($D210&gt;=2,ROUND(($D210-1)*100,0),IF($D210&gt;1,ROUND(-100/($D210-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="211" ht="15" customHeight="1" s="23">
       <c r="A211" s="11" t="n"/>
@@ -5101,6 +5952,10 @@
         <v/>
       </c>
       <c r="J211" s="12" t="n"/>
+      <c r="K211" s="26">
+        <f>IF(ISNUMBER($D211),IF($D211&gt;=2,ROUND(($D211-1)*100,0),IF($D211&gt;1,ROUND(-100/($D211-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="212" ht="15" customHeight="1" s="23">
       <c r="A212" s="11" t="n"/>
@@ -5122,6 +5977,10 @@
         <v/>
       </c>
       <c r="J212" s="12" t="n"/>
+      <c r="K212" s="26">
+        <f>IF(ISNUMBER($D212),IF($D212&gt;=2,ROUND(($D212-1)*100,0),IF($D212&gt;1,ROUND(-100/($D212-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="213" ht="15" customHeight="1" s="23">
       <c r="A213" s="11" t="n"/>
@@ -5143,6 +6002,10 @@
         <v/>
       </c>
       <c r="J213" s="12" t="n"/>
+      <c r="K213" s="26">
+        <f>IF(ISNUMBER($D213),IF($D213&gt;=2,ROUND(($D213-1)*100,0),IF($D213&gt;1,ROUND(-100/($D213-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="214" ht="15" customHeight="1" s="23">
       <c r="A214" s="11" t="n"/>
@@ -5164,6 +6027,10 @@
         <v/>
       </c>
       <c r="J214" s="12" t="n"/>
+      <c r="K214" s="26">
+        <f>IF(ISNUMBER($D214),IF($D214&gt;=2,ROUND(($D214-1)*100,0),IF($D214&gt;1,ROUND(-100/($D214-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="215" ht="15" customHeight="1" s="23">
       <c r="A215" s="11" t="n"/>
@@ -5185,6 +6052,10 @@
         <v/>
       </c>
       <c r="J215" s="12" t="n"/>
+      <c r="K215" s="26">
+        <f>IF(ISNUMBER($D215),IF($D215&gt;=2,ROUND(($D215-1)*100,0),IF($D215&gt;1,ROUND(-100/($D215-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="216" ht="15" customHeight="1" s="23">
       <c r="A216" s="11" t="n"/>
@@ -5206,6 +6077,10 @@
         <v/>
       </c>
       <c r="J216" s="12" t="n"/>
+      <c r="K216" s="26">
+        <f>IF(ISNUMBER($D216),IF($D216&gt;=2,ROUND(($D216-1)*100,0),IF($D216&gt;1,ROUND(-100/($D216-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="217" ht="15" customHeight="1" s="23">
       <c r="A217" s="11" t="n"/>
@@ -5227,6 +6102,10 @@
         <v/>
       </c>
       <c r="J217" s="12" t="n"/>
+      <c r="K217" s="26">
+        <f>IF(ISNUMBER($D217),IF($D217&gt;=2,ROUND(($D217-1)*100,0),IF($D217&gt;1,ROUND(-100/($D217-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="218" ht="15" customHeight="1" s="23">
       <c r="A218" s="11" t="n"/>
@@ -5248,6 +6127,10 @@
         <v/>
       </c>
       <c r="J218" s="12" t="n"/>
+      <c r="K218" s="26">
+        <f>IF(ISNUMBER($D218),IF($D218&gt;=2,ROUND(($D218-1)*100,0),IF($D218&gt;1,ROUND(-100/($D218-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="219" ht="15" customHeight="1" s="23">
       <c r="A219" s="11" t="n"/>
@@ -5269,6 +6152,10 @@
         <v/>
       </c>
       <c r="J219" s="12" t="n"/>
+      <c r="K219" s="26">
+        <f>IF(ISNUMBER($D219),IF($D219&gt;=2,ROUND(($D219-1)*100,0),IF($D219&gt;1,ROUND(-100/($D219-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="220" ht="15" customHeight="1" s="23">
       <c r="A220" s="11" t="n"/>
@@ -5290,6 +6177,10 @@
         <v/>
       </c>
       <c r="J220" s="12" t="n"/>
+      <c r="K220" s="26">
+        <f>IF(ISNUMBER($D220),IF($D220&gt;=2,ROUND(($D220-1)*100,0),IF($D220&gt;1,ROUND(-100/($D220-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="221" ht="15" customHeight="1" s="23">
       <c r="A221" s="11" t="n"/>
@@ -5311,6 +6202,10 @@
         <v/>
       </c>
       <c r="J221" s="12" t="n"/>
+      <c r="K221" s="26">
+        <f>IF(ISNUMBER($D221),IF($D221&gt;=2,ROUND(($D221-1)*100,0),IF($D221&gt;1,ROUND(-100/($D221-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="222" ht="15" customHeight="1" s="23">
       <c r="A222" s="11" t="n"/>
@@ -5332,6 +6227,10 @@
         <v/>
       </c>
       <c r="J222" s="12" t="n"/>
+      <c r="K222" s="26">
+        <f>IF(ISNUMBER($D222),IF($D222&gt;=2,ROUND(($D222-1)*100,0),IF($D222&gt;1,ROUND(-100/($D222-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="223" ht="15" customHeight="1" s="23">
       <c r="A223" s="11" t="n"/>
@@ -5353,6 +6252,10 @@
         <v/>
       </c>
       <c r="J223" s="12" t="n"/>
+      <c r="K223" s="26">
+        <f>IF(ISNUMBER($D223),IF($D223&gt;=2,ROUND(($D223-1)*100,0),IF($D223&gt;1,ROUND(-100/($D223-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="224" ht="15" customHeight="1" s="23">
       <c r="A224" s="11" t="n"/>
@@ -5374,6 +6277,10 @@
         <v/>
       </c>
       <c r="J224" s="12" t="n"/>
+      <c r="K224" s="26">
+        <f>IF(ISNUMBER($D224),IF($D224&gt;=2,ROUND(($D224-1)*100,0),IF($D224&gt;1,ROUND(-100/($D224-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="225" ht="15" customHeight="1" s="23">
       <c r="A225" s="11" t="n"/>
@@ -5395,6 +6302,10 @@
         <v/>
       </c>
       <c r="J225" s="12" t="n"/>
+      <c r="K225" s="26">
+        <f>IF(ISNUMBER($D225),IF($D225&gt;=2,ROUND(($D225-1)*100,0),IF($D225&gt;1,ROUND(-100/($D225-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="226" ht="15" customHeight="1" s="23">
       <c r="A226" s="11" t="n"/>
@@ -5416,6 +6327,10 @@
         <v/>
       </c>
       <c r="J226" s="12" t="n"/>
+      <c r="K226" s="26">
+        <f>IF(ISNUMBER($D226),IF($D226&gt;=2,ROUND(($D226-1)*100,0),IF($D226&gt;1,ROUND(-100/($D226-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="227" ht="15" customHeight="1" s="23">
       <c r="A227" s="11" t="n"/>
@@ -5437,6 +6352,10 @@
         <v/>
       </c>
       <c r="J227" s="12" t="n"/>
+      <c r="K227" s="26">
+        <f>IF(ISNUMBER($D227),IF($D227&gt;=2,ROUND(($D227-1)*100,0),IF($D227&gt;1,ROUND(-100/($D227-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="228" ht="15" customHeight="1" s="23">
       <c r="A228" s="11" t="n"/>
@@ -5458,6 +6377,10 @@
         <v/>
       </c>
       <c r="J228" s="12" t="n"/>
+      <c r="K228" s="26">
+        <f>IF(ISNUMBER($D228),IF($D228&gt;=2,ROUND(($D228-1)*100,0),IF($D228&gt;1,ROUND(-100/($D228-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="229" ht="15" customHeight="1" s="23">
       <c r="A229" s="11" t="n"/>
@@ -5479,6 +6402,10 @@
         <v/>
       </c>
       <c r="J229" s="12" t="n"/>
+      <c r="K229" s="26">
+        <f>IF(ISNUMBER($D229),IF($D229&gt;=2,ROUND(($D229-1)*100,0),IF($D229&gt;1,ROUND(-100/($D229-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="230" ht="15" customHeight="1" s="23">
       <c r="A230" s="11" t="n"/>
@@ -5500,6 +6427,10 @@
         <v/>
       </c>
       <c r="J230" s="12" t="n"/>
+      <c r="K230" s="26">
+        <f>IF(ISNUMBER($D230),IF($D230&gt;=2,ROUND(($D230-1)*100,0),IF($D230&gt;1,ROUND(-100/($D230-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="231" ht="15" customHeight="1" s="23">
       <c r="A231" s="11" t="n"/>
@@ -5521,6 +6452,10 @@
         <v/>
       </c>
       <c r="J231" s="12" t="n"/>
+      <c r="K231" s="26">
+        <f>IF(ISNUMBER($D231),IF($D231&gt;=2,ROUND(($D231-1)*100,0),IF($D231&gt;1,ROUND(-100/($D231-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="232" ht="15" customHeight="1" s="23">
       <c r="A232" s="11" t="n"/>
@@ -5542,6 +6477,10 @@
         <v/>
       </c>
       <c r="J232" s="12" t="n"/>
+      <c r="K232" s="26">
+        <f>IF(ISNUMBER($D232),IF($D232&gt;=2,ROUND(($D232-1)*100,0),IF($D232&gt;1,ROUND(-100/($D232-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="233" ht="15" customHeight="1" s="23">
       <c r="A233" s="11" t="n"/>
@@ -5563,6 +6502,10 @@
         <v/>
       </c>
       <c r="J233" s="12" t="n"/>
+      <c r="K233" s="26">
+        <f>IF(ISNUMBER($D233),IF($D233&gt;=2,ROUND(($D233-1)*100,0),IF($D233&gt;1,ROUND(-100/($D233-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="234" ht="15" customHeight="1" s="23">
       <c r="A234" s="11" t="n"/>
@@ -5584,6 +6527,10 @@
         <v/>
       </c>
       <c r="J234" s="12" t="n"/>
+      <c r="K234" s="26">
+        <f>IF(ISNUMBER($D234),IF($D234&gt;=2,ROUND(($D234-1)*100,0),IF($D234&gt;1,ROUND(-100/($D234-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="235" ht="15" customHeight="1" s="23">
       <c r="A235" s="11" t="n"/>
@@ -5605,6 +6552,10 @@
         <v/>
       </c>
       <c r="J235" s="12" t="n"/>
+      <c r="K235" s="26">
+        <f>IF(ISNUMBER($D235),IF($D235&gt;=2,ROUND(($D235-1)*100,0),IF($D235&gt;1,ROUND(-100/($D235-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="236" ht="15" customHeight="1" s="23">
       <c r="A236" s="11" t="n"/>
@@ -5626,6 +6577,10 @@
         <v/>
       </c>
       <c r="J236" s="12" t="n"/>
+      <c r="K236" s="26">
+        <f>IF(ISNUMBER($D236),IF($D236&gt;=2,ROUND(($D236-1)*100,0),IF($D236&gt;1,ROUND(-100/($D236-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="237" ht="15" customHeight="1" s="23">
       <c r="A237" s="11" t="n"/>
@@ -5647,6 +6602,10 @@
         <v/>
       </c>
       <c r="J237" s="12" t="n"/>
+      <c r="K237" s="26">
+        <f>IF(ISNUMBER($D237),IF($D237&gt;=2,ROUND(($D237-1)*100,0),IF($D237&gt;1,ROUND(-100/($D237-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="238" ht="15" customHeight="1" s="23">
       <c r="A238" s="11" t="n"/>
@@ -5668,6 +6627,10 @@
         <v/>
       </c>
       <c r="J238" s="12" t="n"/>
+      <c r="K238" s="26">
+        <f>IF(ISNUMBER($D238),IF($D238&gt;=2,ROUND(($D238-1)*100,0),IF($D238&gt;1,ROUND(-100/($D238-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="239" ht="15" customHeight="1" s="23">
       <c r="A239" s="11" t="n"/>
@@ -5689,6 +6652,10 @@
         <v/>
       </c>
       <c r="J239" s="12" t="n"/>
+      <c r="K239" s="26">
+        <f>IF(ISNUMBER($D239),IF($D239&gt;=2,ROUND(($D239-1)*100,0),IF($D239&gt;1,ROUND(-100/($D239-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="240" ht="15" customHeight="1" s="23">
       <c r="A240" s="11" t="n"/>
@@ -5710,6 +6677,10 @@
         <v/>
       </c>
       <c r="J240" s="12" t="n"/>
+      <c r="K240" s="26">
+        <f>IF(ISNUMBER($D240),IF($D240&gt;=2,ROUND(($D240-1)*100,0),IF($D240&gt;1,ROUND(-100/($D240-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="241" ht="15" customHeight="1" s="23">
       <c r="A241" s="11" t="n"/>
@@ -5731,6 +6702,10 @@
         <v/>
       </c>
       <c r="J241" s="12" t="n"/>
+      <c r="K241" s="26">
+        <f>IF(ISNUMBER($D241),IF($D241&gt;=2,ROUND(($D241-1)*100,0),IF($D241&gt;1,ROUND(-100/($D241-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="242" ht="15" customHeight="1" s="23">
       <c r="A242" s="11" t="n"/>
@@ -5752,6 +6727,10 @@
         <v/>
       </c>
       <c r="J242" s="12" t="n"/>
+      <c r="K242" s="26">
+        <f>IF(ISNUMBER($D242),IF($D242&gt;=2,ROUND(($D242-1)*100,0),IF($D242&gt;1,ROUND(-100/($D242-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="243" ht="15" customHeight="1" s="23">
       <c r="A243" s="11" t="n"/>
@@ -5773,6 +6752,10 @@
         <v/>
       </c>
       <c r="J243" s="12" t="n"/>
+      <c r="K243" s="26">
+        <f>IF(ISNUMBER($D243),IF($D243&gt;=2,ROUND(($D243-1)*100,0),IF($D243&gt;1,ROUND(-100/($D243-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="244" ht="15" customHeight="1" s="23">
       <c r="A244" s="11" t="n"/>
@@ -5794,6 +6777,10 @@
         <v/>
       </c>
       <c r="J244" s="12" t="n"/>
+      <c r="K244" s="26">
+        <f>IF(ISNUMBER($D244),IF($D244&gt;=2,ROUND(($D244-1)*100,0),IF($D244&gt;1,ROUND(-100/($D244-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="245" ht="15" customHeight="1" s="23">
       <c r="A245" s="11" t="n"/>
@@ -5815,6 +6802,10 @@
         <v/>
       </c>
       <c r="J245" s="12" t="n"/>
+      <c r="K245" s="26">
+        <f>IF(ISNUMBER($D245),IF($D245&gt;=2,ROUND(($D245-1)*100,0),IF($D245&gt;1,ROUND(-100/($D245-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="246" ht="15" customHeight="1" s="23">
       <c r="A246" s="11" t="n"/>
@@ -5836,6 +6827,10 @@
         <v/>
       </c>
       <c r="J246" s="12" t="n"/>
+      <c r="K246" s="26">
+        <f>IF(ISNUMBER($D246),IF($D246&gt;=2,ROUND(($D246-1)*100,0),IF($D246&gt;1,ROUND(-100/($D246-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="247" ht="15" customHeight="1" s="23">
       <c r="A247" s="11" t="n"/>
@@ -5857,6 +6852,10 @@
         <v/>
       </c>
       <c r="J247" s="12" t="n"/>
+      <c r="K247" s="26">
+        <f>IF(ISNUMBER($D247),IF($D247&gt;=2,ROUND(($D247-1)*100,0),IF($D247&gt;1,ROUND(-100/($D247-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="248" ht="15" customHeight="1" s="23">
       <c r="A248" s="11" t="n"/>
@@ -5878,6 +6877,10 @@
         <v/>
       </c>
       <c r="J248" s="12" t="n"/>
+      <c r="K248" s="26">
+        <f>IF(ISNUMBER($D248),IF($D248&gt;=2,ROUND(($D248-1)*100,0),IF($D248&gt;1,ROUND(-100/($D248-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="249" ht="15" customHeight="1" s="23">
       <c r="A249" s="11" t="n"/>
@@ -5899,6 +6902,10 @@
         <v/>
       </c>
       <c r="J249" s="12" t="n"/>
+      <c r="K249" s="26">
+        <f>IF(ISNUMBER($D249),IF($D249&gt;=2,ROUND(($D249-1)*100,0),IF($D249&gt;1,ROUND(-100/($D249-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="250" ht="15" customHeight="1" s="23">
       <c r="A250" s="11" t="n"/>
@@ -5920,6 +6927,10 @@
         <v/>
       </c>
       <c r="J250" s="12" t="n"/>
+      <c r="K250" s="26">
+        <f>IF(ISNUMBER($D250),IF($D250&gt;=2,ROUND(($D250-1)*100,0),IF($D250&gt;1,ROUND(-100/($D250-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="251" ht="15" customHeight="1" s="23">
       <c r="A251" s="11" t="n"/>
@@ -5941,6 +6952,10 @@
         <v/>
       </c>
       <c r="J251" s="12" t="n"/>
+      <c r="K251" s="26">
+        <f>IF(ISNUMBER($D251),IF($D251&gt;=2,ROUND(($D251-1)*100,0),IF($D251&gt;1,ROUND(-100/($D251-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="252" ht="15" customHeight="1" s="23">
       <c r="A252" s="11" t="n"/>
@@ -5962,6 +6977,10 @@
         <v/>
       </c>
       <c r="J252" s="12" t="n"/>
+      <c r="K252" s="26">
+        <f>IF(ISNUMBER($D252),IF($D252&gt;=2,ROUND(($D252-1)*100,0),IF($D252&gt;1,ROUND(-100/($D252-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="253" ht="15" customHeight="1" s="23">
       <c r="A253" s="11" t="n"/>
@@ -5983,6 +7002,10 @@
         <v/>
       </c>
       <c r="J253" s="12" t="n"/>
+      <c r="K253" s="26">
+        <f>IF(ISNUMBER($D253),IF($D253&gt;=2,ROUND(($D253-1)*100,0),IF($D253&gt;1,ROUND(-100/($D253-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="254" ht="15" customHeight="1" s="23">
       <c r="A254" s="11" t="n"/>
@@ -6004,6 +7027,10 @@
         <v/>
       </c>
       <c r="J254" s="12" t="n"/>
+      <c r="K254" s="26">
+        <f>IF(ISNUMBER($D254),IF($D254&gt;=2,ROUND(($D254-1)*100,0),IF($D254&gt;1,ROUND(-100/($D254-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="255" ht="15" customHeight="1" s="23">
       <c r="A255" s="11" t="n"/>
@@ -6025,6 +7052,10 @@
         <v/>
       </c>
       <c r="J255" s="12" t="n"/>
+      <c r="K255" s="26">
+        <f>IF(ISNUMBER($D255),IF($D255&gt;=2,ROUND(($D255-1)*100,0),IF($D255&gt;1,ROUND(-100/($D255-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="256" ht="15" customHeight="1" s="23">
       <c r="A256" s="11" t="n"/>
@@ -6046,6 +7077,10 @@
         <v/>
       </c>
       <c r="J256" s="12" t="n"/>
+      <c r="K256" s="26">
+        <f>IF(ISNUMBER($D256),IF($D256&gt;=2,ROUND(($D256-1)*100,0),IF($D256&gt;1,ROUND(-100/($D256-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="257" ht="15" customHeight="1" s="23">
       <c r="A257" s="11" t="n"/>
@@ -6067,6 +7102,10 @@
         <v/>
       </c>
       <c r="J257" s="12" t="n"/>
+      <c r="K257" s="26">
+        <f>IF(ISNUMBER($D257),IF($D257&gt;=2,ROUND(($D257-1)*100,0),IF($D257&gt;1,ROUND(-100/($D257-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="258" ht="15" customHeight="1" s="23">
       <c r="A258" s="11" t="n"/>
@@ -6088,6 +7127,10 @@
         <v/>
       </c>
       <c r="J258" s="12" t="n"/>
+      <c r="K258" s="26">
+        <f>IF(ISNUMBER($D258),IF($D258&gt;=2,ROUND(($D258-1)*100,0),IF($D258&gt;1,ROUND(-100/($D258-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="259" ht="15" customHeight="1" s="23">
       <c r="A259" s="11" t="n"/>
@@ -6109,6 +7152,10 @@
         <v/>
       </c>
       <c r="J259" s="12" t="n"/>
+      <c r="K259" s="26">
+        <f>IF(ISNUMBER($D259),IF($D259&gt;=2,ROUND(($D259-1)*100,0),IF($D259&gt;1,ROUND(-100/($D259-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="260" ht="15" customHeight="1" s="23">
       <c r="A260" s="11" t="n"/>
@@ -6130,6 +7177,10 @@
         <v/>
       </c>
       <c r="J260" s="12" t="n"/>
+      <c r="K260" s="26">
+        <f>IF(ISNUMBER($D260),IF($D260&gt;=2,ROUND(($D260-1)*100,0),IF($D260&gt;1,ROUND(-100/($D260-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="261" ht="15" customHeight="1" s="23">
       <c r="A261" s="11" t="n"/>
@@ -6151,6 +7202,10 @@
         <v/>
       </c>
       <c r="J261" s="12" t="n"/>
+      <c r="K261" s="26">
+        <f>IF(ISNUMBER($D261),IF($D261&gt;=2,ROUND(($D261-1)*100,0),IF($D261&gt;1,ROUND(-100/($D261-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="262" ht="15" customHeight="1" s="23">
       <c r="A262" s="11" t="n"/>
@@ -6172,6 +7227,10 @@
         <v/>
       </c>
       <c r="J262" s="12" t="n"/>
+      <c r="K262" s="26">
+        <f>IF(ISNUMBER($D262),IF($D262&gt;=2,ROUND(($D262-1)*100,0),IF($D262&gt;1,ROUND(-100/($D262-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="263" ht="15" customHeight="1" s="23">
       <c r="A263" s="11" t="n"/>
@@ -6193,6 +7252,10 @@
         <v/>
       </c>
       <c r="J263" s="12" t="n"/>
+      <c r="K263" s="26">
+        <f>IF(ISNUMBER($D263),IF($D263&gt;=2,ROUND(($D263-1)*100,0),IF($D263&gt;1,ROUND(-100/($D263-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="264" ht="15" customHeight="1" s="23">
       <c r="A264" s="11" t="n"/>
@@ -6214,6 +7277,10 @@
         <v/>
       </c>
       <c r="J264" s="12" t="n"/>
+      <c r="K264" s="26">
+        <f>IF(ISNUMBER($D264),IF($D264&gt;=2,ROUND(($D264-1)*100,0),IF($D264&gt;1,ROUND(-100/($D264-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="265" ht="15" customHeight="1" s="23">
       <c r="A265" s="11" t="n"/>
@@ -6235,6 +7302,10 @@
         <v/>
       </c>
       <c r="J265" s="12" t="n"/>
+      <c r="K265" s="26">
+        <f>IF(ISNUMBER($D265),IF($D265&gt;=2,ROUND(($D265-1)*100,0),IF($D265&gt;1,ROUND(-100/($D265-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="266" ht="15" customHeight="1" s="23">
       <c r="A266" s="11" t="n"/>
@@ -6256,6 +7327,10 @@
         <v/>
       </c>
       <c r="J266" s="12" t="n"/>
+      <c r="K266" s="26">
+        <f>IF(ISNUMBER($D266),IF($D266&gt;=2,ROUND(($D266-1)*100,0),IF($D266&gt;1,ROUND(-100/($D266-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="267" ht="15" customHeight="1" s="23">
       <c r="A267" s="11" t="n"/>
@@ -6277,6 +7352,10 @@
         <v/>
       </c>
       <c r="J267" s="12" t="n"/>
+      <c r="K267" s="26">
+        <f>IF(ISNUMBER($D267),IF($D267&gt;=2,ROUND(($D267-1)*100,0),IF($D267&gt;1,ROUND(-100/($D267-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="268" ht="15" customHeight="1" s="23">
       <c r="A268" s="11" t="n"/>
@@ -6298,6 +7377,10 @@
         <v/>
       </c>
       <c r="J268" s="12" t="n"/>
+      <c r="K268" s="26">
+        <f>IF(ISNUMBER($D268),IF($D268&gt;=2,ROUND(($D268-1)*100,0),IF($D268&gt;1,ROUND(-100/($D268-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="269" ht="15" customHeight="1" s="23">
       <c r="A269" s="11" t="n"/>
@@ -6319,6 +7402,10 @@
         <v/>
       </c>
       <c r="J269" s="12" t="n"/>
+      <c r="K269" s="26">
+        <f>IF(ISNUMBER($D269),IF($D269&gt;=2,ROUND(($D269-1)*100,0),IF($D269&gt;1,ROUND(-100/($D269-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="270" ht="15" customHeight="1" s="23">
       <c r="A270" s="11" t="n"/>
@@ -6340,6 +7427,10 @@
         <v/>
       </c>
       <c r="J270" s="12" t="n"/>
+      <c r="K270" s="26">
+        <f>IF(ISNUMBER($D270),IF($D270&gt;=2,ROUND(($D270-1)*100,0),IF($D270&gt;1,ROUND(-100/($D270-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="271" ht="15" customHeight="1" s="23">
       <c r="A271" s="11" t="n"/>
@@ -6361,6 +7452,10 @@
         <v/>
       </c>
       <c r="J271" s="12" t="n"/>
+      <c r="K271" s="26">
+        <f>IF(ISNUMBER($D271),IF($D271&gt;=2,ROUND(($D271-1)*100,0),IF($D271&gt;1,ROUND(-100/($D271-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="272" ht="15" customHeight="1" s="23">
       <c r="A272" s="11" t="n"/>
@@ -6382,6 +7477,10 @@
         <v/>
       </c>
       <c r="J272" s="12" t="n"/>
+      <c r="K272" s="26">
+        <f>IF(ISNUMBER($D272),IF($D272&gt;=2,ROUND(($D272-1)*100,0),IF($D272&gt;1,ROUND(-100/($D272-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="273" ht="15" customHeight="1" s="23">
       <c r="A273" s="11" t="n"/>
@@ -6403,6 +7502,10 @@
         <v/>
       </c>
       <c r="J273" s="12" t="n"/>
+      <c r="K273" s="26">
+        <f>IF(ISNUMBER($D273),IF($D273&gt;=2,ROUND(($D273-1)*100,0),IF($D273&gt;1,ROUND(-100/($D273-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="274" ht="15" customHeight="1" s="23">
       <c r="A274" s="11" t="n"/>
@@ -6424,6 +7527,10 @@
         <v/>
       </c>
       <c r="J274" s="12" t="n"/>
+      <c r="K274" s="26">
+        <f>IF(ISNUMBER($D274),IF($D274&gt;=2,ROUND(($D274-1)*100,0),IF($D274&gt;1,ROUND(-100/($D274-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="275" ht="15" customHeight="1" s="23">
       <c r="A275" s="11" t="n"/>
@@ -6445,6 +7552,10 @@
         <v/>
       </c>
       <c r="J275" s="12" t="n"/>
+      <c r="K275" s="26">
+        <f>IF(ISNUMBER($D275),IF($D275&gt;=2,ROUND(($D275-1)*100,0),IF($D275&gt;1,ROUND(-100/($D275-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="276" ht="15" customHeight="1" s="23">
       <c r="A276" s="11" t="n"/>
@@ -6466,6 +7577,10 @@
         <v/>
       </c>
       <c r="J276" s="12" t="n"/>
+      <c r="K276" s="26">
+        <f>IF(ISNUMBER($D276),IF($D276&gt;=2,ROUND(($D276-1)*100,0),IF($D276&gt;1,ROUND(-100/($D276-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="277" ht="15" customHeight="1" s="23">
       <c r="A277" s="11" t="n"/>
@@ -6487,6 +7602,10 @@
         <v/>
       </c>
       <c r="J277" s="12" t="n"/>
+      <c r="K277" s="26">
+        <f>IF(ISNUMBER($D277),IF($D277&gt;=2,ROUND(($D277-1)*100,0),IF($D277&gt;1,ROUND(-100/($D277-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="278" ht="15" customHeight="1" s="23">
       <c r="A278" s="11" t="n"/>
@@ -6508,6 +7627,10 @@
         <v/>
       </c>
       <c r="J278" s="12" t="n"/>
+      <c r="K278" s="26">
+        <f>IF(ISNUMBER($D278),IF($D278&gt;=2,ROUND(($D278-1)*100,0),IF($D278&gt;1,ROUND(-100/($D278-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="279" ht="15" customHeight="1" s="23">
       <c r="A279" s="11" t="n"/>
@@ -6529,6 +7652,10 @@
         <v/>
       </c>
       <c r="J279" s="12" t="n"/>
+      <c r="K279" s="26">
+        <f>IF(ISNUMBER($D279),IF($D279&gt;=2,ROUND(($D279-1)*100,0),IF($D279&gt;1,ROUND(-100/($D279-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="280" ht="15" customHeight="1" s="23">
       <c r="A280" s="11" t="n"/>
@@ -6550,6 +7677,10 @@
         <v/>
       </c>
       <c r="J280" s="12" t="n"/>
+      <c r="K280" s="26">
+        <f>IF(ISNUMBER($D280),IF($D280&gt;=2,ROUND(($D280-1)*100,0),IF($D280&gt;1,ROUND(-100/($D280-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="281" ht="15" customHeight="1" s="23">
       <c r="A281" s="11" t="n"/>
@@ -6571,6 +7702,10 @@
         <v/>
       </c>
       <c r="J281" s="12" t="n"/>
+      <c r="K281" s="26">
+        <f>IF(ISNUMBER($D281),IF($D281&gt;=2,ROUND(($D281-1)*100,0),IF($D281&gt;1,ROUND(-100/($D281-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="282" ht="15" customHeight="1" s="23">
       <c r="A282" s="11" t="n"/>
@@ -6592,6 +7727,10 @@
         <v/>
       </c>
       <c r="J282" s="12" t="n"/>
+      <c r="K282" s="26">
+        <f>IF(ISNUMBER($D282),IF($D282&gt;=2,ROUND(($D282-1)*100,0),IF($D282&gt;1,ROUND(-100/($D282-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="283" ht="15" customHeight="1" s="23">
       <c r="A283" s="11" t="n"/>
@@ -6613,6 +7752,10 @@
         <v/>
       </c>
       <c r="J283" s="12" t="n"/>
+      <c r="K283" s="26">
+        <f>IF(ISNUMBER($D283),IF($D283&gt;=2,ROUND(($D283-1)*100,0),IF($D283&gt;1,ROUND(-100/($D283-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="284" ht="15" customHeight="1" s="23">
       <c r="A284" s="11" t="n"/>
@@ -6634,6 +7777,10 @@
         <v/>
       </c>
       <c r="J284" s="12" t="n"/>
+      <c r="K284" s="26">
+        <f>IF(ISNUMBER($D284),IF($D284&gt;=2,ROUND(($D284-1)*100,0),IF($D284&gt;1,ROUND(-100/($D284-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="285" ht="15" customHeight="1" s="23">
       <c r="A285" s="11" t="n"/>
@@ -6655,6 +7802,10 @@
         <v/>
       </c>
       <c r="J285" s="12" t="n"/>
+      <c r="K285" s="26">
+        <f>IF(ISNUMBER($D285),IF($D285&gt;=2,ROUND(($D285-1)*100,0),IF($D285&gt;1,ROUND(-100/($D285-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="286" ht="15" customHeight="1" s="23">
       <c r="A286" s="11" t="n"/>
@@ -6676,6 +7827,10 @@
         <v/>
       </c>
       <c r="J286" s="12" t="n"/>
+      <c r="K286" s="26">
+        <f>IF(ISNUMBER($D286),IF($D286&gt;=2,ROUND(($D286-1)*100,0),IF($D286&gt;1,ROUND(-100/($D286-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="287" ht="15" customHeight="1" s="23">
       <c r="A287" s="11" t="n"/>
@@ -6697,6 +7852,10 @@
         <v/>
       </c>
       <c r="J287" s="12" t="n"/>
+      <c r="K287" s="26">
+        <f>IF(ISNUMBER($D287),IF($D287&gt;=2,ROUND(($D287-1)*100,0),IF($D287&gt;1,ROUND(-100/($D287-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="288" ht="15" customHeight="1" s="23">
       <c r="A288" s="11" t="n"/>
@@ -6718,6 +7877,10 @@
         <v/>
       </c>
       <c r="J288" s="12" t="n"/>
+      <c r="K288" s="26">
+        <f>IF(ISNUMBER($D288),IF($D288&gt;=2,ROUND(($D288-1)*100,0),IF($D288&gt;1,ROUND(-100/($D288-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="289" ht="15" customHeight="1" s="23">
       <c r="A289" s="11" t="n"/>
@@ -6739,6 +7902,10 @@
         <v/>
       </c>
       <c r="J289" s="12" t="n"/>
+      <c r="K289" s="26">
+        <f>IF(ISNUMBER($D289),IF($D289&gt;=2,ROUND(($D289-1)*100,0),IF($D289&gt;1,ROUND(-100/($D289-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="290" ht="15" customHeight="1" s="23">
       <c r="A290" s="11" t="n"/>
@@ -6760,6 +7927,10 @@
         <v/>
       </c>
       <c r="J290" s="12" t="n"/>
+      <c r="K290" s="26">
+        <f>IF(ISNUMBER($D290),IF($D290&gt;=2,ROUND(($D290-1)*100,0),IF($D290&gt;1,ROUND(-100/($D290-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="291" ht="15" customHeight="1" s="23">
       <c r="A291" s="11" t="n"/>
@@ -6781,6 +7952,10 @@
         <v/>
       </c>
       <c r="J291" s="12" t="n"/>
+      <c r="K291" s="26">
+        <f>IF(ISNUMBER($D291),IF($D291&gt;=2,ROUND(($D291-1)*100,0),IF($D291&gt;1,ROUND(-100/($D291-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="292" ht="15" customHeight="1" s="23">
       <c r="A292" s="11" t="n"/>
@@ -6802,6 +7977,10 @@
         <v/>
       </c>
       <c r="J292" s="12" t="n"/>
+      <c r="K292" s="26">
+        <f>IF(ISNUMBER($D292),IF($D292&gt;=2,ROUND(($D292-1)*100,0),IF($D292&gt;1,ROUND(-100/($D292-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="293" ht="15" customHeight="1" s="23">
       <c r="A293" s="11" t="n"/>
@@ -6823,6 +8002,10 @@
         <v/>
       </c>
       <c r="J293" s="12" t="n"/>
+      <c r="K293" s="26">
+        <f>IF(ISNUMBER($D293),IF($D293&gt;=2,ROUND(($D293-1)*100,0),IF($D293&gt;1,ROUND(-100/($D293-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="294" ht="15" customHeight="1" s="23">
       <c r="A294" s="11" t="n"/>
@@ -6844,6 +8027,10 @@
         <v/>
       </c>
       <c r="J294" s="12" t="n"/>
+      <c r="K294" s="26">
+        <f>IF(ISNUMBER($D294),IF($D294&gt;=2,ROUND(($D294-1)*100,0),IF($D294&gt;1,ROUND(-100/($D294-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="295" ht="15" customHeight="1" s="23">
       <c r="A295" s="11" t="n"/>
@@ -6865,6 +8052,10 @@
         <v/>
       </c>
       <c r="J295" s="12" t="n"/>
+      <c r="K295" s="26">
+        <f>IF(ISNUMBER($D295),IF($D295&gt;=2,ROUND(($D295-1)*100,0),IF($D295&gt;1,ROUND(-100/($D295-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="296" ht="15" customHeight="1" s="23">
       <c r="A296" s="11" t="n"/>
@@ -6886,6 +8077,10 @@
         <v/>
       </c>
       <c r="J296" s="12" t="n"/>
+      <c r="K296" s="26">
+        <f>IF(ISNUMBER($D296),IF($D296&gt;=2,ROUND(($D296-1)*100,0),IF($D296&gt;1,ROUND(-100/($D296-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="297" ht="15" customHeight="1" s="23">
       <c r="A297" s="11" t="n"/>
@@ -6907,6 +8102,10 @@
         <v/>
       </c>
       <c r="J297" s="12" t="n"/>
+      <c r="K297" s="26">
+        <f>IF(ISNUMBER($D297),IF($D297&gt;=2,ROUND(($D297-1)*100,0),IF($D297&gt;1,ROUND(-100/($D297-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -6917,6 +8116,7 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Update/model sprint 2026 06 18 (#9)
* Fix World Cup odds sport selection

* Update DC model parameters

* cfb: update EPA/predictor, validation baseline, blend weights, and tests

* golf: update model/validation, calibration, US Open report and three-ball pricing

* club_soccer: update model, validation, ensemble weights and baseline data

* app: update server, provenance, and web UI

* data: refresh odds/ledger/bankroll/ratings and calibration datasets

* sim/backtest: add v5, v6, wc_v4 engines with World Cup backtests and tests

* root: update edge engine, world cup/tournament odds, betting tracker and sprint notes
</commit_message>
<xml_diff>
--- a/Betting Tracker Example.xlsx
+++ b/Betting Tracker Example.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="680" windowWidth="34200" windowHeight="21460" tabRatio="500" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="My Bets" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Ledger" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="My Bets" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Project Ledger" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterateDelta="0.0001"/>
@@ -17,13 +17,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="\£#,##0.00;&quot;(£&quot;#,##0.00\);\-"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="\£#,##0.00;\(\£#,##0.00\);&quot;-&quot;"/>
     <numFmt numFmtId="167" formatCode="\+0.0%;\-0.0%"/>
     <numFmt numFmtId="168" formatCode="£#,##0.00;(£#,##0.00);&quot;-&quot;"/>
     <numFmt numFmtId="169" formatCode="+0.0%;-0.0%"/>
+    <numFmt numFmtId="170" formatCode="+0;-0;0"/>
   </numFmts>
   <fonts count="12">
     <font>
@@ -146,7 +147,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -175,6 +176,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="169" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -249,6 +251,21 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Tracker</author>
+  </authors>
+  <commentList>
+    <comment ref="K3" authorId="0" shapeId="0">
+      <text>
+        <t>American (US) odds, auto-converted from the decimal Odds column (D). Decimal ≥ 2.00 → +(d-1)×100; 1.00–2.00 → -100/(d-1). Blank if no odds entered.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -646,7 +663,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J297"/>
+  <dimension ref="A1:K297"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" style="23" min="1" max="1"/>
@@ -658,6 +675,7 @@
     <col width="11" customWidth="1" style="23" min="7" max="8"/>
     <col width="12" customWidth="1" style="23" min="9" max="9"/>
     <col width="30" customWidth="1" style="23" min="10" max="10"/>
+    <col width="8" customWidth="1" style="23" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="17.25" customHeight="1" s="23">
@@ -731,6 +749,11 @@
       <c r="J3" s="10" t="inlineStr">
         <is>
           <t>Notes</t>
+        </is>
+      </c>
+      <c r="K3" s="10" t="inlineStr">
+        <is>
+          <t>US Odds</t>
         </is>
       </c>
     </row>
@@ -754,6 +777,10 @@
         <v/>
       </c>
       <c r="J4" s="12" t="n"/>
+      <c r="K4" s="26">
+        <f>IF(ISNUMBER($D4),IF($D4&gt;=2,ROUND(($D4-1)*100,0),IF($D4&gt;1,ROUND(-100/($D4-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="23">
       <c r="A5" s="11" t="n"/>
@@ -775,6 +802,10 @@
         <v/>
       </c>
       <c r="J5" s="12" t="n"/>
+      <c r="K5" s="26">
+        <f>IF(ISNUMBER($D5),IF($D5&gt;=2,ROUND(($D5-1)*100,0),IF($D5&gt;1,ROUND(-100/($D5-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="23">
       <c r="A6" s="11" t="n"/>
@@ -796,6 +827,10 @@
         <v/>
       </c>
       <c r="J6" s="12" t="n"/>
+      <c r="K6" s="26">
+        <f>IF(ISNUMBER($D6),IF($D6&gt;=2,ROUND(($D6-1)*100,0),IF($D6&gt;1,ROUND(-100/($D6-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="23">
       <c r="A7" s="11" t="n"/>
@@ -817,6 +852,10 @@
         <v/>
       </c>
       <c r="J7" s="12" t="n"/>
+      <c r="K7" s="26">
+        <f>IF(ISNUMBER($D7),IF($D7&gt;=2,ROUND(($D7-1)*100,0),IF($D7&gt;1,ROUND(-100/($D7-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="23">
       <c r="A8" s="11" t="n"/>
@@ -838,6 +877,10 @@
         <v/>
       </c>
       <c r="J8" s="12" t="n"/>
+      <c r="K8" s="26">
+        <f>IF(ISNUMBER($D8),IF($D8&gt;=2,ROUND(($D8-1)*100,0),IF($D8&gt;1,ROUND(-100/($D8-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="23">
       <c r="A9" s="11" t="n"/>
@@ -859,6 +902,10 @@
         <v/>
       </c>
       <c r="J9" s="12" t="n"/>
+      <c r="K9" s="26">
+        <f>IF(ISNUMBER($D9),IF($D9&gt;=2,ROUND(($D9-1)*100,0),IF($D9&gt;1,ROUND(-100/($D9-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="23">
       <c r="A10" s="11" t="n"/>
@@ -880,6 +927,10 @@
         <v/>
       </c>
       <c r="J10" s="12" t="n"/>
+      <c r="K10" s="26">
+        <f>IF(ISNUMBER($D10),IF($D10&gt;=2,ROUND(($D10-1)*100,0),IF($D10&gt;1,ROUND(-100/($D10-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="23">
       <c r="A11" s="11" t="n"/>
@@ -901,6 +952,10 @@
         <v/>
       </c>
       <c r="J11" s="12" t="n"/>
+      <c r="K11" s="26">
+        <f>IF(ISNUMBER($D11),IF($D11&gt;=2,ROUND(($D11-1)*100,0),IF($D11&gt;1,ROUND(-100/($D11-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="23">
       <c r="A12" s="11" t="n"/>
@@ -922,6 +977,10 @@
         <v/>
       </c>
       <c r="J12" s="12" t="n"/>
+      <c r="K12" s="26">
+        <f>IF(ISNUMBER($D12),IF($D12&gt;=2,ROUND(($D12-1)*100,0),IF($D12&gt;1,ROUND(-100/($D12-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="23">
       <c r="A13" s="11" t="n"/>
@@ -943,6 +1002,10 @@
         <v/>
       </c>
       <c r="J13" s="12" t="n"/>
+      <c r="K13" s="26">
+        <f>IF(ISNUMBER($D13),IF($D13&gt;=2,ROUND(($D13-1)*100,0),IF($D13&gt;1,ROUND(-100/($D13-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="23">
       <c r="A14" s="11" t="n"/>
@@ -964,6 +1027,10 @@
         <v/>
       </c>
       <c r="J14" s="12" t="n"/>
+      <c r="K14" s="26">
+        <f>IF(ISNUMBER($D14),IF($D14&gt;=2,ROUND(($D14-1)*100,0),IF($D14&gt;1,ROUND(-100/($D14-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="23">
       <c r="A15" s="11" t="n"/>
@@ -985,6 +1052,10 @@
         <v/>
       </c>
       <c r="J15" s="12" t="n"/>
+      <c r="K15" s="26">
+        <f>IF(ISNUMBER($D15),IF($D15&gt;=2,ROUND(($D15-1)*100,0),IF($D15&gt;1,ROUND(-100/($D15-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="23">
       <c r="A16" s="11" t="n"/>
@@ -1006,6 +1077,10 @@
         <v/>
       </c>
       <c r="J16" s="12" t="n"/>
+      <c r="K16" s="26">
+        <f>IF(ISNUMBER($D16),IF($D16&gt;=2,ROUND(($D16-1)*100,0),IF($D16&gt;1,ROUND(-100/($D16-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="23">
       <c r="A17" s="11" t="n"/>
@@ -1027,6 +1102,10 @@
         <v/>
       </c>
       <c r="J17" s="12" t="n"/>
+      <c r="K17" s="26">
+        <f>IF(ISNUMBER($D17),IF($D17&gt;=2,ROUND(($D17-1)*100,0),IF($D17&gt;1,ROUND(-100/($D17-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="23">
       <c r="A18" s="11" t="n"/>
@@ -1048,6 +1127,10 @@
         <v/>
       </c>
       <c r="J18" s="12" t="n"/>
+      <c r="K18" s="26">
+        <f>IF(ISNUMBER($D18),IF($D18&gt;=2,ROUND(($D18-1)*100,0),IF($D18&gt;1,ROUND(-100/($D18-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="23">
       <c r="A19" s="11" t="n"/>
@@ -1069,6 +1152,10 @@
         <v/>
       </c>
       <c r="J19" s="12" t="n"/>
+      <c r="K19" s="26">
+        <f>IF(ISNUMBER($D19),IF($D19&gt;=2,ROUND(($D19-1)*100,0),IF($D19&gt;1,ROUND(-100/($D19-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="23">
       <c r="A20" s="11" t="n"/>
@@ -1090,6 +1177,10 @@
         <v/>
       </c>
       <c r="J20" s="12" t="n"/>
+      <c r="K20" s="26">
+        <f>IF(ISNUMBER($D20),IF($D20&gt;=2,ROUND(($D20-1)*100,0),IF($D20&gt;1,ROUND(-100/($D20-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="23">
       <c r="A21" s="11" t="n"/>
@@ -1111,6 +1202,10 @@
         <v/>
       </c>
       <c r="J21" s="12" t="n"/>
+      <c r="K21" s="26">
+        <f>IF(ISNUMBER($D21),IF($D21&gt;=2,ROUND(($D21-1)*100,0),IF($D21&gt;1,ROUND(-100/($D21-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="23">
       <c r="A22" s="11" t="n"/>
@@ -1132,6 +1227,10 @@
         <v/>
       </c>
       <c r="J22" s="12" t="n"/>
+      <c r="K22" s="26">
+        <f>IF(ISNUMBER($D22),IF($D22&gt;=2,ROUND(($D22-1)*100,0),IF($D22&gt;1,ROUND(-100/($D22-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="23">
       <c r="A23" s="11" t="n"/>
@@ -1153,6 +1252,10 @@
         <v/>
       </c>
       <c r="J23" s="12" t="n"/>
+      <c r="K23" s="26">
+        <f>IF(ISNUMBER($D23),IF($D23&gt;=2,ROUND(($D23-1)*100,0),IF($D23&gt;1,ROUND(-100/($D23-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="23">
       <c r="A24" s="11" t="n"/>
@@ -1174,6 +1277,10 @@
         <v/>
       </c>
       <c r="J24" s="12" t="n"/>
+      <c r="K24" s="26">
+        <f>IF(ISNUMBER($D24),IF($D24&gt;=2,ROUND(($D24-1)*100,0),IF($D24&gt;1,ROUND(-100/($D24-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="23">
       <c r="A25" s="11" t="n"/>
@@ -1195,6 +1302,10 @@
         <v/>
       </c>
       <c r="J25" s="12" t="n"/>
+      <c r="K25" s="26">
+        <f>IF(ISNUMBER($D25),IF($D25&gt;=2,ROUND(($D25-1)*100,0),IF($D25&gt;1,ROUND(-100/($D25-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="23">
       <c r="A26" s="11" t="n"/>
@@ -1216,6 +1327,10 @@
         <v/>
       </c>
       <c r="J26" s="12" t="n"/>
+      <c r="K26" s="26">
+        <f>IF(ISNUMBER($D26),IF($D26&gt;=2,ROUND(($D26-1)*100,0),IF($D26&gt;1,ROUND(-100/($D26-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="23">
       <c r="A27" s="11" t="n"/>
@@ -1237,6 +1352,10 @@
         <v/>
       </c>
       <c r="J27" s="12" t="n"/>
+      <c r="K27" s="26">
+        <f>IF(ISNUMBER($D27),IF($D27&gt;=2,ROUND(($D27-1)*100,0),IF($D27&gt;1,ROUND(-100/($D27-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="23">
       <c r="A28" s="11" t="n"/>
@@ -1258,6 +1377,10 @@
         <v/>
       </c>
       <c r="J28" s="12" t="n"/>
+      <c r="K28" s="26">
+        <f>IF(ISNUMBER($D28),IF($D28&gt;=2,ROUND(($D28-1)*100,0),IF($D28&gt;1,ROUND(-100/($D28-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="23">
       <c r="A29" s="11" t="n"/>
@@ -1279,6 +1402,10 @@
         <v/>
       </c>
       <c r="J29" s="12" t="n"/>
+      <c r="K29" s="26">
+        <f>IF(ISNUMBER($D29),IF($D29&gt;=2,ROUND(($D29-1)*100,0),IF($D29&gt;1,ROUND(-100/($D29-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="23">
       <c r="A30" s="11" t="n"/>
@@ -1300,6 +1427,10 @@
         <v/>
       </c>
       <c r="J30" s="12" t="n"/>
+      <c r="K30" s="26">
+        <f>IF(ISNUMBER($D30),IF($D30&gt;=2,ROUND(($D30-1)*100,0),IF($D30&gt;1,ROUND(-100/($D30-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="23">
       <c r="A31" s="11" t="n"/>
@@ -1321,6 +1452,10 @@
         <v/>
       </c>
       <c r="J31" s="12" t="n"/>
+      <c r="K31" s="26">
+        <f>IF(ISNUMBER($D31),IF($D31&gt;=2,ROUND(($D31-1)*100,0),IF($D31&gt;1,ROUND(-100/($D31-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="23">
       <c r="A32" s="11" t="n"/>
@@ -1342,6 +1477,10 @@
         <v/>
       </c>
       <c r="J32" s="12" t="n"/>
+      <c r="K32" s="26">
+        <f>IF(ISNUMBER($D32),IF($D32&gt;=2,ROUND(($D32-1)*100,0),IF($D32&gt;1,ROUND(-100/($D32-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="23">
       <c r="A33" s="11" t="n"/>
@@ -1363,6 +1502,10 @@
         <v/>
       </c>
       <c r="J33" s="12" t="n"/>
+      <c r="K33" s="26">
+        <f>IF(ISNUMBER($D33),IF($D33&gt;=2,ROUND(($D33-1)*100,0),IF($D33&gt;1,ROUND(-100/($D33-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="23">
       <c r="A34" s="11" t="n"/>
@@ -1384,6 +1527,10 @@
         <v/>
       </c>
       <c r="J34" s="12" t="n"/>
+      <c r="K34" s="26">
+        <f>IF(ISNUMBER($D34),IF($D34&gt;=2,ROUND(($D34-1)*100,0),IF($D34&gt;1,ROUND(-100/($D34-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="23">
       <c r="A35" s="11" t="n"/>
@@ -1405,6 +1552,10 @@
         <v/>
       </c>
       <c r="J35" s="12" t="n"/>
+      <c r="K35" s="26">
+        <f>IF(ISNUMBER($D35),IF($D35&gt;=2,ROUND(($D35-1)*100,0),IF($D35&gt;1,ROUND(-100/($D35-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="23">
       <c r="A36" s="11" t="n"/>
@@ -1426,6 +1577,10 @@
         <v/>
       </c>
       <c r="J36" s="12" t="n"/>
+      <c r="K36" s="26">
+        <f>IF(ISNUMBER($D36),IF($D36&gt;=2,ROUND(($D36-1)*100,0),IF($D36&gt;1,ROUND(-100/($D36-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="23">
       <c r="A37" s="11" t="n"/>
@@ -1447,6 +1602,10 @@
         <v/>
       </c>
       <c r="J37" s="12" t="n"/>
+      <c r="K37" s="26">
+        <f>IF(ISNUMBER($D37),IF($D37&gt;=2,ROUND(($D37-1)*100,0),IF($D37&gt;1,ROUND(-100/($D37-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="38" ht="15" customHeight="1" s="23">
       <c r="A38" s="11" t="n"/>
@@ -1468,6 +1627,10 @@
         <v/>
       </c>
       <c r="J38" s="12" t="n"/>
+      <c r="K38" s="26">
+        <f>IF(ISNUMBER($D38),IF($D38&gt;=2,ROUND(($D38-1)*100,0),IF($D38&gt;1,ROUND(-100/($D38-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="23">
       <c r="A39" s="11" t="n"/>
@@ -1489,6 +1652,10 @@
         <v/>
       </c>
       <c r="J39" s="12" t="n"/>
+      <c r="K39" s="26">
+        <f>IF(ISNUMBER($D39),IF($D39&gt;=2,ROUND(($D39-1)*100,0),IF($D39&gt;1,ROUND(-100/($D39-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="23">
       <c r="A40" s="11" t="n"/>
@@ -1510,6 +1677,10 @@
         <v/>
       </c>
       <c r="J40" s="12" t="n"/>
+      <c r="K40" s="26">
+        <f>IF(ISNUMBER($D40),IF($D40&gt;=2,ROUND(($D40-1)*100,0),IF($D40&gt;1,ROUND(-100/($D40-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="23">
       <c r="A41" s="11" t="n"/>
@@ -1531,6 +1702,10 @@
         <v/>
       </c>
       <c r="J41" s="12" t="n"/>
+      <c r="K41" s="26">
+        <f>IF(ISNUMBER($D41),IF($D41&gt;=2,ROUND(($D41-1)*100,0),IF($D41&gt;1,ROUND(-100/($D41-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="23">
       <c r="A42" s="11" t="n"/>
@@ -1552,6 +1727,10 @@
         <v/>
       </c>
       <c r="J42" s="12" t="n"/>
+      <c r="K42" s="26">
+        <f>IF(ISNUMBER($D42),IF($D42&gt;=2,ROUND(($D42-1)*100,0),IF($D42&gt;1,ROUND(-100/($D42-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="23">
       <c r="A43" s="11" t="n"/>
@@ -1573,6 +1752,10 @@
         <v/>
       </c>
       <c r="J43" s="12" t="n"/>
+      <c r="K43" s="26">
+        <f>IF(ISNUMBER($D43),IF($D43&gt;=2,ROUND(($D43-1)*100,0),IF($D43&gt;1,ROUND(-100/($D43-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="23">
       <c r="A44" s="11" t="n"/>
@@ -1594,6 +1777,10 @@
         <v/>
       </c>
       <c r="J44" s="12" t="n"/>
+      <c r="K44" s="26">
+        <f>IF(ISNUMBER($D44),IF($D44&gt;=2,ROUND(($D44-1)*100,0),IF($D44&gt;1,ROUND(-100/($D44-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="23">
       <c r="A45" s="11" t="n"/>
@@ -1615,6 +1802,10 @@
         <v/>
       </c>
       <c r="J45" s="12" t="n"/>
+      <c r="K45" s="26">
+        <f>IF(ISNUMBER($D45),IF($D45&gt;=2,ROUND(($D45-1)*100,0),IF($D45&gt;1,ROUND(-100/($D45-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="23">
       <c r="A46" s="11" t="n"/>
@@ -1636,6 +1827,10 @@
         <v/>
       </c>
       <c r="J46" s="12" t="n"/>
+      <c r="K46" s="26">
+        <f>IF(ISNUMBER($D46),IF($D46&gt;=2,ROUND(($D46-1)*100,0),IF($D46&gt;1,ROUND(-100/($D46-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="23">
       <c r="A47" s="11" t="n"/>
@@ -1657,6 +1852,10 @@
         <v/>
       </c>
       <c r="J47" s="12" t="n"/>
+      <c r="K47" s="26">
+        <f>IF(ISNUMBER($D47),IF($D47&gt;=2,ROUND(($D47-1)*100,0),IF($D47&gt;1,ROUND(-100/($D47-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="48" ht="15" customHeight="1" s="23">
       <c r="A48" s="11" t="n"/>
@@ -1678,6 +1877,10 @@
         <v/>
       </c>
       <c r="J48" s="12" t="n"/>
+      <c r="K48" s="26">
+        <f>IF(ISNUMBER($D48),IF($D48&gt;=2,ROUND(($D48-1)*100,0),IF($D48&gt;1,ROUND(-100/($D48-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="49" ht="15" customHeight="1" s="23">
       <c r="A49" s="11" t="n"/>
@@ -1699,6 +1902,10 @@
         <v/>
       </c>
       <c r="J49" s="12" t="n"/>
+      <c r="K49" s="26">
+        <f>IF(ISNUMBER($D49),IF($D49&gt;=2,ROUND(($D49-1)*100,0),IF($D49&gt;1,ROUND(-100/($D49-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="23">
       <c r="A50" s="11" t="n"/>
@@ -1720,6 +1927,10 @@
         <v/>
       </c>
       <c r="J50" s="12" t="n"/>
+      <c r="K50" s="26">
+        <f>IF(ISNUMBER($D50),IF($D50&gt;=2,ROUND(($D50-1)*100,0),IF($D50&gt;1,ROUND(-100/($D50-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="23">
       <c r="A51" s="11" t="n"/>
@@ -1741,6 +1952,10 @@
         <v/>
       </c>
       <c r="J51" s="12" t="n"/>
+      <c r="K51" s="26">
+        <f>IF(ISNUMBER($D51),IF($D51&gt;=2,ROUND(($D51-1)*100,0),IF($D51&gt;1,ROUND(-100/($D51-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="23">
       <c r="A52" s="11" t="n"/>
@@ -1762,6 +1977,10 @@
         <v/>
       </c>
       <c r="J52" s="12" t="n"/>
+      <c r="K52" s="26">
+        <f>IF(ISNUMBER($D52),IF($D52&gt;=2,ROUND(($D52-1)*100,0),IF($D52&gt;1,ROUND(-100/($D52-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="23">
       <c r="A53" s="11" t="n"/>
@@ -1783,6 +2002,10 @@
         <v/>
       </c>
       <c r="J53" s="12" t="n"/>
+      <c r="K53" s="26">
+        <f>IF(ISNUMBER($D53),IF($D53&gt;=2,ROUND(($D53-1)*100,0),IF($D53&gt;1,ROUND(-100/($D53-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="23">
       <c r="A54" s="11" t="n"/>
@@ -1804,6 +2027,10 @@
         <v/>
       </c>
       <c r="J54" s="12" t="n"/>
+      <c r="K54" s="26">
+        <f>IF(ISNUMBER($D54),IF($D54&gt;=2,ROUND(($D54-1)*100,0),IF($D54&gt;1,ROUND(-100/($D54-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="23">
       <c r="A55" s="11" t="n"/>
@@ -1825,6 +2052,10 @@
         <v/>
       </c>
       <c r="J55" s="12" t="n"/>
+      <c r="K55" s="26">
+        <f>IF(ISNUMBER($D55),IF($D55&gt;=2,ROUND(($D55-1)*100,0),IF($D55&gt;1,ROUND(-100/($D55-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="23">
       <c r="A56" s="11" t="n"/>
@@ -1846,6 +2077,10 @@
         <v/>
       </c>
       <c r="J56" s="12" t="n"/>
+      <c r="K56" s="26">
+        <f>IF(ISNUMBER($D56),IF($D56&gt;=2,ROUND(($D56-1)*100,0),IF($D56&gt;1,ROUND(-100/($D56-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="23">
       <c r="A57" s="11" t="n"/>
@@ -1867,6 +2102,10 @@
         <v/>
       </c>
       <c r="J57" s="12" t="n"/>
+      <c r="K57" s="26">
+        <f>IF(ISNUMBER($D57),IF($D57&gt;=2,ROUND(($D57-1)*100,0),IF($D57&gt;1,ROUND(-100/($D57-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="23">
       <c r="A58" s="11" t="n"/>
@@ -1888,6 +2127,10 @@
         <v/>
       </c>
       <c r="J58" s="12" t="n"/>
+      <c r="K58" s="26">
+        <f>IF(ISNUMBER($D58),IF($D58&gt;=2,ROUND(($D58-1)*100,0),IF($D58&gt;1,ROUND(-100/($D58-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="23">
       <c r="A59" s="11" t="n"/>
@@ -1909,6 +2152,10 @@
         <v/>
       </c>
       <c r="J59" s="12" t="n"/>
+      <c r="K59" s="26">
+        <f>IF(ISNUMBER($D59),IF($D59&gt;=2,ROUND(($D59-1)*100,0),IF($D59&gt;1,ROUND(-100/($D59-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="23">
       <c r="A60" s="11" t="n"/>
@@ -1930,6 +2177,10 @@
         <v/>
       </c>
       <c r="J60" s="12" t="n"/>
+      <c r="K60" s="26">
+        <f>IF(ISNUMBER($D60),IF($D60&gt;=2,ROUND(($D60-1)*100,0),IF($D60&gt;1,ROUND(-100/($D60-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="23">
       <c r="A61" s="11" t="n"/>
@@ -1951,6 +2202,10 @@
         <v/>
       </c>
       <c r="J61" s="12" t="n"/>
+      <c r="K61" s="26">
+        <f>IF(ISNUMBER($D61),IF($D61&gt;=2,ROUND(($D61-1)*100,0),IF($D61&gt;1,ROUND(-100/($D61-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="23">
       <c r="A62" s="11" t="n"/>
@@ -1972,6 +2227,10 @@
         <v/>
       </c>
       <c r="J62" s="12" t="n"/>
+      <c r="K62" s="26">
+        <f>IF(ISNUMBER($D62),IF($D62&gt;=2,ROUND(($D62-1)*100,0),IF($D62&gt;1,ROUND(-100/($D62-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="23">
       <c r="A63" s="11" t="n"/>
@@ -1993,6 +2252,10 @@
         <v/>
       </c>
       <c r="J63" s="12" t="n"/>
+      <c r="K63" s="26">
+        <f>IF(ISNUMBER($D63),IF($D63&gt;=2,ROUND(($D63-1)*100,0),IF($D63&gt;1,ROUND(-100/($D63-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="23">
       <c r="A64" s="11" t="n"/>
@@ -2014,6 +2277,10 @@
         <v/>
       </c>
       <c r="J64" s="12" t="n"/>
+      <c r="K64" s="26">
+        <f>IF(ISNUMBER($D64),IF($D64&gt;=2,ROUND(($D64-1)*100,0),IF($D64&gt;1,ROUND(-100/($D64-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="23">
       <c r="A65" s="11" t="n"/>
@@ -2035,6 +2302,10 @@
         <v/>
       </c>
       <c r="J65" s="12" t="n"/>
+      <c r="K65" s="26">
+        <f>IF(ISNUMBER($D65),IF($D65&gt;=2,ROUND(($D65-1)*100,0),IF($D65&gt;1,ROUND(-100/($D65-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="23">
       <c r="A66" s="11" t="n"/>
@@ -2056,6 +2327,10 @@
         <v/>
       </c>
       <c r="J66" s="12" t="n"/>
+      <c r="K66" s="26">
+        <f>IF(ISNUMBER($D66),IF($D66&gt;=2,ROUND(($D66-1)*100,0),IF($D66&gt;1,ROUND(-100/($D66-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="23">
       <c r="A67" s="11" t="n"/>
@@ -2077,6 +2352,10 @@
         <v/>
       </c>
       <c r="J67" s="12" t="n"/>
+      <c r="K67" s="26">
+        <f>IF(ISNUMBER($D67),IF($D67&gt;=2,ROUND(($D67-1)*100,0),IF($D67&gt;1,ROUND(-100/($D67-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="23">
       <c r="A68" s="11" t="n"/>
@@ -2098,6 +2377,10 @@
         <v/>
       </c>
       <c r="J68" s="12" t="n"/>
+      <c r="K68" s="26">
+        <f>IF(ISNUMBER($D68),IF($D68&gt;=2,ROUND(($D68-1)*100,0),IF($D68&gt;1,ROUND(-100/($D68-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="23">
       <c r="A69" s="11" t="n"/>
@@ -2119,6 +2402,10 @@
         <v/>
       </c>
       <c r="J69" s="12" t="n"/>
+      <c r="K69" s="26">
+        <f>IF(ISNUMBER($D69),IF($D69&gt;=2,ROUND(($D69-1)*100,0),IF($D69&gt;1,ROUND(-100/($D69-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="23">
       <c r="A70" s="11" t="n"/>
@@ -2140,6 +2427,10 @@
         <v/>
       </c>
       <c r="J70" s="12" t="n"/>
+      <c r="K70" s="26">
+        <f>IF(ISNUMBER($D70),IF($D70&gt;=2,ROUND(($D70-1)*100,0),IF($D70&gt;1,ROUND(-100/($D70-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="23">
       <c r="A71" s="11" t="n"/>
@@ -2161,6 +2452,10 @@
         <v/>
       </c>
       <c r="J71" s="12" t="n"/>
+      <c r="K71" s="26">
+        <f>IF(ISNUMBER($D71),IF($D71&gt;=2,ROUND(($D71-1)*100,0),IF($D71&gt;1,ROUND(-100/($D71-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="23">
       <c r="A72" s="11" t="n"/>
@@ -2182,6 +2477,10 @@
         <v/>
       </c>
       <c r="J72" s="12" t="n"/>
+      <c r="K72" s="26">
+        <f>IF(ISNUMBER($D72),IF($D72&gt;=2,ROUND(($D72-1)*100,0),IF($D72&gt;1,ROUND(-100/($D72-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="23">
       <c r="A73" s="11" t="n"/>
@@ -2203,6 +2502,10 @@
         <v/>
       </c>
       <c r="J73" s="12" t="n"/>
+      <c r="K73" s="26">
+        <f>IF(ISNUMBER($D73),IF($D73&gt;=2,ROUND(($D73-1)*100,0),IF($D73&gt;1,ROUND(-100/($D73-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="23">
       <c r="A74" s="11" t="n"/>
@@ -2224,6 +2527,10 @@
         <v/>
       </c>
       <c r="J74" s="12" t="n"/>
+      <c r="K74" s="26">
+        <f>IF(ISNUMBER($D74),IF($D74&gt;=2,ROUND(($D74-1)*100,0),IF($D74&gt;1,ROUND(-100/($D74-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="75" ht="15" customHeight="1" s="23">
       <c r="A75" s="11" t="n"/>
@@ -2245,6 +2552,10 @@
         <v/>
       </c>
       <c r="J75" s="12" t="n"/>
+      <c r="K75" s="26">
+        <f>IF(ISNUMBER($D75),IF($D75&gt;=2,ROUND(($D75-1)*100,0),IF($D75&gt;1,ROUND(-100/($D75-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="23">
       <c r="A76" s="11" t="n"/>
@@ -2266,6 +2577,10 @@
         <v/>
       </c>
       <c r="J76" s="12" t="n"/>
+      <c r="K76" s="26">
+        <f>IF(ISNUMBER($D76),IF($D76&gt;=2,ROUND(($D76-1)*100,0),IF($D76&gt;1,ROUND(-100/($D76-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="23">
       <c r="A77" s="11" t="n"/>
@@ -2287,6 +2602,10 @@
         <v/>
       </c>
       <c r="J77" s="12" t="n"/>
+      <c r="K77" s="26">
+        <f>IF(ISNUMBER($D77),IF($D77&gt;=2,ROUND(($D77-1)*100,0),IF($D77&gt;1,ROUND(-100/($D77-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="78" ht="15" customHeight="1" s="23">
       <c r="A78" s="11" t="n"/>
@@ -2308,6 +2627,10 @@
         <v/>
       </c>
       <c r="J78" s="12" t="n"/>
+      <c r="K78" s="26">
+        <f>IF(ISNUMBER($D78),IF($D78&gt;=2,ROUND(($D78-1)*100,0),IF($D78&gt;1,ROUND(-100/($D78-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="23">
       <c r="A79" s="11" t="n"/>
@@ -2329,6 +2652,10 @@
         <v/>
       </c>
       <c r="J79" s="12" t="n"/>
+      <c r="K79" s="26">
+        <f>IF(ISNUMBER($D79),IF($D79&gt;=2,ROUND(($D79-1)*100,0),IF($D79&gt;1,ROUND(-100/($D79-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="80" ht="15" customHeight="1" s="23">
       <c r="A80" s="11" t="n"/>
@@ -2350,6 +2677,10 @@
         <v/>
       </c>
       <c r="J80" s="12" t="n"/>
+      <c r="K80" s="26">
+        <f>IF(ISNUMBER($D80),IF($D80&gt;=2,ROUND(($D80-1)*100,0),IF($D80&gt;1,ROUND(-100/($D80-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="23">
       <c r="A81" s="11" t="n"/>
@@ -2371,6 +2702,10 @@
         <v/>
       </c>
       <c r="J81" s="12" t="n"/>
+      <c r="K81" s="26">
+        <f>IF(ISNUMBER($D81),IF($D81&gt;=2,ROUND(($D81-1)*100,0),IF($D81&gt;1,ROUND(-100/($D81-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="23">
       <c r="A82" s="11" t="n"/>
@@ -2392,6 +2727,10 @@
         <v/>
       </c>
       <c r="J82" s="12" t="n"/>
+      <c r="K82" s="26">
+        <f>IF(ISNUMBER($D82),IF($D82&gt;=2,ROUND(($D82-1)*100,0),IF($D82&gt;1,ROUND(-100/($D82-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="23">
       <c r="A83" s="11" t="n"/>
@@ -2413,6 +2752,10 @@
         <v/>
       </c>
       <c r="J83" s="12" t="n"/>
+      <c r="K83" s="26">
+        <f>IF(ISNUMBER($D83),IF($D83&gt;=2,ROUND(($D83-1)*100,0),IF($D83&gt;1,ROUND(-100/($D83-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="23">
       <c r="A84" s="11" t="n"/>
@@ -2434,6 +2777,10 @@
         <v/>
       </c>
       <c r="J84" s="12" t="n"/>
+      <c r="K84" s="26">
+        <f>IF(ISNUMBER($D84),IF($D84&gt;=2,ROUND(($D84-1)*100,0),IF($D84&gt;1,ROUND(-100/($D84-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="23">
       <c r="A85" s="11" t="n"/>
@@ -2455,6 +2802,10 @@
         <v/>
       </c>
       <c r="J85" s="12" t="n"/>
+      <c r="K85" s="26">
+        <f>IF(ISNUMBER($D85),IF($D85&gt;=2,ROUND(($D85-1)*100,0),IF($D85&gt;1,ROUND(-100/($D85-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="23">
       <c r="A86" s="11" t="n"/>
@@ -2476,6 +2827,10 @@
         <v/>
       </c>
       <c r="J86" s="12" t="n"/>
+      <c r="K86" s="26">
+        <f>IF(ISNUMBER($D86),IF($D86&gt;=2,ROUND(($D86-1)*100,0),IF($D86&gt;1,ROUND(-100/($D86-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="23">
       <c r="A87" s="11" t="n"/>
@@ -2497,6 +2852,10 @@
         <v/>
       </c>
       <c r="J87" s="12" t="n"/>
+      <c r="K87" s="26">
+        <f>IF(ISNUMBER($D87),IF($D87&gt;=2,ROUND(($D87-1)*100,0),IF($D87&gt;1,ROUND(-100/($D87-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="23">
       <c r="A88" s="11" t="n"/>
@@ -2518,6 +2877,10 @@
         <v/>
       </c>
       <c r="J88" s="12" t="n"/>
+      <c r="K88" s="26">
+        <f>IF(ISNUMBER($D88),IF($D88&gt;=2,ROUND(($D88-1)*100,0),IF($D88&gt;1,ROUND(-100/($D88-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="23">
       <c r="A89" s="11" t="n"/>
@@ -2539,6 +2902,10 @@
         <v/>
       </c>
       <c r="J89" s="12" t="n"/>
+      <c r="K89" s="26">
+        <f>IF(ISNUMBER($D89),IF($D89&gt;=2,ROUND(($D89-1)*100,0),IF($D89&gt;1,ROUND(-100/($D89-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="23">
       <c r="A90" s="11" t="n"/>
@@ -2560,6 +2927,10 @@
         <v/>
       </c>
       <c r="J90" s="12" t="n"/>
+      <c r="K90" s="26">
+        <f>IF(ISNUMBER($D90),IF($D90&gt;=2,ROUND(($D90-1)*100,0),IF($D90&gt;1,ROUND(-100/($D90-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="23">
       <c r="A91" s="11" t="n"/>
@@ -2581,6 +2952,10 @@
         <v/>
       </c>
       <c r="J91" s="12" t="n"/>
+      <c r="K91" s="26">
+        <f>IF(ISNUMBER($D91),IF($D91&gt;=2,ROUND(($D91-1)*100,0),IF($D91&gt;1,ROUND(-100/($D91-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="92" ht="15" customHeight="1" s="23">
       <c r="A92" s="11" t="n"/>
@@ -2602,6 +2977,10 @@
         <v/>
       </c>
       <c r="J92" s="12" t="n"/>
+      <c r="K92" s="26">
+        <f>IF(ISNUMBER($D92),IF($D92&gt;=2,ROUND(($D92-1)*100,0),IF($D92&gt;1,ROUND(-100/($D92-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="23">
       <c r="A93" s="11" t="n"/>
@@ -2623,6 +3002,10 @@
         <v/>
       </c>
       <c r="J93" s="12" t="n"/>
+      <c r="K93" s="26">
+        <f>IF(ISNUMBER($D93),IF($D93&gt;=2,ROUND(($D93-1)*100,0),IF($D93&gt;1,ROUND(-100/($D93-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="23">
       <c r="A94" s="11" t="n"/>
@@ -2644,6 +3027,10 @@
         <v/>
       </c>
       <c r="J94" s="12" t="n"/>
+      <c r="K94" s="26">
+        <f>IF(ISNUMBER($D94),IF($D94&gt;=2,ROUND(($D94-1)*100,0),IF($D94&gt;1,ROUND(-100/($D94-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="23">
       <c r="A95" s="11" t="n"/>
@@ -2665,6 +3052,10 @@
         <v/>
       </c>
       <c r="J95" s="12" t="n"/>
+      <c r="K95" s="26">
+        <f>IF(ISNUMBER($D95),IF($D95&gt;=2,ROUND(($D95-1)*100,0),IF($D95&gt;1,ROUND(-100/($D95-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="23">
       <c r="A96" s="11" t="n"/>
@@ -2686,6 +3077,10 @@
         <v/>
       </c>
       <c r="J96" s="12" t="n"/>
+      <c r="K96" s="26">
+        <f>IF(ISNUMBER($D96),IF($D96&gt;=2,ROUND(($D96-1)*100,0),IF($D96&gt;1,ROUND(-100/($D96-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="23">
       <c r="A97" s="11" t="n"/>
@@ -2707,6 +3102,10 @@
         <v/>
       </c>
       <c r="J97" s="12" t="n"/>
+      <c r="K97" s="26">
+        <f>IF(ISNUMBER($D97),IF($D97&gt;=2,ROUND(($D97-1)*100,0),IF($D97&gt;1,ROUND(-100/($D97-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="23">
       <c r="A98" s="11" t="n"/>
@@ -2728,6 +3127,10 @@
         <v/>
       </c>
       <c r="J98" s="12" t="n"/>
+      <c r="K98" s="26">
+        <f>IF(ISNUMBER($D98),IF($D98&gt;=2,ROUND(($D98-1)*100,0),IF($D98&gt;1,ROUND(-100/($D98-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="23">
       <c r="A99" s="11" t="n"/>
@@ -2749,6 +3152,10 @@
         <v/>
       </c>
       <c r="J99" s="12" t="n"/>
+      <c r="K99" s="26">
+        <f>IF(ISNUMBER($D99),IF($D99&gt;=2,ROUND(($D99-1)*100,0),IF($D99&gt;1,ROUND(-100/($D99-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="23">
       <c r="A100" s="11" t="n"/>
@@ -2770,6 +3177,10 @@
         <v/>
       </c>
       <c r="J100" s="12" t="n"/>
+      <c r="K100" s="26">
+        <f>IF(ISNUMBER($D100),IF($D100&gt;=2,ROUND(($D100-1)*100,0),IF($D100&gt;1,ROUND(-100/($D100-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="23">
       <c r="A101" s="11" t="n"/>
@@ -2791,6 +3202,10 @@
         <v/>
       </c>
       <c r="J101" s="12" t="n"/>
+      <c r="K101" s="26">
+        <f>IF(ISNUMBER($D101),IF($D101&gt;=2,ROUND(($D101-1)*100,0),IF($D101&gt;1,ROUND(-100/($D101-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="23">
       <c r="A102" s="11" t="n"/>
@@ -2812,6 +3227,10 @@
         <v/>
       </c>
       <c r="J102" s="12" t="n"/>
+      <c r="K102" s="26">
+        <f>IF(ISNUMBER($D102),IF($D102&gt;=2,ROUND(($D102-1)*100,0),IF($D102&gt;1,ROUND(-100/($D102-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="23">
       <c r="A103" s="11" t="n"/>
@@ -2833,6 +3252,10 @@
         <v/>
       </c>
       <c r="J103" s="12" t="n"/>
+      <c r="K103" s="26">
+        <f>IF(ISNUMBER($D103),IF($D103&gt;=2,ROUND(($D103-1)*100,0),IF($D103&gt;1,ROUND(-100/($D103-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="104" ht="15" customHeight="1" s="23">
       <c r="A104" s="11" t="n"/>
@@ -2854,6 +3277,10 @@
         <v/>
       </c>
       <c r="J104" s="12" t="n"/>
+      <c r="K104" s="26">
+        <f>IF(ISNUMBER($D104),IF($D104&gt;=2,ROUND(($D104-1)*100,0),IF($D104&gt;1,ROUND(-100/($D104-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="105" ht="15" customHeight="1" s="23">
       <c r="A105" s="11" t="n"/>
@@ -2875,6 +3302,10 @@
         <v/>
       </c>
       <c r="J105" s="12" t="n"/>
+      <c r="K105" s="26">
+        <f>IF(ISNUMBER($D105),IF($D105&gt;=2,ROUND(($D105-1)*100,0),IF($D105&gt;1,ROUND(-100/($D105-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="23">
       <c r="A106" s="11" t="n"/>
@@ -2896,6 +3327,10 @@
         <v/>
       </c>
       <c r="J106" s="12" t="n"/>
+      <c r="K106" s="26">
+        <f>IF(ISNUMBER($D106),IF($D106&gt;=2,ROUND(($D106-1)*100,0),IF($D106&gt;1,ROUND(-100/($D106-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="23">
       <c r="A107" s="11" t="n"/>
@@ -2917,6 +3352,10 @@
         <v/>
       </c>
       <c r="J107" s="12" t="n"/>
+      <c r="K107" s="26">
+        <f>IF(ISNUMBER($D107),IF($D107&gt;=2,ROUND(($D107-1)*100,0),IF($D107&gt;1,ROUND(-100/($D107-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="108" ht="15" customHeight="1" s="23">
       <c r="A108" s="11" t="n"/>
@@ -2938,6 +3377,10 @@
         <v/>
       </c>
       <c r="J108" s="12" t="n"/>
+      <c r="K108" s="26">
+        <f>IF(ISNUMBER($D108),IF($D108&gt;=2,ROUND(($D108-1)*100,0),IF($D108&gt;1,ROUND(-100/($D108-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="109" ht="15" customHeight="1" s="23">
       <c r="A109" s="11" t="n"/>
@@ -2959,6 +3402,10 @@
         <v/>
       </c>
       <c r="J109" s="12" t="n"/>
+      <c r="K109" s="26">
+        <f>IF(ISNUMBER($D109),IF($D109&gt;=2,ROUND(($D109-1)*100,0),IF($D109&gt;1,ROUND(-100/($D109-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="110" ht="15" customHeight="1" s="23">
       <c r="A110" s="11" t="n"/>
@@ -2980,6 +3427,10 @@
         <v/>
       </c>
       <c r="J110" s="12" t="n"/>
+      <c r="K110" s="26">
+        <f>IF(ISNUMBER($D110),IF($D110&gt;=2,ROUND(($D110-1)*100,0),IF($D110&gt;1,ROUND(-100/($D110-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="111" ht="15" customHeight="1" s="23">
       <c r="A111" s="11" t="n"/>
@@ -3001,6 +3452,10 @@
         <v/>
       </c>
       <c r="J111" s="12" t="n"/>
+      <c r="K111" s="26">
+        <f>IF(ISNUMBER($D111),IF($D111&gt;=2,ROUND(($D111-1)*100,0),IF($D111&gt;1,ROUND(-100/($D111-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="112" ht="15" customHeight="1" s="23">
       <c r="A112" s="11" t="n"/>
@@ -3022,6 +3477,10 @@
         <v/>
       </c>
       <c r="J112" s="12" t="n"/>
+      <c r="K112" s="26">
+        <f>IF(ISNUMBER($D112),IF($D112&gt;=2,ROUND(($D112-1)*100,0),IF($D112&gt;1,ROUND(-100/($D112-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="113" ht="15" customHeight="1" s="23">
       <c r="A113" s="11" t="n"/>
@@ -3043,6 +3502,10 @@
         <v/>
       </c>
       <c r="J113" s="12" t="n"/>
+      <c r="K113" s="26">
+        <f>IF(ISNUMBER($D113),IF($D113&gt;=2,ROUND(($D113-1)*100,0),IF($D113&gt;1,ROUND(-100/($D113-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="114" ht="15" customHeight="1" s="23">
       <c r="A114" s="11" t="n"/>
@@ -3064,6 +3527,10 @@
         <v/>
       </c>
       <c r="J114" s="12" t="n"/>
+      <c r="K114" s="26">
+        <f>IF(ISNUMBER($D114),IF($D114&gt;=2,ROUND(($D114-1)*100,0),IF($D114&gt;1,ROUND(-100/($D114-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="115" ht="15" customHeight="1" s="23">
       <c r="A115" s="11" t="n"/>
@@ -3085,6 +3552,10 @@
         <v/>
       </c>
       <c r="J115" s="12" t="n"/>
+      <c r="K115" s="26">
+        <f>IF(ISNUMBER($D115),IF($D115&gt;=2,ROUND(($D115-1)*100,0),IF($D115&gt;1,ROUND(-100/($D115-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="116" ht="15" customHeight="1" s="23">
       <c r="A116" s="11" t="n"/>
@@ -3106,6 +3577,10 @@
         <v/>
       </c>
       <c r="J116" s="12" t="n"/>
+      <c r="K116" s="26">
+        <f>IF(ISNUMBER($D116),IF($D116&gt;=2,ROUND(($D116-1)*100,0),IF($D116&gt;1,ROUND(-100/($D116-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="117" ht="15" customHeight="1" s="23">
       <c r="A117" s="11" t="n"/>
@@ -3127,6 +3602,10 @@
         <v/>
       </c>
       <c r="J117" s="12" t="n"/>
+      <c r="K117" s="26">
+        <f>IF(ISNUMBER($D117),IF($D117&gt;=2,ROUND(($D117-1)*100,0),IF($D117&gt;1,ROUND(-100/($D117-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="118" ht="15" customHeight="1" s="23">
       <c r="A118" s="11" t="n"/>
@@ -3148,6 +3627,10 @@
         <v/>
       </c>
       <c r="J118" s="12" t="n"/>
+      <c r="K118" s="26">
+        <f>IF(ISNUMBER($D118),IF($D118&gt;=2,ROUND(($D118-1)*100,0),IF($D118&gt;1,ROUND(-100/($D118-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="119" ht="15" customHeight="1" s="23">
       <c r="A119" s="11" t="n"/>
@@ -3169,6 +3652,10 @@
         <v/>
       </c>
       <c r="J119" s="12" t="n"/>
+      <c r="K119" s="26">
+        <f>IF(ISNUMBER($D119),IF($D119&gt;=2,ROUND(($D119-1)*100,0),IF($D119&gt;1,ROUND(-100/($D119-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="120" ht="15" customHeight="1" s="23">
       <c r="A120" s="11" t="n"/>
@@ -3190,6 +3677,10 @@
         <v/>
       </c>
       <c r="J120" s="12" t="n"/>
+      <c r="K120" s="26">
+        <f>IF(ISNUMBER($D120),IF($D120&gt;=2,ROUND(($D120-1)*100,0),IF($D120&gt;1,ROUND(-100/($D120-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="121" ht="15" customHeight="1" s="23">
       <c r="A121" s="11" t="n"/>
@@ -3211,6 +3702,10 @@
         <v/>
       </c>
       <c r="J121" s="12" t="n"/>
+      <c r="K121" s="26">
+        <f>IF(ISNUMBER($D121),IF($D121&gt;=2,ROUND(($D121-1)*100,0),IF($D121&gt;1,ROUND(-100/($D121-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="122" ht="15" customHeight="1" s="23">
       <c r="A122" s="11" t="n"/>
@@ -3232,6 +3727,10 @@
         <v/>
       </c>
       <c r="J122" s="12" t="n"/>
+      <c r="K122" s="26">
+        <f>IF(ISNUMBER($D122),IF($D122&gt;=2,ROUND(($D122-1)*100,0),IF($D122&gt;1,ROUND(-100/($D122-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="123" ht="15" customHeight="1" s="23">
       <c r="A123" s="11" t="n"/>
@@ -3253,6 +3752,10 @@
         <v/>
       </c>
       <c r="J123" s="12" t="n"/>
+      <c r="K123" s="26">
+        <f>IF(ISNUMBER($D123),IF($D123&gt;=2,ROUND(($D123-1)*100,0),IF($D123&gt;1,ROUND(-100/($D123-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="124" ht="15" customHeight="1" s="23">
       <c r="A124" s="11" t="n"/>
@@ -3274,6 +3777,10 @@
         <v/>
       </c>
       <c r="J124" s="12" t="n"/>
+      <c r="K124" s="26">
+        <f>IF(ISNUMBER($D124),IF($D124&gt;=2,ROUND(($D124-1)*100,0),IF($D124&gt;1,ROUND(-100/($D124-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="125" ht="15" customHeight="1" s="23">
       <c r="A125" s="11" t="n"/>
@@ -3295,6 +3802,10 @@
         <v/>
       </c>
       <c r="J125" s="12" t="n"/>
+      <c r="K125" s="26">
+        <f>IF(ISNUMBER($D125),IF($D125&gt;=2,ROUND(($D125-1)*100,0),IF($D125&gt;1,ROUND(-100/($D125-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="126" ht="15" customHeight="1" s="23">
       <c r="A126" s="11" t="n"/>
@@ -3316,6 +3827,10 @@
         <v/>
       </c>
       <c r="J126" s="12" t="n"/>
+      <c r="K126" s="26">
+        <f>IF(ISNUMBER($D126),IF($D126&gt;=2,ROUND(($D126-1)*100,0),IF($D126&gt;1,ROUND(-100/($D126-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="127" ht="15" customHeight="1" s="23">
       <c r="A127" s="11" t="n"/>
@@ -3337,6 +3852,10 @@
         <v/>
       </c>
       <c r="J127" s="12" t="n"/>
+      <c r="K127" s="26">
+        <f>IF(ISNUMBER($D127),IF($D127&gt;=2,ROUND(($D127-1)*100,0),IF($D127&gt;1,ROUND(-100/($D127-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="128" ht="15" customHeight="1" s="23">
       <c r="A128" s="11" t="n"/>
@@ -3358,6 +3877,10 @@
         <v/>
       </c>
       <c r="J128" s="12" t="n"/>
+      <c r="K128" s="26">
+        <f>IF(ISNUMBER($D128),IF($D128&gt;=2,ROUND(($D128-1)*100,0),IF($D128&gt;1,ROUND(-100/($D128-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="129" ht="15" customHeight="1" s="23">
       <c r="A129" s="11" t="n"/>
@@ -3379,6 +3902,10 @@
         <v/>
       </c>
       <c r="J129" s="12" t="n"/>
+      <c r="K129" s="26">
+        <f>IF(ISNUMBER($D129),IF($D129&gt;=2,ROUND(($D129-1)*100,0),IF($D129&gt;1,ROUND(-100/($D129-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="130" ht="15" customHeight="1" s="23">
       <c r="A130" s="11" t="n"/>
@@ -3400,6 +3927,10 @@
         <v/>
       </c>
       <c r="J130" s="12" t="n"/>
+      <c r="K130" s="26">
+        <f>IF(ISNUMBER($D130),IF($D130&gt;=2,ROUND(($D130-1)*100,0),IF($D130&gt;1,ROUND(-100/($D130-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="131" ht="15" customHeight="1" s="23">
       <c r="A131" s="11" t="n"/>
@@ -3421,6 +3952,10 @@
         <v/>
       </c>
       <c r="J131" s="12" t="n"/>
+      <c r="K131" s="26">
+        <f>IF(ISNUMBER($D131),IF($D131&gt;=2,ROUND(($D131-1)*100,0),IF($D131&gt;1,ROUND(-100/($D131-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="132" ht="15" customHeight="1" s="23">
       <c r="A132" s="11" t="n"/>
@@ -3442,6 +3977,10 @@
         <v/>
       </c>
       <c r="J132" s="12" t="n"/>
+      <c r="K132" s="26">
+        <f>IF(ISNUMBER($D132),IF($D132&gt;=2,ROUND(($D132-1)*100,0),IF($D132&gt;1,ROUND(-100/($D132-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="133" ht="15" customHeight="1" s="23">
       <c r="A133" s="11" t="n"/>
@@ -3463,6 +4002,10 @@
         <v/>
       </c>
       <c r="J133" s="12" t="n"/>
+      <c r="K133" s="26">
+        <f>IF(ISNUMBER($D133),IF($D133&gt;=2,ROUND(($D133-1)*100,0),IF($D133&gt;1,ROUND(-100/($D133-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="134" ht="15" customHeight="1" s="23">
       <c r="A134" s="11" t="n"/>
@@ -3484,6 +4027,10 @@
         <v/>
       </c>
       <c r="J134" s="12" t="n"/>
+      <c r="K134" s="26">
+        <f>IF(ISNUMBER($D134),IF($D134&gt;=2,ROUND(($D134-1)*100,0),IF($D134&gt;1,ROUND(-100/($D134-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="135" ht="15" customHeight="1" s="23">
       <c r="A135" s="11" t="n"/>
@@ -3505,6 +4052,10 @@
         <v/>
       </c>
       <c r="J135" s="12" t="n"/>
+      <c r="K135" s="26">
+        <f>IF(ISNUMBER($D135),IF($D135&gt;=2,ROUND(($D135-1)*100,0),IF($D135&gt;1,ROUND(-100/($D135-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="136" ht="15" customHeight="1" s="23">
       <c r="A136" s="11" t="n"/>
@@ -3526,6 +4077,10 @@
         <v/>
       </c>
       <c r="J136" s="12" t="n"/>
+      <c r="K136" s="26">
+        <f>IF(ISNUMBER($D136),IF($D136&gt;=2,ROUND(($D136-1)*100,0),IF($D136&gt;1,ROUND(-100/($D136-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="137" ht="15" customHeight="1" s="23">
       <c r="A137" s="11" t="n"/>
@@ -3547,6 +4102,10 @@
         <v/>
       </c>
       <c r="J137" s="12" t="n"/>
+      <c r="K137" s="26">
+        <f>IF(ISNUMBER($D137),IF($D137&gt;=2,ROUND(($D137-1)*100,0),IF($D137&gt;1,ROUND(-100/($D137-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="138" ht="15" customHeight="1" s="23">
       <c r="A138" s="11" t="n"/>
@@ -3568,6 +4127,10 @@
         <v/>
       </c>
       <c r="J138" s="12" t="n"/>
+      <c r="K138" s="26">
+        <f>IF(ISNUMBER($D138),IF($D138&gt;=2,ROUND(($D138-1)*100,0),IF($D138&gt;1,ROUND(-100/($D138-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="139" ht="15" customHeight="1" s="23">
       <c r="A139" s="11" t="n"/>
@@ -3589,6 +4152,10 @@
         <v/>
       </c>
       <c r="J139" s="12" t="n"/>
+      <c r="K139" s="26">
+        <f>IF(ISNUMBER($D139),IF($D139&gt;=2,ROUND(($D139-1)*100,0),IF($D139&gt;1,ROUND(-100/($D139-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="140" ht="15" customHeight="1" s="23">
       <c r="A140" s="11" t="n"/>
@@ -3610,6 +4177,10 @@
         <v/>
       </c>
       <c r="J140" s="12" t="n"/>
+      <c r="K140" s="26">
+        <f>IF(ISNUMBER($D140),IF($D140&gt;=2,ROUND(($D140-1)*100,0),IF($D140&gt;1,ROUND(-100/($D140-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="141" ht="15" customHeight="1" s="23">
       <c r="A141" s="11" t="n"/>
@@ -3631,6 +4202,10 @@
         <v/>
       </c>
       <c r="J141" s="12" t="n"/>
+      <c r="K141" s="26">
+        <f>IF(ISNUMBER($D141),IF($D141&gt;=2,ROUND(($D141-1)*100,0),IF($D141&gt;1,ROUND(-100/($D141-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="142" ht="15" customHeight="1" s="23">
       <c r="A142" s="11" t="n"/>
@@ -3652,6 +4227,10 @@
         <v/>
       </c>
       <c r="J142" s="12" t="n"/>
+      <c r="K142" s="26">
+        <f>IF(ISNUMBER($D142),IF($D142&gt;=2,ROUND(($D142-1)*100,0),IF($D142&gt;1,ROUND(-100/($D142-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="143" ht="15" customHeight="1" s="23">
       <c r="A143" s="11" t="n"/>
@@ -3673,6 +4252,10 @@
         <v/>
       </c>
       <c r="J143" s="12" t="n"/>
+      <c r="K143" s="26">
+        <f>IF(ISNUMBER($D143),IF($D143&gt;=2,ROUND(($D143-1)*100,0),IF($D143&gt;1,ROUND(-100/($D143-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="144" ht="15" customHeight="1" s="23">
       <c r="A144" s="11" t="n"/>
@@ -3694,6 +4277,10 @@
         <v/>
       </c>
       <c r="J144" s="12" t="n"/>
+      <c r="K144" s="26">
+        <f>IF(ISNUMBER($D144),IF($D144&gt;=2,ROUND(($D144-1)*100,0),IF($D144&gt;1,ROUND(-100/($D144-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="145" ht="15" customHeight="1" s="23">
       <c r="A145" s="11" t="n"/>
@@ -3715,6 +4302,10 @@
         <v/>
       </c>
       <c r="J145" s="12" t="n"/>
+      <c r="K145" s="26">
+        <f>IF(ISNUMBER($D145),IF($D145&gt;=2,ROUND(($D145-1)*100,0),IF($D145&gt;1,ROUND(-100/($D145-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="146" ht="15" customHeight="1" s="23">
       <c r="A146" s="11" t="n"/>
@@ -3736,6 +4327,10 @@
         <v/>
       </c>
       <c r="J146" s="12" t="n"/>
+      <c r="K146" s="26">
+        <f>IF(ISNUMBER($D146),IF($D146&gt;=2,ROUND(($D146-1)*100,0),IF($D146&gt;1,ROUND(-100/($D146-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="147" ht="15" customHeight="1" s="23">
       <c r="A147" s="11" t="n"/>
@@ -3757,6 +4352,10 @@
         <v/>
       </c>
       <c r="J147" s="12" t="n"/>
+      <c r="K147" s="26">
+        <f>IF(ISNUMBER($D147),IF($D147&gt;=2,ROUND(($D147-1)*100,0),IF($D147&gt;1,ROUND(-100/($D147-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="148" ht="15" customHeight="1" s="23">
       <c r="A148" s="11" t="n"/>
@@ -3778,6 +4377,10 @@
         <v/>
       </c>
       <c r="J148" s="12" t="n"/>
+      <c r="K148" s="26">
+        <f>IF(ISNUMBER($D148),IF($D148&gt;=2,ROUND(($D148-1)*100,0),IF($D148&gt;1,ROUND(-100/($D148-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="149" ht="15" customHeight="1" s="23">
       <c r="A149" s="11" t="n"/>
@@ -3799,6 +4402,10 @@
         <v/>
       </c>
       <c r="J149" s="12" t="n"/>
+      <c r="K149" s="26">
+        <f>IF(ISNUMBER($D149),IF($D149&gt;=2,ROUND(($D149-1)*100,0),IF($D149&gt;1,ROUND(-100/($D149-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="150" ht="15" customHeight="1" s="23">
       <c r="A150" s="11" t="n"/>
@@ -3820,6 +4427,10 @@
         <v/>
       </c>
       <c r="J150" s="12" t="n"/>
+      <c r="K150" s="26">
+        <f>IF(ISNUMBER($D150),IF($D150&gt;=2,ROUND(($D150-1)*100,0),IF($D150&gt;1,ROUND(-100/($D150-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="151" ht="15" customHeight="1" s="23">
       <c r="A151" s="11" t="n"/>
@@ -3841,6 +4452,10 @@
         <v/>
       </c>
       <c r="J151" s="12" t="n"/>
+      <c r="K151" s="26">
+        <f>IF(ISNUMBER($D151),IF($D151&gt;=2,ROUND(($D151-1)*100,0),IF($D151&gt;1,ROUND(-100/($D151-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="152" ht="15" customHeight="1" s="23">
       <c r="A152" s="11" t="n"/>
@@ -3862,6 +4477,10 @@
         <v/>
       </c>
       <c r="J152" s="12" t="n"/>
+      <c r="K152" s="26">
+        <f>IF(ISNUMBER($D152),IF($D152&gt;=2,ROUND(($D152-1)*100,0),IF($D152&gt;1,ROUND(-100/($D152-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="153" ht="15" customHeight="1" s="23">
       <c r="A153" s="11" t="n"/>
@@ -3883,6 +4502,10 @@
         <v/>
       </c>
       <c r="J153" s="12" t="n"/>
+      <c r="K153" s="26">
+        <f>IF(ISNUMBER($D153),IF($D153&gt;=2,ROUND(($D153-1)*100,0),IF($D153&gt;1,ROUND(-100/($D153-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="154" ht="15" customHeight="1" s="23">
       <c r="A154" s="11" t="n"/>
@@ -3904,6 +4527,10 @@
         <v/>
       </c>
       <c r="J154" s="12" t="n"/>
+      <c r="K154" s="26">
+        <f>IF(ISNUMBER($D154),IF($D154&gt;=2,ROUND(($D154-1)*100,0),IF($D154&gt;1,ROUND(-100/($D154-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="155" ht="15" customHeight="1" s="23">
       <c r="A155" s="11" t="n"/>
@@ -3925,6 +4552,10 @@
         <v/>
       </c>
       <c r="J155" s="12" t="n"/>
+      <c r="K155" s="26">
+        <f>IF(ISNUMBER($D155),IF($D155&gt;=2,ROUND(($D155-1)*100,0),IF($D155&gt;1,ROUND(-100/($D155-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="156" ht="15" customHeight="1" s="23">
       <c r="A156" s="11" t="n"/>
@@ -3946,6 +4577,10 @@
         <v/>
       </c>
       <c r="J156" s="12" t="n"/>
+      <c r="K156" s="26">
+        <f>IF(ISNUMBER($D156),IF($D156&gt;=2,ROUND(($D156-1)*100,0),IF($D156&gt;1,ROUND(-100/($D156-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="157" ht="15" customHeight="1" s="23">
       <c r="A157" s="11" t="n"/>
@@ -3967,6 +4602,10 @@
         <v/>
       </c>
       <c r="J157" s="12" t="n"/>
+      <c r="K157" s="26">
+        <f>IF(ISNUMBER($D157),IF($D157&gt;=2,ROUND(($D157-1)*100,0),IF($D157&gt;1,ROUND(-100/($D157-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="158" ht="15" customHeight="1" s="23">
       <c r="A158" s="11" t="n"/>
@@ -3988,6 +4627,10 @@
         <v/>
       </c>
       <c r="J158" s="12" t="n"/>
+      <c r="K158" s="26">
+        <f>IF(ISNUMBER($D158),IF($D158&gt;=2,ROUND(($D158-1)*100,0),IF($D158&gt;1,ROUND(-100/($D158-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="159" ht="15" customHeight="1" s="23">
       <c r="A159" s="11" t="n"/>
@@ -4009,6 +4652,10 @@
         <v/>
       </c>
       <c r="J159" s="12" t="n"/>
+      <c r="K159" s="26">
+        <f>IF(ISNUMBER($D159),IF($D159&gt;=2,ROUND(($D159-1)*100,0),IF($D159&gt;1,ROUND(-100/($D159-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="160" ht="15" customHeight="1" s="23">
       <c r="A160" s="11" t="n"/>
@@ -4030,6 +4677,10 @@
         <v/>
       </c>
       <c r="J160" s="12" t="n"/>
+      <c r="K160" s="26">
+        <f>IF(ISNUMBER($D160),IF($D160&gt;=2,ROUND(($D160-1)*100,0),IF($D160&gt;1,ROUND(-100/($D160-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="161" ht="15" customHeight="1" s="23">
       <c r="A161" s="11" t="n"/>
@@ -4051,6 +4702,10 @@
         <v/>
       </c>
       <c r="J161" s="12" t="n"/>
+      <c r="K161" s="26">
+        <f>IF(ISNUMBER($D161),IF($D161&gt;=2,ROUND(($D161-1)*100,0),IF($D161&gt;1,ROUND(-100/($D161-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="162" ht="15" customHeight="1" s="23">
       <c r="A162" s="11" t="n"/>
@@ -4072,6 +4727,10 @@
         <v/>
       </c>
       <c r="J162" s="12" t="n"/>
+      <c r="K162" s="26">
+        <f>IF(ISNUMBER($D162),IF($D162&gt;=2,ROUND(($D162-1)*100,0),IF($D162&gt;1,ROUND(-100/($D162-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="163" ht="15" customHeight="1" s="23">
       <c r="A163" s="11" t="n"/>
@@ -4093,6 +4752,10 @@
         <v/>
       </c>
       <c r="J163" s="12" t="n"/>
+      <c r="K163" s="26">
+        <f>IF(ISNUMBER($D163),IF($D163&gt;=2,ROUND(($D163-1)*100,0),IF($D163&gt;1,ROUND(-100/($D163-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="164" ht="15" customHeight="1" s="23">
       <c r="A164" s="11" t="n"/>
@@ -4114,6 +4777,10 @@
         <v/>
       </c>
       <c r="J164" s="12" t="n"/>
+      <c r="K164" s="26">
+        <f>IF(ISNUMBER($D164),IF($D164&gt;=2,ROUND(($D164-1)*100,0),IF($D164&gt;1,ROUND(-100/($D164-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="165" ht="15" customHeight="1" s="23">
       <c r="A165" s="11" t="n"/>
@@ -4135,6 +4802,10 @@
         <v/>
       </c>
       <c r="J165" s="12" t="n"/>
+      <c r="K165" s="26">
+        <f>IF(ISNUMBER($D165),IF($D165&gt;=2,ROUND(($D165-1)*100,0),IF($D165&gt;1,ROUND(-100/($D165-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="166" ht="15" customHeight="1" s="23">
       <c r="A166" s="11" t="n"/>
@@ -4156,6 +4827,10 @@
         <v/>
       </c>
       <c r="J166" s="12" t="n"/>
+      <c r="K166" s="26">
+        <f>IF(ISNUMBER($D166),IF($D166&gt;=2,ROUND(($D166-1)*100,0),IF($D166&gt;1,ROUND(-100/($D166-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="167" ht="15" customHeight="1" s="23">
       <c r="A167" s="11" t="n"/>
@@ -4177,6 +4852,10 @@
         <v/>
       </c>
       <c r="J167" s="12" t="n"/>
+      <c r="K167" s="26">
+        <f>IF(ISNUMBER($D167),IF($D167&gt;=2,ROUND(($D167-1)*100,0),IF($D167&gt;1,ROUND(-100/($D167-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="168" ht="15" customHeight="1" s="23">
       <c r="A168" s="11" t="n"/>
@@ -4198,6 +4877,10 @@
         <v/>
       </c>
       <c r="J168" s="12" t="n"/>
+      <c r="K168" s="26">
+        <f>IF(ISNUMBER($D168),IF($D168&gt;=2,ROUND(($D168-1)*100,0),IF($D168&gt;1,ROUND(-100/($D168-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="169" ht="15" customHeight="1" s="23">
       <c r="A169" s="11" t="n"/>
@@ -4219,6 +4902,10 @@
         <v/>
       </c>
       <c r="J169" s="12" t="n"/>
+      <c r="K169" s="26">
+        <f>IF(ISNUMBER($D169),IF($D169&gt;=2,ROUND(($D169-1)*100,0),IF($D169&gt;1,ROUND(-100/($D169-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="170" ht="15" customHeight="1" s="23">
       <c r="A170" s="11" t="n"/>
@@ -4240,6 +4927,10 @@
         <v/>
       </c>
       <c r="J170" s="12" t="n"/>
+      <c r="K170" s="26">
+        <f>IF(ISNUMBER($D170),IF($D170&gt;=2,ROUND(($D170-1)*100,0),IF($D170&gt;1,ROUND(-100/($D170-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="171" ht="15" customHeight="1" s="23">
       <c r="A171" s="11" t="n"/>
@@ -4261,6 +4952,10 @@
         <v/>
       </c>
       <c r="J171" s="12" t="n"/>
+      <c r="K171" s="26">
+        <f>IF(ISNUMBER($D171),IF($D171&gt;=2,ROUND(($D171-1)*100,0),IF($D171&gt;1,ROUND(-100/($D171-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="172" ht="15" customHeight="1" s="23">
       <c r="A172" s="11" t="n"/>
@@ -4282,6 +4977,10 @@
         <v/>
       </c>
       <c r="J172" s="12" t="n"/>
+      <c r="K172" s="26">
+        <f>IF(ISNUMBER($D172),IF($D172&gt;=2,ROUND(($D172-1)*100,0),IF($D172&gt;1,ROUND(-100/($D172-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="173" ht="15" customHeight="1" s="23">
       <c r="A173" s="11" t="n"/>
@@ -4303,6 +5002,10 @@
         <v/>
       </c>
       <c r="J173" s="12" t="n"/>
+      <c r="K173" s="26">
+        <f>IF(ISNUMBER($D173),IF($D173&gt;=2,ROUND(($D173-1)*100,0),IF($D173&gt;1,ROUND(-100/($D173-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="174" ht="15" customHeight="1" s="23">
       <c r="A174" s="11" t="n"/>
@@ -4324,6 +5027,10 @@
         <v/>
       </c>
       <c r="J174" s="12" t="n"/>
+      <c r="K174" s="26">
+        <f>IF(ISNUMBER($D174),IF($D174&gt;=2,ROUND(($D174-1)*100,0),IF($D174&gt;1,ROUND(-100/($D174-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="175" ht="15" customHeight="1" s="23">
       <c r="A175" s="11" t="n"/>
@@ -4345,6 +5052,10 @@
         <v/>
       </c>
       <c r="J175" s="12" t="n"/>
+      <c r="K175" s="26">
+        <f>IF(ISNUMBER($D175),IF($D175&gt;=2,ROUND(($D175-1)*100,0),IF($D175&gt;1,ROUND(-100/($D175-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="176" ht="15" customHeight="1" s="23">
       <c r="A176" s="11" t="n"/>
@@ -4366,6 +5077,10 @@
         <v/>
       </c>
       <c r="J176" s="12" t="n"/>
+      <c r="K176" s="26">
+        <f>IF(ISNUMBER($D176),IF($D176&gt;=2,ROUND(($D176-1)*100,0),IF($D176&gt;1,ROUND(-100/($D176-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="177" ht="15" customHeight="1" s="23">
       <c r="A177" s="11" t="n"/>
@@ -4387,6 +5102,10 @@
         <v/>
       </c>
       <c r="J177" s="12" t="n"/>
+      <c r="K177" s="26">
+        <f>IF(ISNUMBER($D177),IF($D177&gt;=2,ROUND(($D177-1)*100,0),IF($D177&gt;1,ROUND(-100/($D177-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="178" ht="15" customHeight="1" s="23">
       <c r="A178" s="11" t="n"/>
@@ -4408,6 +5127,10 @@
         <v/>
       </c>
       <c r="J178" s="12" t="n"/>
+      <c r="K178" s="26">
+        <f>IF(ISNUMBER($D178),IF($D178&gt;=2,ROUND(($D178-1)*100,0),IF($D178&gt;1,ROUND(-100/($D178-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="179" ht="15" customHeight="1" s="23">
       <c r="A179" s="11" t="n"/>
@@ -4429,6 +5152,10 @@
         <v/>
       </c>
       <c r="J179" s="12" t="n"/>
+      <c r="K179" s="26">
+        <f>IF(ISNUMBER($D179),IF($D179&gt;=2,ROUND(($D179-1)*100,0),IF($D179&gt;1,ROUND(-100/($D179-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="180" ht="15" customHeight="1" s="23">
       <c r="A180" s="11" t="n"/>
@@ -4450,6 +5177,10 @@
         <v/>
       </c>
       <c r="J180" s="12" t="n"/>
+      <c r="K180" s="26">
+        <f>IF(ISNUMBER($D180),IF($D180&gt;=2,ROUND(($D180-1)*100,0),IF($D180&gt;1,ROUND(-100/($D180-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="181" ht="15" customHeight="1" s="23">
       <c r="A181" s="11" t="n"/>
@@ -4471,6 +5202,10 @@
         <v/>
       </c>
       <c r="J181" s="12" t="n"/>
+      <c r="K181" s="26">
+        <f>IF(ISNUMBER($D181),IF($D181&gt;=2,ROUND(($D181-1)*100,0),IF($D181&gt;1,ROUND(-100/($D181-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="182" ht="15" customHeight="1" s="23">
       <c r="A182" s="11" t="n"/>
@@ -4492,6 +5227,10 @@
         <v/>
       </c>
       <c r="J182" s="12" t="n"/>
+      <c r="K182" s="26">
+        <f>IF(ISNUMBER($D182),IF($D182&gt;=2,ROUND(($D182-1)*100,0),IF($D182&gt;1,ROUND(-100/($D182-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="183" ht="15" customHeight="1" s="23">
       <c r="A183" s="11" t="n"/>
@@ -4513,6 +5252,10 @@
         <v/>
       </c>
       <c r="J183" s="12" t="n"/>
+      <c r="K183" s="26">
+        <f>IF(ISNUMBER($D183),IF($D183&gt;=2,ROUND(($D183-1)*100,0),IF($D183&gt;1,ROUND(-100/($D183-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="184" ht="15" customHeight="1" s="23">
       <c r="A184" s="11" t="n"/>
@@ -4534,6 +5277,10 @@
         <v/>
       </c>
       <c r="J184" s="12" t="n"/>
+      <c r="K184" s="26">
+        <f>IF(ISNUMBER($D184),IF($D184&gt;=2,ROUND(($D184-1)*100,0),IF($D184&gt;1,ROUND(-100/($D184-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="185" ht="15" customHeight="1" s="23">
       <c r="A185" s="11" t="n"/>
@@ -4555,6 +5302,10 @@
         <v/>
       </c>
       <c r="J185" s="12" t="n"/>
+      <c r="K185" s="26">
+        <f>IF(ISNUMBER($D185),IF($D185&gt;=2,ROUND(($D185-1)*100,0),IF($D185&gt;1,ROUND(-100/($D185-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="186" ht="15" customHeight="1" s="23">
       <c r="A186" s="11" t="n"/>
@@ -4576,6 +5327,10 @@
         <v/>
       </c>
       <c r="J186" s="12" t="n"/>
+      <c r="K186" s="26">
+        <f>IF(ISNUMBER($D186),IF($D186&gt;=2,ROUND(($D186-1)*100,0),IF($D186&gt;1,ROUND(-100/($D186-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="187" ht="15" customHeight="1" s="23">
       <c r="A187" s="11" t="n"/>
@@ -4597,6 +5352,10 @@
         <v/>
       </c>
       <c r="J187" s="12" t="n"/>
+      <c r="K187" s="26">
+        <f>IF(ISNUMBER($D187),IF($D187&gt;=2,ROUND(($D187-1)*100,0),IF($D187&gt;1,ROUND(-100/($D187-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="188" ht="15" customHeight="1" s="23">
       <c r="A188" s="11" t="n"/>
@@ -4618,6 +5377,10 @@
         <v/>
       </c>
       <c r="J188" s="12" t="n"/>
+      <c r="K188" s="26">
+        <f>IF(ISNUMBER($D188),IF($D188&gt;=2,ROUND(($D188-1)*100,0),IF($D188&gt;1,ROUND(-100/($D188-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="189" ht="15" customHeight="1" s="23">
       <c r="A189" s="11" t="n"/>
@@ -4639,6 +5402,10 @@
         <v/>
       </c>
       <c r="J189" s="12" t="n"/>
+      <c r="K189" s="26">
+        <f>IF(ISNUMBER($D189),IF($D189&gt;=2,ROUND(($D189-1)*100,0),IF($D189&gt;1,ROUND(-100/($D189-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="190" ht="15" customHeight="1" s="23">
       <c r="A190" s="11" t="n"/>
@@ -4660,6 +5427,10 @@
         <v/>
       </c>
       <c r="J190" s="12" t="n"/>
+      <c r="K190" s="26">
+        <f>IF(ISNUMBER($D190),IF($D190&gt;=2,ROUND(($D190-1)*100,0),IF($D190&gt;1,ROUND(-100/($D190-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="191" ht="15" customHeight="1" s="23">
       <c r="A191" s="11" t="n"/>
@@ -4681,6 +5452,10 @@
         <v/>
       </c>
       <c r="J191" s="12" t="n"/>
+      <c r="K191" s="26">
+        <f>IF(ISNUMBER($D191),IF($D191&gt;=2,ROUND(($D191-1)*100,0),IF($D191&gt;1,ROUND(-100/($D191-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="192" ht="15" customHeight="1" s="23">
       <c r="A192" s="11" t="n"/>
@@ -4702,6 +5477,10 @@
         <v/>
       </c>
       <c r="J192" s="12" t="n"/>
+      <c r="K192" s="26">
+        <f>IF(ISNUMBER($D192),IF($D192&gt;=2,ROUND(($D192-1)*100,0),IF($D192&gt;1,ROUND(-100/($D192-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="193" ht="15" customHeight="1" s="23">
       <c r="A193" s="11" t="n"/>
@@ -4723,6 +5502,10 @@
         <v/>
       </c>
       <c r="J193" s="12" t="n"/>
+      <c r="K193" s="26">
+        <f>IF(ISNUMBER($D193),IF($D193&gt;=2,ROUND(($D193-1)*100,0),IF($D193&gt;1,ROUND(-100/($D193-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="194" ht="15" customHeight="1" s="23">
       <c r="A194" s="11" t="n"/>
@@ -4744,6 +5527,10 @@
         <v/>
       </c>
       <c r="J194" s="12" t="n"/>
+      <c r="K194" s="26">
+        <f>IF(ISNUMBER($D194),IF($D194&gt;=2,ROUND(($D194-1)*100,0),IF($D194&gt;1,ROUND(-100/($D194-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="195" ht="15" customHeight="1" s="23">
       <c r="A195" s="11" t="n"/>
@@ -4765,6 +5552,10 @@
         <v/>
       </c>
       <c r="J195" s="12" t="n"/>
+      <c r="K195" s="26">
+        <f>IF(ISNUMBER($D195),IF($D195&gt;=2,ROUND(($D195-1)*100,0),IF($D195&gt;1,ROUND(-100/($D195-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="196" ht="15" customHeight="1" s="23">
       <c r="A196" s="11" t="n"/>
@@ -4786,6 +5577,10 @@
         <v/>
       </c>
       <c r="J196" s="12" t="n"/>
+      <c r="K196" s="26">
+        <f>IF(ISNUMBER($D196),IF($D196&gt;=2,ROUND(($D196-1)*100,0),IF($D196&gt;1,ROUND(-100/($D196-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="197" ht="15" customHeight="1" s="23">
       <c r="A197" s="11" t="n"/>
@@ -4807,6 +5602,10 @@
         <v/>
       </c>
       <c r="J197" s="12" t="n"/>
+      <c r="K197" s="26">
+        <f>IF(ISNUMBER($D197),IF($D197&gt;=2,ROUND(($D197-1)*100,0),IF($D197&gt;1,ROUND(-100/($D197-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="198" ht="15" customHeight="1" s="23">
       <c r="A198" s="11" t="n"/>
@@ -4828,6 +5627,10 @@
         <v/>
       </c>
       <c r="J198" s="12" t="n"/>
+      <c r="K198" s="26">
+        <f>IF(ISNUMBER($D198),IF($D198&gt;=2,ROUND(($D198-1)*100,0),IF($D198&gt;1,ROUND(-100/($D198-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="199" ht="15" customHeight="1" s="23">
       <c r="A199" s="11" t="n"/>
@@ -4849,6 +5652,10 @@
         <v/>
       </c>
       <c r="J199" s="12" t="n"/>
+      <c r="K199" s="26">
+        <f>IF(ISNUMBER($D199),IF($D199&gt;=2,ROUND(($D199-1)*100,0),IF($D199&gt;1,ROUND(-100/($D199-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="200" ht="15" customHeight="1" s="23">
       <c r="A200" s="11" t="n"/>
@@ -4870,6 +5677,10 @@
         <v/>
       </c>
       <c r="J200" s="12" t="n"/>
+      <c r="K200" s="26">
+        <f>IF(ISNUMBER($D200),IF($D200&gt;=2,ROUND(($D200-1)*100,0),IF($D200&gt;1,ROUND(-100/($D200-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="201" ht="15" customHeight="1" s="23">
       <c r="A201" s="11" t="n"/>
@@ -4891,6 +5702,10 @@
         <v/>
       </c>
       <c r="J201" s="12" t="n"/>
+      <c r="K201" s="26">
+        <f>IF(ISNUMBER($D201),IF($D201&gt;=2,ROUND(($D201-1)*100,0),IF($D201&gt;1,ROUND(-100/($D201-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="202" ht="15" customHeight="1" s="23">
       <c r="A202" s="11" t="n"/>
@@ -4912,6 +5727,10 @@
         <v/>
       </c>
       <c r="J202" s="12" t="n"/>
+      <c r="K202" s="26">
+        <f>IF(ISNUMBER($D202),IF($D202&gt;=2,ROUND(($D202-1)*100,0),IF($D202&gt;1,ROUND(-100/($D202-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="203" ht="15" customHeight="1" s="23">
       <c r="A203" s="11" t="n"/>
@@ -4933,6 +5752,10 @@
         <v/>
       </c>
       <c r="J203" s="12" t="n"/>
+      <c r="K203" s="26">
+        <f>IF(ISNUMBER($D203),IF($D203&gt;=2,ROUND(($D203-1)*100,0),IF($D203&gt;1,ROUND(-100/($D203-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="204" ht="15" customHeight="1" s="23">
       <c r="A204" s="11" t="n"/>
@@ -4954,6 +5777,10 @@
         <v/>
       </c>
       <c r="J204" s="12" t="n"/>
+      <c r="K204" s="26">
+        <f>IF(ISNUMBER($D204),IF($D204&gt;=2,ROUND(($D204-1)*100,0),IF($D204&gt;1,ROUND(-100/($D204-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="205" ht="15" customHeight="1" s="23">
       <c r="A205" s="11" t="n"/>
@@ -4975,6 +5802,10 @@
         <v/>
       </c>
       <c r="J205" s="12" t="n"/>
+      <c r="K205" s="26">
+        <f>IF(ISNUMBER($D205),IF($D205&gt;=2,ROUND(($D205-1)*100,0),IF($D205&gt;1,ROUND(-100/($D205-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="206" ht="15" customHeight="1" s="23">
       <c r="A206" s="11" t="n"/>
@@ -4996,6 +5827,10 @@
         <v/>
       </c>
       <c r="J206" s="12" t="n"/>
+      <c r="K206" s="26">
+        <f>IF(ISNUMBER($D206),IF($D206&gt;=2,ROUND(($D206-1)*100,0),IF($D206&gt;1,ROUND(-100/($D206-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="207" ht="15" customHeight="1" s="23">
       <c r="A207" s="11" t="n"/>
@@ -5017,6 +5852,10 @@
         <v/>
       </c>
       <c r="J207" s="12" t="n"/>
+      <c r="K207" s="26">
+        <f>IF(ISNUMBER($D207),IF($D207&gt;=2,ROUND(($D207-1)*100,0),IF($D207&gt;1,ROUND(-100/($D207-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="208" ht="15" customHeight="1" s="23">
       <c r="A208" s="11" t="n"/>
@@ -5038,6 +5877,10 @@
         <v/>
       </c>
       <c r="J208" s="12" t="n"/>
+      <c r="K208" s="26">
+        <f>IF(ISNUMBER($D208),IF($D208&gt;=2,ROUND(($D208-1)*100,0),IF($D208&gt;1,ROUND(-100/($D208-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="209" ht="15" customHeight="1" s="23">
       <c r="A209" s="11" t="n"/>
@@ -5059,6 +5902,10 @@
         <v/>
       </c>
       <c r="J209" s="12" t="n"/>
+      <c r="K209" s="26">
+        <f>IF(ISNUMBER($D209),IF($D209&gt;=2,ROUND(($D209-1)*100,0),IF($D209&gt;1,ROUND(-100/($D209-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="210" ht="15" customHeight="1" s="23">
       <c r="A210" s="11" t="n"/>
@@ -5080,6 +5927,10 @@
         <v/>
       </c>
       <c r="J210" s="12" t="n"/>
+      <c r="K210" s="26">
+        <f>IF(ISNUMBER($D210),IF($D210&gt;=2,ROUND(($D210-1)*100,0),IF($D210&gt;1,ROUND(-100/($D210-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="211" ht="15" customHeight="1" s="23">
       <c r="A211" s="11" t="n"/>
@@ -5101,6 +5952,10 @@
         <v/>
       </c>
       <c r="J211" s="12" t="n"/>
+      <c r="K211" s="26">
+        <f>IF(ISNUMBER($D211),IF($D211&gt;=2,ROUND(($D211-1)*100,0),IF($D211&gt;1,ROUND(-100/($D211-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="212" ht="15" customHeight="1" s="23">
       <c r="A212" s="11" t="n"/>
@@ -5122,6 +5977,10 @@
         <v/>
       </c>
       <c r="J212" s="12" t="n"/>
+      <c r="K212" s="26">
+        <f>IF(ISNUMBER($D212),IF($D212&gt;=2,ROUND(($D212-1)*100,0),IF($D212&gt;1,ROUND(-100/($D212-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="213" ht="15" customHeight="1" s="23">
       <c r="A213" s="11" t="n"/>
@@ -5143,6 +6002,10 @@
         <v/>
       </c>
       <c r="J213" s="12" t="n"/>
+      <c r="K213" s="26">
+        <f>IF(ISNUMBER($D213),IF($D213&gt;=2,ROUND(($D213-1)*100,0),IF($D213&gt;1,ROUND(-100/($D213-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="214" ht="15" customHeight="1" s="23">
       <c r="A214" s="11" t="n"/>
@@ -5164,6 +6027,10 @@
         <v/>
       </c>
       <c r="J214" s="12" t="n"/>
+      <c r="K214" s="26">
+        <f>IF(ISNUMBER($D214),IF($D214&gt;=2,ROUND(($D214-1)*100,0),IF($D214&gt;1,ROUND(-100/($D214-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="215" ht="15" customHeight="1" s="23">
       <c r="A215" s="11" t="n"/>
@@ -5185,6 +6052,10 @@
         <v/>
       </c>
       <c r="J215" s="12" t="n"/>
+      <c r="K215" s="26">
+        <f>IF(ISNUMBER($D215),IF($D215&gt;=2,ROUND(($D215-1)*100,0),IF($D215&gt;1,ROUND(-100/($D215-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="216" ht="15" customHeight="1" s="23">
       <c r="A216" s="11" t="n"/>
@@ -5206,6 +6077,10 @@
         <v/>
       </c>
       <c r="J216" s="12" t="n"/>
+      <c r="K216" s="26">
+        <f>IF(ISNUMBER($D216),IF($D216&gt;=2,ROUND(($D216-1)*100,0),IF($D216&gt;1,ROUND(-100/($D216-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="217" ht="15" customHeight="1" s="23">
       <c r="A217" s="11" t="n"/>
@@ -5227,6 +6102,10 @@
         <v/>
       </c>
       <c r="J217" s="12" t="n"/>
+      <c r="K217" s="26">
+        <f>IF(ISNUMBER($D217),IF($D217&gt;=2,ROUND(($D217-1)*100,0),IF($D217&gt;1,ROUND(-100/($D217-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="218" ht="15" customHeight="1" s="23">
       <c r="A218" s="11" t="n"/>
@@ -5248,6 +6127,10 @@
         <v/>
       </c>
       <c r="J218" s="12" t="n"/>
+      <c r="K218" s="26">
+        <f>IF(ISNUMBER($D218),IF($D218&gt;=2,ROUND(($D218-1)*100,0),IF($D218&gt;1,ROUND(-100/($D218-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="219" ht="15" customHeight="1" s="23">
       <c r="A219" s="11" t="n"/>
@@ -5269,6 +6152,10 @@
         <v/>
       </c>
       <c r="J219" s="12" t="n"/>
+      <c r="K219" s="26">
+        <f>IF(ISNUMBER($D219),IF($D219&gt;=2,ROUND(($D219-1)*100,0),IF($D219&gt;1,ROUND(-100/($D219-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="220" ht="15" customHeight="1" s="23">
       <c r="A220" s="11" t="n"/>
@@ -5290,6 +6177,10 @@
         <v/>
       </c>
       <c r="J220" s="12" t="n"/>
+      <c r="K220" s="26">
+        <f>IF(ISNUMBER($D220),IF($D220&gt;=2,ROUND(($D220-1)*100,0),IF($D220&gt;1,ROUND(-100/($D220-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="221" ht="15" customHeight="1" s="23">
       <c r="A221" s="11" t="n"/>
@@ -5311,6 +6202,10 @@
         <v/>
       </c>
       <c r="J221" s="12" t="n"/>
+      <c r="K221" s="26">
+        <f>IF(ISNUMBER($D221),IF($D221&gt;=2,ROUND(($D221-1)*100,0),IF($D221&gt;1,ROUND(-100/($D221-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="222" ht="15" customHeight="1" s="23">
       <c r="A222" s="11" t="n"/>
@@ -5332,6 +6227,10 @@
         <v/>
       </c>
       <c r="J222" s="12" t="n"/>
+      <c r="K222" s="26">
+        <f>IF(ISNUMBER($D222),IF($D222&gt;=2,ROUND(($D222-1)*100,0),IF($D222&gt;1,ROUND(-100/($D222-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="223" ht="15" customHeight="1" s="23">
       <c r="A223" s="11" t="n"/>
@@ -5353,6 +6252,10 @@
         <v/>
       </c>
       <c r="J223" s="12" t="n"/>
+      <c r="K223" s="26">
+        <f>IF(ISNUMBER($D223),IF($D223&gt;=2,ROUND(($D223-1)*100,0),IF($D223&gt;1,ROUND(-100/($D223-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="224" ht="15" customHeight="1" s="23">
       <c r="A224" s="11" t="n"/>
@@ -5374,6 +6277,10 @@
         <v/>
       </c>
       <c r="J224" s="12" t="n"/>
+      <c r="K224" s="26">
+        <f>IF(ISNUMBER($D224),IF($D224&gt;=2,ROUND(($D224-1)*100,0),IF($D224&gt;1,ROUND(-100/($D224-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="225" ht="15" customHeight="1" s="23">
       <c r="A225" s="11" t="n"/>
@@ -5395,6 +6302,10 @@
         <v/>
       </c>
       <c r="J225" s="12" t="n"/>
+      <c r="K225" s="26">
+        <f>IF(ISNUMBER($D225),IF($D225&gt;=2,ROUND(($D225-1)*100,0),IF($D225&gt;1,ROUND(-100/($D225-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="226" ht="15" customHeight="1" s="23">
       <c r="A226" s="11" t="n"/>
@@ -5416,6 +6327,10 @@
         <v/>
       </c>
       <c r="J226" s="12" t="n"/>
+      <c r="K226" s="26">
+        <f>IF(ISNUMBER($D226),IF($D226&gt;=2,ROUND(($D226-1)*100,0),IF($D226&gt;1,ROUND(-100/($D226-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="227" ht="15" customHeight="1" s="23">
       <c r="A227" s="11" t="n"/>
@@ -5437,6 +6352,10 @@
         <v/>
       </c>
       <c r="J227" s="12" t="n"/>
+      <c r="K227" s="26">
+        <f>IF(ISNUMBER($D227),IF($D227&gt;=2,ROUND(($D227-1)*100,0),IF($D227&gt;1,ROUND(-100/($D227-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="228" ht="15" customHeight="1" s="23">
       <c r="A228" s="11" t="n"/>
@@ -5458,6 +6377,10 @@
         <v/>
       </c>
       <c r="J228" s="12" t="n"/>
+      <c r="K228" s="26">
+        <f>IF(ISNUMBER($D228),IF($D228&gt;=2,ROUND(($D228-1)*100,0),IF($D228&gt;1,ROUND(-100/($D228-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="229" ht="15" customHeight="1" s="23">
       <c r="A229" s="11" t="n"/>
@@ -5479,6 +6402,10 @@
         <v/>
       </c>
       <c r="J229" s="12" t="n"/>
+      <c r="K229" s="26">
+        <f>IF(ISNUMBER($D229),IF($D229&gt;=2,ROUND(($D229-1)*100,0),IF($D229&gt;1,ROUND(-100/($D229-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="230" ht="15" customHeight="1" s="23">
       <c r="A230" s="11" t="n"/>
@@ -5500,6 +6427,10 @@
         <v/>
       </c>
       <c r="J230" s="12" t="n"/>
+      <c r="K230" s="26">
+        <f>IF(ISNUMBER($D230),IF($D230&gt;=2,ROUND(($D230-1)*100,0),IF($D230&gt;1,ROUND(-100/($D230-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="231" ht="15" customHeight="1" s="23">
       <c r="A231" s="11" t="n"/>
@@ -5521,6 +6452,10 @@
         <v/>
       </c>
       <c r="J231" s="12" t="n"/>
+      <c r="K231" s="26">
+        <f>IF(ISNUMBER($D231),IF($D231&gt;=2,ROUND(($D231-1)*100,0),IF($D231&gt;1,ROUND(-100/($D231-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="232" ht="15" customHeight="1" s="23">
       <c r="A232" s="11" t="n"/>
@@ -5542,6 +6477,10 @@
         <v/>
       </c>
       <c r="J232" s="12" t="n"/>
+      <c r="K232" s="26">
+        <f>IF(ISNUMBER($D232),IF($D232&gt;=2,ROUND(($D232-1)*100,0),IF($D232&gt;1,ROUND(-100/($D232-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="233" ht="15" customHeight="1" s="23">
       <c r="A233" s="11" t="n"/>
@@ -5563,6 +6502,10 @@
         <v/>
       </c>
       <c r="J233" s="12" t="n"/>
+      <c r="K233" s="26">
+        <f>IF(ISNUMBER($D233),IF($D233&gt;=2,ROUND(($D233-1)*100,0),IF($D233&gt;1,ROUND(-100/($D233-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="234" ht="15" customHeight="1" s="23">
       <c r="A234" s="11" t="n"/>
@@ -5584,6 +6527,10 @@
         <v/>
       </c>
       <c r="J234" s="12" t="n"/>
+      <c r="K234" s="26">
+        <f>IF(ISNUMBER($D234),IF($D234&gt;=2,ROUND(($D234-1)*100,0),IF($D234&gt;1,ROUND(-100/($D234-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="235" ht="15" customHeight="1" s="23">
       <c r="A235" s="11" t="n"/>
@@ -5605,6 +6552,10 @@
         <v/>
       </c>
       <c r="J235" s="12" t="n"/>
+      <c r="K235" s="26">
+        <f>IF(ISNUMBER($D235),IF($D235&gt;=2,ROUND(($D235-1)*100,0),IF($D235&gt;1,ROUND(-100/($D235-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="236" ht="15" customHeight="1" s="23">
       <c r="A236" s="11" t="n"/>
@@ -5626,6 +6577,10 @@
         <v/>
       </c>
       <c r="J236" s="12" t="n"/>
+      <c r="K236" s="26">
+        <f>IF(ISNUMBER($D236),IF($D236&gt;=2,ROUND(($D236-1)*100,0),IF($D236&gt;1,ROUND(-100/($D236-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="237" ht="15" customHeight="1" s="23">
       <c r="A237" s="11" t="n"/>
@@ -5647,6 +6602,10 @@
         <v/>
       </c>
       <c r="J237" s="12" t="n"/>
+      <c r="K237" s="26">
+        <f>IF(ISNUMBER($D237),IF($D237&gt;=2,ROUND(($D237-1)*100,0),IF($D237&gt;1,ROUND(-100/($D237-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="238" ht="15" customHeight="1" s="23">
       <c r="A238" s="11" t="n"/>
@@ -5668,6 +6627,10 @@
         <v/>
       </c>
       <c r="J238" s="12" t="n"/>
+      <c r="K238" s="26">
+        <f>IF(ISNUMBER($D238),IF($D238&gt;=2,ROUND(($D238-1)*100,0),IF($D238&gt;1,ROUND(-100/($D238-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="239" ht="15" customHeight="1" s="23">
       <c r="A239" s="11" t="n"/>
@@ -5689,6 +6652,10 @@
         <v/>
       </c>
       <c r="J239" s="12" t="n"/>
+      <c r="K239" s="26">
+        <f>IF(ISNUMBER($D239),IF($D239&gt;=2,ROUND(($D239-1)*100,0),IF($D239&gt;1,ROUND(-100/($D239-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="240" ht="15" customHeight="1" s="23">
       <c r="A240" s="11" t="n"/>
@@ -5710,6 +6677,10 @@
         <v/>
       </c>
       <c r="J240" s="12" t="n"/>
+      <c r="K240" s="26">
+        <f>IF(ISNUMBER($D240),IF($D240&gt;=2,ROUND(($D240-1)*100,0),IF($D240&gt;1,ROUND(-100/($D240-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="241" ht="15" customHeight="1" s="23">
       <c r="A241" s="11" t="n"/>
@@ -5731,6 +6702,10 @@
         <v/>
       </c>
       <c r="J241" s="12" t="n"/>
+      <c r="K241" s="26">
+        <f>IF(ISNUMBER($D241),IF($D241&gt;=2,ROUND(($D241-1)*100,0),IF($D241&gt;1,ROUND(-100/($D241-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="242" ht="15" customHeight="1" s="23">
       <c r="A242" s="11" t="n"/>
@@ -5752,6 +6727,10 @@
         <v/>
       </c>
       <c r="J242" s="12" t="n"/>
+      <c r="K242" s="26">
+        <f>IF(ISNUMBER($D242),IF($D242&gt;=2,ROUND(($D242-1)*100,0),IF($D242&gt;1,ROUND(-100/($D242-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="243" ht="15" customHeight="1" s="23">
       <c r="A243" s="11" t="n"/>
@@ -5773,6 +6752,10 @@
         <v/>
       </c>
       <c r="J243" s="12" t="n"/>
+      <c r="K243" s="26">
+        <f>IF(ISNUMBER($D243),IF($D243&gt;=2,ROUND(($D243-1)*100,0),IF($D243&gt;1,ROUND(-100/($D243-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="244" ht="15" customHeight="1" s="23">
       <c r="A244" s="11" t="n"/>
@@ -5794,6 +6777,10 @@
         <v/>
       </c>
       <c r="J244" s="12" t="n"/>
+      <c r="K244" s="26">
+        <f>IF(ISNUMBER($D244),IF($D244&gt;=2,ROUND(($D244-1)*100,0),IF($D244&gt;1,ROUND(-100/($D244-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="245" ht="15" customHeight="1" s="23">
       <c r="A245" s="11" t="n"/>
@@ -5815,6 +6802,10 @@
         <v/>
       </c>
       <c r="J245" s="12" t="n"/>
+      <c r="K245" s="26">
+        <f>IF(ISNUMBER($D245),IF($D245&gt;=2,ROUND(($D245-1)*100,0),IF($D245&gt;1,ROUND(-100/($D245-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="246" ht="15" customHeight="1" s="23">
       <c r="A246" s="11" t="n"/>
@@ -5836,6 +6827,10 @@
         <v/>
       </c>
       <c r="J246" s="12" t="n"/>
+      <c r="K246" s="26">
+        <f>IF(ISNUMBER($D246),IF($D246&gt;=2,ROUND(($D246-1)*100,0),IF($D246&gt;1,ROUND(-100/($D246-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="247" ht="15" customHeight="1" s="23">
       <c r="A247" s="11" t="n"/>
@@ -5857,6 +6852,10 @@
         <v/>
       </c>
       <c r="J247" s="12" t="n"/>
+      <c r="K247" s="26">
+        <f>IF(ISNUMBER($D247),IF($D247&gt;=2,ROUND(($D247-1)*100,0),IF($D247&gt;1,ROUND(-100/($D247-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="248" ht="15" customHeight="1" s="23">
       <c r="A248" s="11" t="n"/>
@@ -5878,6 +6877,10 @@
         <v/>
       </c>
       <c r="J248" s="12" t="n"/>
+      <c r="K248" s="26">
+        <f>IF(ISNUMBER($D248),IF($D248&gt;=2,ROUND(($D248-1)*100,0),IF($D248&gt;1,ROUND(-100/($D248-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="249" ht="15" customHeight="1" s="23">
       <c r="A249" s="11" t="n"/>
@@ -5899,6 +6902,10 @@
         <v/>
       </c>
       <c r="J249" s="12" t="n"/>
+      <c r="K249" s="26">
+        <f>IF(ISNUMBER($D249),IF($D249&gt;=2,ROUND(($D249-1)*100,0),IF($D249&gt;1,ROUND(-100/($D249-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="250" ht="15" customHeight="1" s="23">
       <c r="A250" s="11" t="n"/>
@@ -5920,6 +6927,10 @@
         <v/>
       </c>
       <c r="J250" s="12" t="n"/>
+      <c r="K250" s="26">
+        <f>IF(ISNUMBER($D250),IF($D250&gt;=2,ROUND(($D250-1)*100,0),IF($D250&gt;1,ROUND(-100/($D250-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="251" ht="15" customHeight="1" s="23">
       <c r="A251" s="11" t="n"/>
@@ -5941,6 +6952,10 @@
         <v/>
       </c>
       <c r="J251" s="12" t="n"/>
+      <c r="K251" s="26">
+        <f>IF(ISNUMBER($D251),IF($D251&gt;=2,ROUND(($D251-1)*100,0),IF($D251&gt;1,ROUND(-100/($D251-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="252" ht="15" customHeight="1" s="23">
       <c r="A252" s="11" t="n"/>
@@ -5962,6 +6977,10 @@
         <v/>
       </c>
       <c r="J252" s="12" t="n"/>
+      <c r="K252" s="26">
+        <f>IF(ISNUMBER($D252),IF($D252&gt;=2,ROUND(($D252-1)*100,0),IF($D252&gt;1,ROUND(-100/($D252-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="253" ht="15" customHeight="1" s="23">
       <c r="A253" s="11" t="n"/>
@@ -5983,6 +7002,10 @@
         <v/>
       </c>
       <c r="J253" s="12" t="n"/>
+      <c r="K253" s="26">
+        <f>IF(ISNUMBER($D253),IF($D253&gt;=2,ROUND(($D253-1)*100,0),IF($D253&gt;1,ROUND(-100/($D253-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="254" ht="15" customHeight="1" s="23">
       <c r="A254" s="11" t="n"/>
@@ -6004,6 +7027,10 @@
         <v/>
       </c>
       <c r="J254" s="12" t="n"/>
+      <c r="K254" s="26">
+        <f>IF(ISNUMBER($D254),IF($D254&gt;=2,ROUND(($D254-1)*100,0),IF($D254&gt;1,ROUND(-100/($D254-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="255" ht="15" customHeight="1" s="23">
       <c r="A255" s="11" t="n"/>
@@ -6025,6 +7052,10 @@
         <v/>
       </c>
       <c r="J255" s="12" t="n"/>
+      <c r="K255" s="26">
+        <f>IF(ISNUMBER($D255),IF($D255&gt;=2,ROUND(($D255-1)*100,0),IF($D255&gt;1,ROUND(-100/($D255-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="256" ht="15" customHeight="1" s="23">
       <c r="A256" s="11" t="n"/>
@@ -6046,6 +7077,10 @@
         <v/>
       </c>
       <c r="J256" s="12" t="n"/>
+      <c r="K256" s="26">
+        <f>IF(ISNUMBER($D256),IF($D256&gt;=2,ROUND(($D256-1)*100,0),IF($D256&gt;1,ROUND(-100/($D256-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="257" ht="15" customHeight="1" s="23">
       <c r="A257" s="11" t="n"/>
@@ -6067,6 +7102,10 @@
         <v/>
       </c>
       <c r="J257" s="12" t="n"/>
+      <c r="K257" s="26">
+        <f>IF(ISNUMBER($D257),IF($D257&gt;=2,ROUND(($D257-1)*100,0),IF($D257&gt;1,ROUND(-100/($D257-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="258" ht="15" customHeight="1" s="23">
       <c r="A258" s="11" t="n"/>
@@ -6088,6 +7127,10 @@
         <v/>
       </c>
       <c r="J258" s="12" t="n"/>
+      <c r="K258" s="26">
+        <f>IF(ISNUMBER($D258),IF($D258&gt;=2,ROUND(($D258-1)*100,0),IF($D258&gt;1,ROUND(-100/($D258-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="259" ht="15" customHeight="1" s="23">
       <c r="A259" s="11" t="n"/>
@@ -6109,6 +7152,10 @@
         <v/>
       </c>
       <c r="J259" s="12" t="n"/>
+      <c r="K259" s="26">
+        <f>IF(ISNUMBER($D259),IF($D259&gt;=2,ROUND(($D259-1)*100,0),IF($D259&gt;1,ROUND(-100/($D259-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="260" ht="15" customHeight="1" s="23">
       <c r="A260" s="11" t="n"/>
@@ -6130,6 +7177,10 @@
         <v/>
       </c>
       <c r="J260" s="12" t="n"/>
+      <c r="K260" s="26">
+        <f>IF(ISNUMBER($D260),IF($D260&gt;=2,ROUND(($D260-1)*100,0),IF($D260&gt;1,ROUND(-100/($D260-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="261" ht="15" customHeight="1" s="23">
       <c r="A261" s="11" t="n"/>
@@ -6151,6 +7202,10 @@
         <v/>
       </c>
       <c r="J261" s="12" t="n"/>
+      <c r="K261" s="26">
+        <f>IF(ISNUMBER($D261),IF($D261&gt;=2,ROUND(($D261-1)*100,0),IF($D261&gt;1,ROUND(-100/($D261-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="262" ht="15" customHeight="1" s="23">
       <c r="A262" s="11" t="n"/>
@@ -6172,6 +7227,10 @@
         <v/>
       </c>
       <c r="J262" s="12" t="n"/>
+      <c r="K262" s="26">
+        <f>IF(ISNUMBER($D262),IF($D262&gt;=2,ROUND(($D262-1)*100,0),IF($D262&gt;1,ROUND(-100/($D262-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="263" ht="15" customHeight="1" s="23">
       <c r="A263" s="11" t="n"/>
@@ -6193,6 +7252,10 @@
         <v/>
       </c>
       <c r="J263" s="12" t="n"/>
+      <c r="K263" s="26">
+        <f>IF(ISNUMBER($D263),IF($D263&gt;=2,ROUND(($D263-1)*100,0),IF($D263&gt;1,ROUND(-100/($D263-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="264" ht="15" customHeight="1" s="23">
       <c r="A264" s="11" t="n"/>
@@ -6214,6 +7277,10 @@
         <v/>
       </c>
       <c r="J264" s="12" t="n"/>
+      <c r="K264" s="26">
+        <f>IF(ISNUMBER($D264),IF($D264&gt;=2,ROUND(($D264-1)*100,0),IF($D264&gt;1,ROUND(-100/($D264-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="265" ht="15" customHeight="1" s="23">
       <c r="A265" s="11" t="n"/>
@@ -6235,6 +7302,10 @@
         <v/>
       </c>
       <c r="J265" s="12" t="n"/>
+      <c r="K265" s="26">
+        <f>IF(ISNUMBER($D265),IF($D265&gt;=2,ROUND(($D265-1)*100,0),IF($D265&gt;1,ROUND(-100/($D265-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="266" ht="15" customHeight="1" s="23">
       <c r="A266" s="11" t="n"/>
@@ -6256,6 +7327,10 @@
         <v/>
       </c>
       <c r="J266" s="12" t="n"/>
+      <c r="K266" s="26">
+        <f>IF(ISNUMBER($D266),IF($D266&gt;=2,ROUND(($D266-1)*100,0),IF($D266&gt;1,ROUND(-100/($D266-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="267" ht="15" customHeight="1" s="23">
       <c r="A267" s="11" t="n"/>
@@ -6277,6 +7352,10 @@
         <v/>
       </c>
       <c r="J267" s="12" t="n"/>
+      <c r="K267" s="26">
+        <f>IF(ISNUMBER($D267),IF($D267&gt;=2,ROUND(($D267-1)*100,0),IF($D267&gt;1,ROUND(-100/($D267-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="268" ht="15" customHeight="1" s="23">
       <c r="A268" s="11" t="n"/>
@@ -6298,6 +7377,10 @@
         <v/>
       </c>
       <c r="J268" s="12" t="n"/>
+      <c r="K268" s="26">
+        <f>IF(ISNUMBER($D268),IF($D268&gt;=2,ROUND(($D268-1)*100,0),IF($D268&gt;1,ROUND(-100/($D268-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="269" ht="15" customHeight="1" s="23">
       <c r="A269" s="11" t="n"/>
@@ -6319,6 +7402,10 @@
         <v/>
       </c>
       <c r="J269" s="12" t="n"/>
+      <c r="K269" s="26">
+        <f>IF(ISNUMBER($D269),IF($D269&gt;=2,ROUND(($D269-1)*100,0),IF($D269&gt;1,ROUND(-100/($D269-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="270" ht="15" customHeight="1" s="23">
       <c r="A270" s="11" t="n"/>
@@ -6340,6 +7427,10 @@
         <v/>
       </c>
       <c r="J270" s="12" t="n"/>
+      <c r="K270" s="26">
+        <f>IF(ISNUMBER($D270),IF($D270&gt;=2,ROUND(($D270-1)*100,0),IF($D270&gt;1,ROUND(-100/($D270-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="271" ht="15" customHeight="1" s="23">
       <c r="A271" s="11" t="n"/>
@@ -6361,6 +7452,10 @@
         <v/>
       </c>
       <c r="J271" s="12" t="n"/>
+      <c r="K271" s="26">
+        <f>IF(ISNUMBER($D271),IF($D271&gt;=2,ROUND(($D271-1)*100,0),IF($D271&gt;1,ROUND(-100/($D271-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="272" ht="15" customHeight="1" s="23">
       <c r="A272" s="11" t="n"/>
@@ -6382,6 +7477,10 @@
         <v/>
       </c>
       <c r="J272" s="12" t="n"/>
+      <c r="K272" s="26">
+        <f>IF(ISNUMBER($D272),IF($D272&gt;=2,ROUND(($D272-1)*100,0),IF($D272&gt;1,ROUND(-100/($D272-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="273" ht="15" customHeight="1" s="23">
       <c r="A273" s="11" t="n"/>
@@ -6403,6 +7502,10 @@
         <v/>
       </c>
       <c r="J273" s="12" t="n"/>
+      <c r="K273" s="26">
+        <f>IF(ISNUMBER($D273),IF($D273&gt;=2,ROUND(($D273-1)*100,0),IF($D273&gt;1,ROUND(-100/($D273-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="274" ht="15" customHeight="1" s="23">
       <c r="A274" s="11" t="n"/>
@@ -6424,6 +7527,10 @@
         <v/>
       </c>
       <c r="J274" s="12" t="n"/>
+      <c r="K274" s="26">
+        <f>IF(ISNUMBER($D274),IF($D274&gt;=2,ROUND(($D274-1)*100,0),IF($D274&gt;1,ROUND(-100/($D274-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="275" ht="15" customHeight="1" s="23">
       <c r="A275" s="11" t="n"/>
@@ -6445,6 +7552,10 @@
         <v/>
       </c>
       <c r="J275" s="12" t="n"/>
+      <c r="K275" s="26">
+        <f>IF(ISNUMBER($D275),IF($D275&gt;=2,ROUND(($D275-1)*100,0),IF($D275&gt;1,ROUND(-100/($D275-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="276" ht="15" customHeight="1" s="23">
       <c r="A276" s="11" t="n"/>
@@ -6466,6 +7577,10 @@
         <v/>
       </c>
       <c r="J276" s="12" t="n"/>
+      <c r="K276" s="26">
+        <f>IF(ISNUMBER($D276),IF($D276&gt;=2,ROUND(($D276-1)*100,0),IF($D276&gt;1,ROUND(-100/($D276-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="277" ht="15" customHeight="1" s="23">
       <c r="A277" s="11" t="n"/>
@@ -6487,6 +7602,10 @@
         <v/>
       </c>
       <c r="J277" s="12" t="n"/>
+      <c r="K277" s="26">
+        <f>IF(ISNUMBER($D277),IF($D277&gt;=2,ROUND(($D277-1)*100,0),IF($D277&gt;1,ROUND(-100/($D277-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="278" ht="15" customHeight="1" s="23">
       <c r="A278" s="11" t="n"/>
@@ -6508,6 +7627,10 @@
         <v/>
       </c>
       <c r="J278" s="12" t="n"/>
+      <c r="K278" s="26">
+        <f>IF(ISNUMBER($D278),IF($D278&gt;=2,ROUND(($D278-1)*100,0),IF($D278&gt;1,ROUND(-100/($D278-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="279" ht="15" customHeight="1" s="23">
       <c r="A279" s="11" t="n"/>
@@ -6529,6 +7652,10 @@
         <v/>
       </c>
       <c r="J279" s="12" t="n"/>
+      <c r="K279" s="26">
+        <f>IF(ISNUMBER($D279),IF($D279&gt;=2,ROUND(($D279-1)*100,0),IF($D279&gt;1,ROUND(-100/($D279-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="280" ht="15" customHeight="1" s="23">
       <c r="A280" s="11" t="n"/>
@@ -6550,6 +7677,10 @@
         <v/>
       </c>
       <c r="J280" s="12" t="n"/>
+      <c r="K280" s="26">
+        <f>IF(ISNUMBER($D280),IF($D280&gt;=2,ROUND(($D280-1)*100,0),IF($D280&gt;1,ROUND(-100/($D280-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="281" ht="15" customHeight="1" s="23">
       <c r="A281" s="11" t="n"/>
@@ -6571,6 +7702,10 @@
         <v/>
       </c>
       <c r="J281" s="12" t="n"/>
+      <c r="K281" s="26">
+        <f>IF(ISNUMBER($D281),IF($D281&gt;=2,ROUND(($D281-1)*100,0),IF($D281&gt;1,ROUND(-100/($D281-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="282" ht="15" customHeight="1" s="23">
       <c r="A282" s="11" t="n"/>
@@ -6592,6 +7727,10 @@
         <v/>
       </c>
       <c r="J282" s="12" t="n"/>
+      <c r="K282" s="26">
+        <f>IF(ISNUMBER($D282),IF($D282&gt;=2,ROUND(($D282-1)*100,0),IF($D282&gt;1,ROUND(-100/($D282-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="283" ht="15" customHeight="1" s="23">
       <c r="A283" s="11" t="n"/>
@@ -6613,6 +7752,10 @@
         <v/>
       </c>
       <c r="J283" s="12" t="n"/>
+      <c r="K283" s="26">
+        <f>IF(ISNUMBER($D283),IF($D283&gt;=2,ROUND(($D283-1)*100,0),IF($D283&gt;1,ROUND(-100/($D283-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="284" ht="15" customHeight="1" s="23">
       <c r="A284" s="11" t="n"/>
@@ -6634,6 +7777,10 @@
         <v/>
       </c>
       <c r="J284" s="12" t="n"/>
+      <c r="K284" s="26">
+        <f>IF(ISNUMBER($D284),IF($D284&gt;=2,ROUND(($D284-1)*100,0),IF($D284&gt;1,ROUND(-100/($D284-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="285" ht="15" customHeight="1" s="23">
       <c r="A285" s="11" t="n"/>
@@ -6655,6 +7802,10 @@
         <v/>
       </c>
       <c r="J285" s="12" t="n"/>
+      <c r="K285" s="26">
+        <f>IF(ISNUMBER($D285),IF($D285&gt;=2,ROUND(($D285-1)*100,0),IF($D285&gt;1,ROUND(-100/($D285-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="286" ht="15" customHeight="1" s="23">
       <c r="A286" s="11" t="n"/>
@@ -6676,6 +7827,10 @@
         <v/>
       </c>
       <c r="J286" s="12" t="n"/>
+      <c r="K286" s="26">
+        <f>IF(ISNUMBER($D286),IF($D286&gt;=2,ROUND(($D286-1)*100,0),IF($D286&gt;1,ROUND(-100/($D286-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="287" ht="15" customHeight="1" s="23">
       <c r="A287" s="11" t="n"/>
@@ -6697,6 +7852,10 @@
         <v/>
       </c>
       <c r="J287" s="12" t="n"/>
+      <c r="K287" s="26">
+        <f>IF(ISNUMBER($D287),IF($D287&gt;=2,ROUND(($D287-1)*100,0),IF($D287&gt;1,ROUND(-100/($D287-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="288" ht="15" customHeight="1" s="23">
       <c r="A288" s="11" t="n"/>
@@ -6718,6 +7877,10 @@
         <v/>
       </c>
       <c r="J288" s="12" t="n"/>
+      <c r="K288" s="26">
+        <f>IF(ISNUMBER($D288),IF($D288&gt;=2,ROUND(($D288-1)*100,0),IF($D288&gt;1,ROUND(-100/($D288-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="289" ht="15" customHeight="1" s="23">
       <c r="A289" s="11" t="n"/>
@@ -6739,6 +7902,10 @@
         <v/>
       </c>
       <c r="J289" s="12" t="n"/>
+      <c r="K289" s="26">
+        <f>IF(ISNUMBER($D289),IF($D289&gt;=2,ROUND(($D289-1)*100,0),IF($D289&gt;1,ROUND(-100/($D289-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="290" ht="15" customHeight="1" s="23">
       <c r="A290" s="11" t="n"/>
@@ -6760,6 +7927,10 @@
         <v/>
       </c>
       <c r="J290" s="12" t="n"/>
+      <c r="K290" s="26">
+        <f>IF(ISNUMBER($D290),IF($D290&gt;=2,ROUND(($D290-1)*100,0),IF($D290&gt;1,ROUND(-100/($D290-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="291" ht="15" customHeight="1" s="23">
       <c r="A291" s="11" t="n"/>
@@ -6781,6 +7952,10 @@
         <v/>
       </c>
       <c r="J291" s="12" t="n"/>
+      <c r="K291" s="26">
+        <f>IF(ISNUMBER($D291),IF($D291&gt;=2,ROUND(($D291-1)*100,0),IF($D291&gt;1,ROUND(-100/($D291-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="292" ht="15" customHeight="1" s="23">
       <c r="A292" s="11" t="n"/>
@@ -6802,6 +7977,10 @@
         <v/>
       </c>
       <c r="J292" s="12" t="n"/>
+      <c r="K292" s="26">
+        <f>IF(ISNUMBER($D292),IF($D292&gt;=2,ROUND(($D292-1)*100,0),IF($D292&gt;1,ROUND(-100/($D292-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="293" ht="15" customHeight="1" s="23">
       <c r="A293" s="11" t="n"/>
@@ -6823,6 +8002,10 @@
         <v/>
       </c>
       <c r="J293" s="12" t="n"/>
+      <c r="K293" s="26">
+        <f>IF(ISNUMBER($D293),IF($D293&gt;=2,ROUND(($D293-1)*100,0),IF($D293&gt;1,ROUND(-100/($D293-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="294" ht="15" customHeight="1" s="23">
       <c r="A294" s="11" t="n"/>
@@ -6844,6 +8027,10 @@
         <v/>
       </c>
       <c r="J294" s="12" t="n"/>
+      <c r="K294" s="26">
+        <f>IF(ISNUMBER($D294),IF($D294&gt;=2,ROUND(($D294-1)*100,0),IF($D294&gt;1,ROUND(-100/($D294-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="295" ht="15" customHeight="1" s="23">
       <c r="A295" s="11" t="n"/>
@@ -6865,6 +8052,10 @@
         <v/>
       </c>
       <c r="J295" s="12" t="n"/>
+      <c r="K295" s="26">
+        <f>IF(ISNUMBER($D295),IF($D295&gt;=2,ROUND(($D295-1)*100,0),IF($D295&gt;1,ROUND(-100/($D295-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="296" ht="15" customHeight="1" s="23">
       <c r="A296" s="11" t="n"/>
@@ -6886,6 +8077,10 @@
         <v/>
       </c>
       <c r="J296" s="12" t="n"/>
+      <c r="K296" s="26">
+        <f>IF(ISNUMBER($D296),IF($D296&gt;=2,ROUND(($D296-1)*100,0),IF($D296&gt;1,ROUND(-100/($D296-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="297" ht="15" customHeight="1" s="23">
       <c r="A297" s="11" t="n"/>
@@ -6907,6 +8102,10 @@
         <v/>
       </c>
       <c r="J297" s="12" t="n"/>
+      <c r="K297" s="26">
+        <f>IF(ISNUMBER($D297),IF($D297&gt;=2,ROUND(($D297-1)*100,0),IF($D297&gt;1,ROUND(-100/($D297-1),0),"")),"")</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -6917,6 +8116,7 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 

</xml_diff>